<commit_message>
Mark .env hygiene pass as Done in roadmap tracking
Update status.md and roadmap_backlog.xlsx for the .env.example rollout
across all 3 repos and the dead-code/missing-var findings from this
session's hygiene pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -119,7 +119,7 @@
     <t>backend</t>
   </si>
   <si>
-    <t>Prompted by finding the local Postgres port mismatch (app config assumes 5432, actual local Postgres is 5433) and DATABASE_URL silently overriding local dev intent.</t>
+    <t>Prompted by finding the local Postgres port mismatch (app config assumes 5432, actual local Postgres is 5433) and DATABASE_URL silently overriding local dev intent. Done 2026-08-23. Added .env.example to all 3 repos (backend/designer/services), documenting every process.env.* var actually referenced in code. Found and flagged (not removed): backend's DB_HOST/DB_NAME/DB_USER/DB_PASS + config/database.js are dead code (DATABASE_URL always wins); EMAIL_USER/EMAIL_PASS/Password_Reset_Url/Email_verify_Url/AllowedOrigins are unused leftovers. designer + services were both missing NEXT_PUBLIC_STRIPE_LINK_3/_5/_10 locally (only _CUSTOM set). services was also missing WEATHER_API_KEY2, NEXT_PUBLIC_SUPPORT_LINK, and 4 CARTO_WRI_MAP_TILE_URL vars. Confirmed no .env/.env.local currently tracked in any repo. Historical finding: services had a real .env.local committed to git history on 2025-04-23 (c6ae545) -- every secret in it has since been rotated, no live exposure, left history as-is. See status.md for full detail.</t>
   </si>
   <si>
     <t>Replace sequelize.sync({alter:true}) with real, reviewable migrations</t>
@@ -1515,7 +1515,7 @@
         <v>17</v>
       </c>
       <c r="I7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J7" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Mark Neon branch-per-PR CI as (partially) done in roadmap tracking
Update status.md and roadmap_backlog.xlsx for the neon_workflow.yml
GitHub Actions workaround merged as be916dc (PR #3), after Vercel's own
Neon integration got permanently stuck. Marked "In progress" rather than
"Done" since wiring the branch into the live Vercel Preview deployment's
DATABASE_URL is still an open follow-up.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="298">
   <si>
     <t>Phase</t>
   </si>
@@ -134,7 +134,10 @@
     <t>Adopt Neon DB branching + Vercel Preview Deployments as the standard pre-merge testing workflow</t>
   </si>
   <si>
-    <t>Gives an isolated database + isolated deployment per branch/PR with zero risk to production, without needing separate repos or projects.</t>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Gives an isolated database + isolated deployment per branch/PR with zero risk to production, without needing separate repos or projects. Partially done 2026-08-23. Vercel Preview Deployments already worked. Vercel's own Neon 'Connect a Project' dialog got permanently stuck with 'This project is already connected to the target store in one of the chosen environments', surviving deleting the DATABASE_URL vars, a hard reload, and reinstalling the integration -- unresolved, likely needs Vercel Support. Worked around it via Neon's GitHub integration instead: added .github/workflows/neon_workflow.yml giving every PR an isolated Neon branch forked from main, running npm run migrate against it as a pre-merge check, deleting the branch on PR close. Caught and fixed a wrong output name in Neon's own template (db_url_with_pooler doesn't exist; real one is db_url_pooled). Verified working end-to-end on PR #3, merged to main as be916dc. Still missing: wiring the branch into the live Vercel Preview deployment's DATABASE_URL for that PR (needs a VERCEL_TOKEN secret + a step calling Vercel's env API) -- pending a decision from Omar. See status.md.</t>
   </si>
   <si>
     <t>Fix Google Sign-In: verify real Google id_token server-side (Option 1)</t>
@@ -1579,10 +1582,10 @@
         <v>17</v>
       </c>
       <c r="I9" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="J9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1593,10 +1596,10 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -1614,7 +1617,7 @@
         <v>18</v>
       </c>
       <c r="J10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1625,7 +1628,7 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
         <v>30</v>
@@ -1646,24 +1649,24 @@
         <v>18</v>
       </c>
       <c r="J11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12" t="s">
         <v>27</v>
@@ -1672,30 +1675,30 @@
         <v>16</v>
       </c>
       <c r="H12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I12" t="s">
         <v>22</v>
       </c>
       <c r="J12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F13" t="s">
         <v>33</v>
@@ -1704,30 +1707,30 @@
         <v>16</v>
       </c>
       <c r="H13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I13" t="s">
         <v>22</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F14" t="s">
         <v>27</v>
@@ -1736,30 +1739,30 @@
         <v>16</v>
       </c>
       <c r="H14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I14" t="s">
         <v>22</v>
       </c>
       <c r="J14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
         <v>33</v>
@@ -1768,30 +1771,30 @@
         <v>16</v>
       </c>
       <c r="H15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I15" t="s">
         <v>22</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F16" t="s">
         <v>33</v>
@@ -1800,30 +1803,30 @@
         <v>16</v>
       </c>
       <c r="H16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I16" t="s">
         <v>18</v>
       </c>
       <c r="J16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F17" t="s">
         <v>27</v>
@@ -1832,62 +1835,62 @@
         <v>16</v>
       </c>
       <c r="H17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I17" t="s">
         <v>22</v>
       </c>
       <c r="J17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G18" t="s">
         <v>16</v>
       </c>
       <c r="H18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I18" t="s">
         <v>22</v>
       </c>
       <c r="J18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
         <v>33</v>
@@ -1896,30 +1899,30 @@
         <v>16</v>
       </c>
       <c r="H19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I19" t="s">
         <v>22</v>
       </c>
       <c r="J19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F20" t="s">
         <v>33</v>
@@ -1928,30 +1931,30 @@
         <v>16</v>
       </c>
       <c r="H20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I20" t="s">
         <v>22</v>
       </c>
       <c r="J20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
         <v>27</v>
@@ -1960,30 +1963,30 @@
         <v>21</v>
       </c>
       <c r="H21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I21" t="s">
         <v>22</v>
       </c>
       <c r="J21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F22" t="s">
         <v>33</v>
@@ -1992,30 +1995,30 @@
         <v>21</v>
       </c>
       <c r="H22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I22" t="s">
         <v>22</v>
       </c>
       <c r="J22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F23" t="s">
         <v>27</v>
@@ -2024,30 +2027,30 @@
         <v>16</v>
       </c>
       <c r="H23" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I23" t="s">
         <v>22</v>
       </c>
       <c r="J23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F24" t="s">
         <v>27</v>
@@ -2056,30 +2059,30 @@
         <v>16</v>
       </c>
       <c r="H24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
       </c>
       <c r="J24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F25" t="s">
         <v>27</v>
@@ -2088,30 +2091,30 @@
         <v>16</v>
       </c>
       <c r="H25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I25" t="s">
         <v>22</v>
       </c>
       <c r="J25" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F26" t="s">
         <v>27</v>
@@ -2120,7 +2123,7 @@
         <v>21</v>
       </c>
       <c r="H26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I26" t="s">
         <v>22</v>
@@ -2128,19 +2131,19 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F27" t="s">
         <v>27</v>
@@ -2149,30 +2152,30 @@
         <v>21</v>
       </c>
       <c r="H27" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I27" t="s">
         <v>22</v>
       </c>
       <c r="J27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F28" t="s">
         <v>27</v>
@@ -2181,30 +2184,30 @@
         <v>21</v>
       </c>
       <c r="H28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I28" t="s">
         <v>22</v>
       </c>
       <c r="J28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E29" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F29" t="s">
         <v>27</v>
@@ -2213,30 +2216,30 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I29" t="s">
         <v>22</v>
       </c>
       <c r="J29" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F30" t="s">
         <v>27</v>
@@ -2245,30 +2248,30 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I30" t="s">
         <v>22</v>
       </c>
       <c r="J30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D31" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F31" t="s">
         <v>27</v>
@@ -2277,7 +2280,7 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I31" t="s">
         <v>22</v>
@@ -2285,19 +2288,19 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F32" t="s">
         <v>27</v>
@@ -2306,7 +2309,7 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I32" t="s">
         <v>22</v>
@@ -2314,19 +2317,19 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D33" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F33" t="s">
         <v>27</v>
@@ -2335,7 +2338,7 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I33" t="s">
         <v>22</v>
@@ -2343,19 +2346,19 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C34" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D34" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F34" t="s">
         <v>27</v>
@@ -2364,30 +2367,30 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I34" t="s">
         <v>22</v>
       </c>
       <c r="J34" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B35" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D35" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F35" t="s">
         <v>27</v>
@@ -2396,7 +2399,7 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I35" t="s">
         <v>22</v>
@@ -2404,28 +2407,28 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D36" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F36" t="s">
         <v>27</v>
       </c>
       <c r="G36" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H36" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I36" t="s">
         <v>22</v>
@@ -2433,28 +2436,28 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D37" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F37" t="s">
         <v>27</v>
       </c>
       <c r="G37" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H37" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I37" t="s">
         <v>22</v>
@@ -2462,28 +2465,28 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F38" t="s">
         <v>27</v>
       </c>
       <c r="G38" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H38" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I38" t="s">
         <v>22</v>
@@ -2491,60 +2494,60 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D39" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F39" t="s">
         <v>27</v>
       </c>
       <c r="G39" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H39" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I39" t="s">
         <v>22</v>
       </c>
       <c r="J39" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C40" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D40" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F40" t="s">
         <v>27</v>
       </c>
       <c r="G40" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H40" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I40" t="s">
         <v>22</v>
@@ -2552,28 +2555,28 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C41" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D41" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F41" t="s">
         <v>27</v>
       </c>
       <c r="G41" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H41" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I41" t="s">
         <v>22</v>
@@ -2581,28 +2584,28 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C42" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D42" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F42" t="s">
         <v>27</v>
       </c>
       <c r="G42" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H42" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I42" t="s">
         <v>22</v>
@@ -2610,220 +2613,220 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B43" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C43" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D43" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E43" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F43" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G43" t="s">
         <v>16</v>
       </c>
       <c r="H43" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I43" t="s">
         <v>22</v>
       </c>
       <c r="J43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D44" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F44" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G44" t="s">
         <v>16</v>
       </c>
       <c r="H44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I44" t="s">
         <v>22</v>
       </c>
       <c r="J44" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B45" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C45" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E45" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F45" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G45" t="s">
         <v>16</v>
       </c>
       <c r="H45" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I45" t="s">
         <v>22</v>
       </c>
       <c r="J45" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B46" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C46" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D46" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E46" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F46" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G46" t="s">
         <v>16</v>
       </c>
       <c r="H46" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I46" t="s">
         <v>22</v>
       </c>
       <c r="J46" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E47" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F47" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G47" t="s">
         <v>21</v>
       </c>
       <c r="H47" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I47" t="s">
         <v>22</v>
       </c>
       <c r="J47" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E48" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F48" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G48" t="s">
         <v>16</v>
       </c>
       <c r="H48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I48" t="s">
         <v>22</v>
       </c>
       <c r="J48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B49" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E49" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G49" t="s">
         <v>16</v>
       </c>
       <c r="H49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I49" t="s">
         <v>22</v>
@@ -2831,92 +2834,92 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B50" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F50" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G50" t="s">
         <v>21</v>
       </c>
       <c r="H50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I50" t="s">
         <v>22</v>
       </c>
       <c r="J50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D51" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E51" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F51" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G51" t="s">
         <v>21</v>
       </c>
       <c r="H51" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I51" t="s">
         <v>22</v>
       </c>
       <c r="J51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B52" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C52" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D52" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E52" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F52" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G52" t="s">
         <v>21</v>
       </c>
       <c r="H52" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I52" t="s">
         <v>22</v>
@@ -2924,188 +2927,188 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B53" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D53" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E53" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F53" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G53" t="s">
         <v>21</v>
       </c>
       <c r="H53" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I53" t="s">
         <v>22</v>
       </c>
       <c r="J53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B54" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F54" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G54" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H54" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I54" t="s">
         <v>22</v>
       </c>
       <c r="J54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B55" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D55" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E55" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F55" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H55" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I55" t="s">
         <v>22</v>
       </c>
       <c r="J55" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B56" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C56" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D56" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E56" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F56" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G56" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H56" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I56" t="s">
         <v>22</v>
       </c>
       <c r="J56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B57" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C57" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D57" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E57" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F57" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G57" t="s">
         <v>16</v>
       </c>
       <c r="H57" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I57" t="s">
         <v>22</v>
       </c>
       <c r="J57" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B58" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C58" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E58" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F58" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G58" t="s">
         <v>21</v>
       </c>
       <c r="H58" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I58" t="s">
         <v>22</v>
@@ -3113,124 +3116,124 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B59" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C59" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D59" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E59" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F59" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G59" t="s">
         <v>21</v>
       </c>
       <c r="H59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I59" t="s">
         <v>22</v>
       </c>
       <c r="J59" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C60" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D60" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E60" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F60" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G60" t="s">
         <v>21</v>
       </c>
       <c r="H60" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I60" t="s">
         <v>22</v>
       </c>
       <c r="J60" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C61" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D61" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E61" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F61" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G61" t="s">
         <v>21</v>
       </c>
       <c r="H61" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I61" t="s">
         <v>22</v>
       </c>
       <c r="J61" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B62" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D62" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E62" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F62" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G62" t="s">
         <v>21</v>
       </c>
       <c r="H62" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I62" t="s">
         <v>22</v>
@@ -3238,51 +3241,51 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C63" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D63" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E63" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F63" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G63" t="s">
         <v>21</v>
       </c>
       <c r="H63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I63" t="s">
         <v>22</v>
       </c>
       <c r="J63" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C64" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D64" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E64" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F64" t="s">
         <v>27</v>
@@ -3291,7 +3294,7 @@
         <v>21</v>
       </c>
       <c r="H64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I64" t="s">
         <v>22</v>
@@ -3299,124 +3302,124 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C65" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D65" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E65" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G65" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H65" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I65" t="s">
         <v>22</v>
       </c>
       <c r="J65" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C66" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D66" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E66" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F66" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G66" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H66" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I66" t="s">
         <v>22</v>
       </c>
       <c r="J66" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C67" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D67" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F67" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G67" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I67" t="s">
         <v>22</v>
       </c>
       <c r="J67" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B68" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C68" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D68" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E68" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F68" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G68" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I68" t="s">
         <v>22</v>
@@ -3424,28 +3427,28 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C69" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D69" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E69" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F69" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G69" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H69" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I69" t="s">
         <v>22</v>
@@ -3453,92 +3456,92 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C70" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E70" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F70" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H70" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I70" t="s">
         <v>22</v>
       </c>
       <c r="J70" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C71" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E71" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F71" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G71" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H71" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I71" t="s">
         <v>22</v>
       </c>
       <c r="J71" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B72" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C72" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D72" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E72" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F72" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G72" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H72" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I72" t="s">
         <v>22</v>
@@ -3546,28 +3549,28 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B73" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C73" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D73" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E73" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F73" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G73" t="s">
         <v>21</v>
       </c>
       <c r="H73" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I73" t="s">
         <v>22</v>
@@ -3575,28 +3578,28 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B74" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C74" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D74" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E74" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F74" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G74" t="s">
         <v>21</v>
       </c>
       <c r="H74" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I74" t="s">
         <v>22</v>
@@ -3604,92 +3607,92 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B75" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C75" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D75" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E75" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F75" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G75" t="s">
         <v>21</v>
       </c>
       <c r="H75" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I75" t="s">
         <v>22</v>
       </c>
       <c r="J75" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B76" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C76" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D76" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E76" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F76" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G76" t="s">
         <v>21</v>
       </c>
       <c r="H76" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I76" t="s">
         <v>22</v>
       </c>
       <c r="J76" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B77" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C77" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D77" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E77" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F77" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G77" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H77" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I77" t="s">
         <v>22</v>
@@ -3697,188 +3700,188 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C78" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D78" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E78" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F78" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G78" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H78" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I78" t="s">
         <v>22</v>
       </c>
       <c r="J78" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B79" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C79" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D79" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E79" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F79" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G79" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H79" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I79" t="s">
         <v>22</v>
       </c>
       <c r="J79" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B80" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C80" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D80" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E80" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F80" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G80" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H80" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I80" t="s">
         <v>22</v>
       </c>
       <c r="J80" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B81" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C81" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D81" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E81" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F81" t="s">
         <v>27</v>
       </c>
       <c r="G81" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H81" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I81" t="s">
         <v>22</v>
       </c>
       <c r="J81" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B82" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C82" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D82" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E82" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F82" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G82" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H82" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I82" t="s">
         <v>22</v>
       </c>
       <c r="J82" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B83" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C83" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D83" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E83" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F83" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G83" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H83" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I83" t="s">
         <v>22</v>
@@ -3886,252 +3889,252 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B84" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C84" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D84" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E84" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F84" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G84" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H84" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I84" t="s">
         <v>22</v>
       </c>
       <c r="J84" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B85" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C85" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D85" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E85" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F85" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G85" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H85" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I85" t="s">
         <v>22</v>
       </c>
       <c r="J85" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B86" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C86" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D86" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E86" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F86" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G86" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H86" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I86" t="s">
         <v>22</v>
       </c>
       <c r="J86" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B87" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C87" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D87" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E87" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F87" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G87" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H87" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I87" t="s">
         <v>22</v>
       </c>
       <c r="J87" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B88" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C88" t="s">
+        <v>233</v>
+      </c>
+      <c r="D88" t="s">
+        <v>169</v>
+      </c>
+      <c r="E88" t="s">
+        <v>128</v>
+      </c>
+      <c r="F88" t="s">
+        <v>71</v>
+      </c>
+      <c r="G88" t="s">
+        <v>218</v>
+      </c>
+      <c r="H88" t="s">
+        <v>219</v>
+      </c>
+      <c r="I88" t="s">
+        <v>22</v>
+      </c>
+      <c r="J88" t="s">
         <v>232</v>
-      </c>
-      <c r="D88" t="s">
-        <v>168</v>
-      </c>
-      <c r="E88" t="s">
-        <v>127</v>
-      </c>
-      <c r="F88" t="s">
-        <v>70</v>
-      </c>
-      <c r="G88" t="s">
-        <v>217</v>
-      </c>
-      <c r="H88" t="s">
-        <v>218</v>
-      </c>
-      <c r="I88" t="s">
-        <v>22</v>
-      </c>
-      <c r="J88" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B89" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C89" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D89" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E89" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F89" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G89" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H89" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I89" t="s">
         <v>22</v>
       </c>
       <c r="J89" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B90" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C90" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D90" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E90" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F90" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G90" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H90" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I90" t="s">
         <v>22</v>
       </c>
       <c r="J90" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B91" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C91" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D91" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E91" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F91" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G91" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H91" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I91" t="s">
         <v>22</v>
@@ -4139,60 +4142,60 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B92" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C92" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D92" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E92" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F92" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G92" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H92" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I92" t="s">
         <v>22</v>
       </c>
       <c r="J92" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B93" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C93" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D93" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E93" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F93" t="s">
         <v>33</v>
       </c>
       <c r="G93" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H93" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I93" t="s">
         <v>22</v>
@@ -4200,51 +4203,51 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B94" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C94" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D94" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E94" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F94" t="s">
         <v>33</v>
       </c>
       <c r="G94" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H94" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I94" t="s">
         <v>22</v>
       </c>
       <c r="J94" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B95" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C95" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D95" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E95" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F95" t="s">
         <v>27</v>
@@ -4253,30 +4256,30 @@
         <v>16</v>
       </c>
       <c r="H95" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I95" t="s">
         <v>22</v>
       </c>
       <c r="J95" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B96" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C96" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D96" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E96" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F96" t="s">
         <v>27</v>
@@ -4285,30 +4288,30 @@
         <v>16</v>
       </c>
       <c r="H96" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I96" t="s">
         <v>22</v>
       </c>
       <c r="J96" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B97" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C97" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D97" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E97" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F97" t="s">
         <v>27</v>
@@ -4317,30 +4320,30 @@
         <v>16</v>
       </c>
       <c r="H97" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I97" t="s">
         <v>22</v>
       </c>
       <c r="J97" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B98" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C98" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D98" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E98" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F98" t="s">
         <v>27</v>
@@ -4349,30 +4352,30 @@
         <v>21</v>
       </c>
       <c r="H98" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I98" t="s">
         <v>22</v>
       </c>
       <c r="J98" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B99" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C99" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D99" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E99" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F99" t="s">
         <v>27</v>
@@ -4381,7 +4384,7 @@
         <v>21</v>
       </c>
       <c r="H99" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I99" t="s">
         <v>22</v>
@@ -4389,19 +4392,19 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B100" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C100" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D100" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E100" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F100" t="s">
         <v>27</v>
@@ -4410,7 +4413,7 @@
         <v>21</v>
       </c>
       <c r="H100" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I100" t="s">
         <v>22</v>
@@ -4418,19 +4421,19 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B101" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C101" t="s">
+        <v>262</v>
+      </c>
+      <c r="D101" t="s">
+        <v>58</v>
+      </c>
+      <c r="E101" t="s">
         <v>261</v>
-      </c>
-      <c r="D101" t="s">
-        <v>57</v>
-      </c>
-      <c r="E101" t="s">
-        <v>260</v>
       </c>
       <c r="F101" t="s">
         <v>27</v>
@@ -4439,7 +4442,7 @@
         <v>21</v>
       </c>
       <c r="H101" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I101" t="s">
         <v>22</v>
@@ -4447,19 +4450,19 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B102" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C102" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D102" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E102" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F102" t="s">
         <v>27</v>
@@ -4468,103 +4471,103 @@
         <v>21</v>
       </c>
       <c r="H102" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I102" t="s">
         <v>22</v>
       </c>
       <c r="J102" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B103" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C103" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D103" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E103" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F103" t="s">
         <v>27</v>
       </c>
       <c r="G103" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H103" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I103" t="s">
         <v>22</v>
       </c>
       <c r="J103" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B104" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C104" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D104" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E104" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F104" t="s">
         <v>27</v>
       </c>
       <c r="G104" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H104" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I104" t="s">
         <v>22</v>
       </c>
       <c r="J104" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B105" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C105" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D105" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E105" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F105" t="s">
         <v>27</v>
       </c>
       <c r="G105" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H105" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I105" t="s">
         <v>22</v>
@@ -4572,28 +4575,28 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B106" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C106" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D106" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E106" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F106" t="s">
         <v>27</v>
       </c>
       <c r="G106" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H106" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I106" t="s">
         <v>22</v>
@@ -4601,34 +4604,34 @@
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B107" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C107" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D107" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E107" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I107" t="s">
         <v>22</v>
       </c>
       <c r="J107" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -4654,19 +4657,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E1" t="s">
         <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G1" t="s">
         <v>16</v>
@@ -4675,10 +4678,10 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4692,10 +4695,10 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -4715,19 +4718,19 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F3">
         <v>11</v>
@@ -4747,19 +4750,19 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F4">
         <v>20</v>
@@ -4779,19 +4782,19 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -4811,19 +4814,19 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
+        <v>291</v>
+      </c>
+      <c r="E6" t="s">
         <v>290</v>
-      </c>
-      <c r="E6" t="s">
-        <v>289</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -4843,19 +4846,19 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F7">
         <v>16</v>
@@ -4875,19 +4878,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F8">
         <v>8</v>
@@ -4907,19 +4910,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D9" t="s">
+        <v>296</v>
+      </c>
+      <c r="E9" t="s">
         <v>295</v>
-      </c>
-      <c r="E9" t="s">
-        <v>294</v>
       </c>
       <c r="F9">
         <v>14</v>
@@ -4939,19 +4942,19 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F10">
         <v>12</v>
@@ -4971,19 +4974,19 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F11">
         <v>1</v>

</xml_diff>

<commit_message>
Mark Neon branching + Vercel Preview wiring as fully Done
Update status.md and roadmap_backlog.xlsx: the Vercel Preview
DATABASE_URL wiring (chore/wire-vercel-preview-db, merged as 5a3067d)
closes the gap left by the earlier CI-only version. Also documents the
branch protection added to main and the security incident (leaked
encrypted envelope in a public Actions log) caught and fixed same
session.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="297">
   <si>
     <t>Phase</t>
   </si>
@@ -134,10 +134,7 @@
     <t>Adopt Neon DB branching + Vercel Preview Deployments as the standard pre-merge testing workflow</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
-    <t>Gives an isolated database + isolated deployment per branch/PR with zero risk to production, without needing separate repos or projects. Partially done 2026-08-23. Vercel Preview Deployments already worked. Vercel's own Neon 'Connect a Project' dialog got permanently stuck with 'This project is already connected to the target store in one of the chosen environments', surviving deleting the DATABASE_URL vars, a hard reload, and reinstalling the integration -- unresolved, likely needs Vercel Support. Worked around it via Neon's GitHub integration instead: added .github/workflows/neon_workflow.yml giving every PR an isolated Neon branch forked from main, running npm run migrate against it as a pre-merge check, deleting the branch on PR close. Caught and fixed a wrong output name in Neon's own template (db_url_with_pooler doesn't exist; real one is db_url_pooled). Verified working end-to-end on PR #3, merged to main as be916dc. Still missing: wiring the branch into the live Vercel Preview deployment's DATABASE_URL for that PR (needs a VERCEL_TOKEN secret + a step calling Vercel's env API) -- pending a decision from Omar. See status.md.</t>
+    <t>Gives an isolated database + isolated deployment per branch/PR with zero risk to production, without needing separate repos or projects. Partially done 2026-08-23. Vercel Preview Deployments already worked. Vercel's own Neon 'Connect a Project' dialog got permanently stuck with 'This project is already connected to the target store in one of the chosen environments', surviving deleting the DATABASE_URL vars, a hard reload, and reinstalling the integration -- unresolved, likely needs Vercel Support. Worked around it via Neon's GitHub integration instead: added .github/workflows/neon_workflow.yml giving every PR an isolated Neon branch forked from main, running npm run migrate against it as a pre-merge check, deleting the branch on PR close. Caught and fixed a wrong output name in Neon's own template (db_url_with_pooler doesn't exist; real one is db_url_pooled). Verified working end-to-end on PR #3, merged to main as be916dc. Still missing: wiring the branch into the live Vercel Preview deployment's DATABASE_URL for that PR (needs a VERCEL_TOKEN secret + a step calling Vercel's env API) -- pending a decision from Omar. See status.md. Fully done 2026-08-23: closed the remaining gap by wiring Neon branches into live Vercel Preview deployments too, via a workflow step calling Vercel's env API (VERCEL_TOKEN secret + VERCEL_PROJECT_ID/VERCEL_TEAM_ID variables), scoped to each PR's git branch. Added branch protection to main (blocks force-push/deletion, requires the Neon migration job to pass). Self-caught and fixed a security bug same session: a botched jq redaction leaked Vercel's encrypted DATABASE_URL envelope into this public repo's Actions log for one run; fixed the redaction and deleted that run's logs. Shipped on chore/wire-vercel-preview-db, merged as 5a3067d. See status.md for full detail.</t>
   </si>
   <si>
     <t>Fix Google Sign-In: verify real Google id_token server-side (Option 1)</t>
@@ -1582,10 +1579,10 @@
         <v>17</v>
       </c>
       <c r="I9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" t="s">
         <v>39</v>
-      </c>
-      <c r="J9" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1596,10 +1593,10 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
         <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>42</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -1617,7 +1614,7 @@
         <v>18</v>
       </c>
       <c r="J10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1628,7 +1625,7 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
         <v>30</v>
@@ -1649,24 +1646,24 @@
         <v>18</v>
       </c>
       <c r="J11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" t="s">
         <v>46</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>47</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>48</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>49</v>
-      </c>
-      <c r="E12" t="s">
-        <v>50</v>
       </c>
       <c r="F12" t="s">
         <v>27</v>
@@ -1675,30 +1672,30 @@
         <v>16</v>
       </c>
       <c r="H12" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12" t="s">
+        <v>22</v>
+      </c>
+      <c r="J12" t="s">
         <v>51</v>
-      </c>
-      <c r="I12" t="s">
-        <v>22</v>
-      </c>
-      <c r="J12" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
         <v>46</v>
       </c>
-      <c r="B13" t="s">
-        <v>47</v>
-      </c>
       <c r="C13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
         <v>53</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>54</v>
-      </c>
-      <c r="E13" t="s">
-        <v>55</v>
       </c>
       <c r="F13" t="s">
         <v>33</v>
@@ -1707,30 +1704,30 @@
         <v>16</v>
       </c>
       <c r="H13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I13" t="s">
         <v>22</v>
       </c>
       <c r="J13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" t="s">
         <v>46</v>
       </c>
-      <c r="B14" t="s">
-        <v>47</v>
-      </c>
       <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" t="s">
         <v>57</v>
       </c>
-      <c r="D14" t="s">
-        <v>58</v>
-      </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F14" t="s">
         <v>27</v>
@@ -1739,30 +1736,30 @@
         <v>16</v>
       </c>
       <c r="H14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I14" t="s">
         <v>22</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" t="s">
         <v>46</v>
       </c>
-      <c r="B15" t="s">
-        <v>47</v>
-      </c>
       <c r="C15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" t="s">
         <v>60</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>61</v>
-      </c>
-      <c r="E15" t="s">
-        <v>62</v>
       </c>
       <c r="F15" t="s">
         <v>33</v>
@@ -1771,30 +1768,30 @@
         <v>16</v>
       </c>
       <c r="H15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I15" t="s">
         <v>22</v>
       </c>
       <c r="J15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
         <v>46</v>
       </c>
-      <c r="B16" t="s">
-        <v>47</v>
-      </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" t="s">
         <v>61</v>
-      </c>
-      <c r="E16" t="s">
-        <v>62</v>
       </c>
       <c r="F16" t="s">
         <v>33</v>
@@ -1803,30 +1800,30 @@
         <v>16</v>
       </c>
       <c r="H16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I16" t="s">
         <v>18</v>
       </c>
       <c r="J16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
         <v>46</v>
       </c>
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" t="s">
         <v>61</v>
-      </c>
-      <c r="E17" t="s">
-        <v>62</v>
       </c>
       <c r="F17" t="s">
         <v>27</v>
@@ -1835,62 +1832,62 @@
         <v>16</v>
       </c>
       <c r="H17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I17" t="s">
         <v>22</v>
       </c>
       <c r="J17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
         <v>46</v>
       </c>
-      <c r="B18" t="s">
-        <v>47</v>
-      </c>
       <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" t="s">
         <v>68</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>69</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>70</v>
-      </c>
-      <c r="F18" t="s">
-        <v>71</v>
       </c>
       <c r="G18" t="s">
         <v>16</v>
       </c>
       <c r="H18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I18" t="s">
         <v>22</v>
       </c>
       <c r="J18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" t="s">
         <v>46</v>
       </c>
-      <c r="B19" t="s">
-        <v>47</v>
-      </c>
       <c r="C19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" t="s">
         <v>73</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>74</v>
-      </c>
-      <c r="E19" t="s">
-        <v>75</v>
       </c>
       <c r="F19" t="s">
         <v>33</v>
@@ -1899,30 +1896,30 @@
         <v>16</v>
       </c>
       <c r="H19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I19" t="s">
         <v>22</v>
       </c>
       <c r="J19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" t="s">
         <v>46</v>
       </c>
-      <c r="B20" t="s">
-        <v>47</v>
-      </c>
       <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" t="s">
         <v>77</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>78</v>
-      </c>
-      <c r="E20" t="s">
-        <v>79</v>
       </c>
       <c r="F20" t="s">
         <v>33</v>
@@ -1931,30 +1928,30 @@
         <v>16</v>
       </c>
       <c r="H20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I20" t="s">
         <v>22</v>
       </c>
       <c r="J20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" t="s">
         <v>46</v>
       </c>
-      <c r="B21" t="s">
-        <v>47</v>
-      </c>
       <c r="C21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D21" t="s">
         <v>81</v>
       </c>
-      <c r="D21" t="s">
-        <v>82</v>
-      </c>
       <c r="E21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F21" t="s">
         <v>27</v>
@@ -1963,30 +1960,30 @@
         <v>21</v>
       </c>
       <c r="H21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I21" t="s">
         <v>22</v>
       </c>
       <c r="J21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" t="s">
         <v>46</v>
       </c>
-      <c r="B22" t="s">
-        <v>47</v>
-      </c>
       <c r="C22" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" t="s">
         <v>84</v>
-      </c>
-      <c r="D22" t="s">
-        <v>54</v>
-      </c>
-      <c r="E22" t="s">
-        <v>85</v>
       </c>
       <c r="F22" t="s">
         <v>33</v>
@@ -1995,30 +1992,30 @@
         <v>21</v>
       </c>
       <c r="H22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I22" t="s">
         <v>22</v>
       </c>
       <c r="J22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" t="s">
         <v>87</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>88</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>89</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>90</v>
-      </c>
-      <c r="E23" t="s">
-        <v>91</v>
       </c>
       <c r="F23" t="s">
         <v>27</v>
@@ -2027,30 +2024,30 @@
         <v>16</v>
       </c>
       <c r="H23" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" t="s">
+        <v>22</v>
+      </c>
+      <c r="J23" t="s">
         <v>92</v>
-      </c>
-      <c r="I23" t="s">
-        <v>22</v>
-      </c>
-      <c r="J23" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" t="s">
         <v>87</v>
       </c>
-      <c r="B24" t="s">
-        <v>88</v>
-      </c>
       <c r="C24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D24" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" t="s">
         <v>90</v>
-      </c>
-      <c r="E24" t="s">
-        <v>91</v>
       </c>
       <c r="F24" t="s">
         <v>27</v>
@@ -2059,30 +2056,30 @@
         <v>16</v>
       </c>
       <c r="H24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
       </c>
       <c r="J24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" t="s">
         <v>87</v>
       </c>
-      <c r="B25" t="s">
-        <v>88</v>
-      </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D25" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" t="s">
         <v>90</v>
-      </c>
-      <c r="E25" t="s">
-        <v>91</v>
       </c>
       <c r="F25" t="s">
         <v>27</v>
@@ -2091,30 +2088,30 @@
         <v>16</v>
       </c>
       <c r="H25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I25" t="s">
         <v>22</v>
       </c>
       <c r="J25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" t="s">
         <v>87</v>
       </c>
-      <c r="B26" t="s">
-        <v>88</v>
-      </c>
       <c r="C26" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D26" t="s">
+        <v>89</v>
+      </c>
+      <c r="E26" t="s">
         <v>90</v>
-      </c>
-      <c r="E26" t="s">
-        <v>91</v>
       </c>
       <c r="F26" t="s">
         <v>27</v>
@@ -2123,7 +2120,7 @@
         <v>21</v>
       </c>
       <c r="H26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I26" t="s">
         <v>22</v>
@@ -2131,19 +2128,19 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" t="s">
         <v>87</v>
       </c>
-      <c r="B27" t="s">
-        <v>88</v>
-      </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D27" t="s">
+        <v>89</v>
+      </c>
+      <c r="E27" t="s">
         <v>90</v>
-      </c>
-      <c r="E27" t="s">
-        <v>91</v>
       </c>
       <c r="F27" t="s">
         <v>27</v>
@@ -2152,30 +2149,30 @@
         <v>21</v>
       </c>
       <c r="H27" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I27" t="s">
         <v>22</v>
       </c>
       <c r="J27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" t="s">
         <v>87</v>
       </c>
-      <c r="B28" t="s">
-        <v>88</v>
-      </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D28" t="s">
+        <v>89</v>
+      </c>
+      <c r="E28" t="s">
         <v>90</v>
-      </c>
-      <c r="E28" t="s">
-        <v>91</v>
       </c>
       <c r="F28" t="s">
         <v>27</v>
@@ -2184,30 +2181,30 @@
         <v>21</v>
       </c>
       <c r="H28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I28" t="s">
         <v>22</v>
       </c>
       <c r="J28" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" t="s">
         <v>87</v>
       </c>
-      <c r="B29" t="s">
-        <v>88</v>
-      </c>
       <c r="C29" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" t="s">
         <v>103</v>
       </c>
-      <c r="D29" t="s">
-        <v>104</v>
-      </c>
       <c r="E29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F29" t="s">
         <v>27</v>
@@ -2216,30 +2213,30 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I29" t="s">
         <v>22</v>
       </c>
       <c r="J29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" t="s">
         <v>87</v>
       </c>
-      <c r="B30" t="s">
-        <v>88</v>
-      </c>
       <c r="C30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D30" t="s">
+        <v>89</v>
+      </c>
+      <c r="E30" t="s">
         <v>90</v>
-      </c>
-      <c r="E30" t="s">
-        <v>91</v>
       </c>
       <c r="F30" t="s">
         <v>27</v>
@@ -2248,30 +2245,30 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I30" t="s">
         <v>22</v>
       </c>
       <c r="J30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" t="s">
         <v>87</v>
       </c>
-      <c r="B31" t="s">
-        <v>88</v>
-      </c>
       <c r="C31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D31" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" t="s">
         <v>90</v>
-      </c>
-      <c r="E31" t="s">
-        <v>91</v>
       </c>
       <c r="F31" t="s">
         <v>27</v>
@@ -2280,7 +2277,7 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I31" t="s">
         <v>22</v>
@@ -2288,19 +2285,19 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>86</v>
+      </c>
+      <c r="B32" t="s">
         <v>87</v>
       </c>
-      <c r="B32" t="s">
-        <v>88</v>
-      </c>
       <c r="C32" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D32" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" t="s">
         <v>90</v>
-      </c>
-      <c r="E32" t="s">
-        <v>91</v>
       </c>
       <c r="F32" t="s">
         <v>27</v>
@@ -2309,7 +2306,7 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I32" t="s">
         <v>22</v>
@@ -2317,19 +2314,19 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" t="s">
         <v>87</v>
       </c>
-      <c r="B33" t="s">
-        <v>88</v>
-      </c>
       <c r="C33" t="s">
+        <v>109</v>
+      </c>
+      <c r="D33" t="s">
         <v>110</v>
       </c>
-      <c r="D33" t="s">
-        <v>111</v>
-      </c>
       <c r="E33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F33" t="s">
         <v>27</v>
@@ -2338,7 +2335,7 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I33" t="s">
         <v>22</v>
@@ -2346,19 +2343,19 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" t="s">
         <v>87</v>
       </c>
-      <c r="B34" t="s">
-        <v>88</v>
-      </c>
       <c r="C34" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" t="s">
         <v>112</v>
       </c>
-      <c r="D34" t="s">
-        <v>113</v>
-      </c>
       <c r="E34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F34" t="s">
         <v>27</v>
@@ -2367,30 +2364,30 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I34" t="s">
         <v>22</v>
       </c>
       <c r="J34" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35" t="s">
         <v>87</v>
       </c>
-      <c r="B35" t="s">
-        <v>88</v>
-      </c>
       <c r="C35" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D35" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F35" t="s">
         <v>27</v>
@@ -2399,7 +2396,7 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I35" t="s">
         <v>22</v>
@@ -2407,28 +2404,28 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" t="s">
         <v>87</v>
       </c>
-      <c r="B36" t="s">
-        <v>88</v>
-      </c>
       <c r="C36" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D36" t="s">
+        <v>89</v>
+      </c>
+      <c r="E36" t="s">
         <v>90</v>
-      </c>
-      <c r="E36" t="s">
-        <v>91</v>
       </c>
       <c r="F36" t="s">
         <v>27</v>
       </c>
       <c r="G36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H36" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I36" t="s">
         <v>22</v>
@@ -2436,28 +2433,28 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" t="s">
         <v>87</v>
       </c>
-      <c r="B37" t="s">
-        <v>88</v>
-      </c>
       <c r="C37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D37" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" t="s">
         <v>90</v>
-      </c>
-      <c r="E37" t="s">
-        <v>91</v>
       </c>
       <c r="F37" t="s">
         <v>27</v>
       </c>
       <c r="G37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I37" t="s">
         <v>22</v>
@@ -2465,28 +2462,28 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" t="s">
         <v>87</v>
       </c>
-      <c r="B38" t="s">
-        <v>88</v>
-      </c>
       <c r="C38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D38" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" t="s">
         <v>90</v>
-      </c>
-      <c r="E38" t="s">
-        <v>91</v>
       </c>
       <c r="F38" t="s">
         <v>27</v>
       </c>
       <c r="G38" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I38" t="s">
         <v>22</v>
@@ -2494,60 +2491,60 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" t="s">
         <v>87</v>
       </c>
-      <c r="B39" t="s">
-        <v>88</v>
-      </c>
       <c r="C39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D39" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F39" t="s">
         <v>27</v>
       </c>
       <c r="G39" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I39" t="s">
         <v>22</v>
       </c>
       <c r="J39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>86</v>
+      </c>
+      <c r="B40" t="s">
         <v>87</v>
       </c>
-      <c r="B40" t="s">
-        <v>88</v>
-      </c>
       <c r="C40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D40" t="s">
+        <v>89</v>
+      </c>
+      <c r="E40" t="s">
         <v>90</v>
-      </c>
-      <c r="E40" t="s">
-        <v>91</v>
       </c>
       <c r="F40" t="s">
         <v>27</v>
       </c>
       <c r="G40" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H40" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I40" t="s">
         <v>22</v>
@@ -2555,28 +2552,28 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>86</v>
+      </c>
+      <c r="B41" t="s">
         <v>87</v>
       </c>
-      <c r="B41" t="s">
-        <v>88</v>
-      </c>
       <c r="C41" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D41" t="s">
+        <v>89</v>
+      </c>
+      <c r="E41" t="s">
         <v>90</v>
-      </c>
-      <c r="E41" t="s">
-        <v>91</v>
       </c>
       <c r="F41" t="s">
         <v>27</v>
       </c>
       <c r="G41" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I41" t="s">
         <v>22</v>
@@ -2584,28 +2581,28 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>86</v>
+      </c>
+      <c r="B42" t="s">
         <v>87</v>
       </c>
-      <c r="B42" t="s">
-        <v>88</v>
-      </c>
       <c r="C42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D42" t="s">
+        <v>89</v>
+      </c>
+      <c r="E42" t="s">
         <v>90</v>
-      </c>
-      <c r="E42" t="s">
-        <v>91</v>
       </c>
       <c r="F42" t="s">
         <v>27</v>
       </c>
       <c r="G42" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H42" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I42" t="s">
         <v>22</v>
@@ -2613,220 +2610,220 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>124</v>
+      </c>
+      <c r="B43" t="s">
         <v>125</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>126</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
+        <v>112</v>
+      </c>
+      <c r="E43" t="s">
         <v>127</v>
       </c>
-      <c r="D43" t="s">
-        <v>113</v>
-      </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>128</v>
-      </c>
-      <c r="F43" t="s">
-        <v>129</v>
       </c>
       <c r="G43" t="s">
         <v>16</v>
       </c>
       <c r="H43" t="s">
+        <v>129</v>
+      </c>
+      <c r="I43" t="s">
+        <v>22</v>
+      </c>
+      <c r="J43" t="s">
         <v>130</v>
-      </c>
-      <c r="I43" t="s">
-        <v>22</v>
-      </c>
-      <c r="J43" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>124</v>
+      </c>
+      <c r="B44" t="s">
         <v>125</v>
       </c>
-      <c r="B44" t="s">
-        <v>126</v>
-      </c>
       <c r="C44" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D44" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F44" t="s">
         <v>128</v>
-      </c>
-      <c r="F44" t="s">
-        <v>129</v>
       </c>
       <c r="G44" t="s">
         <v>16</v>
       </c>
       <c r="H44" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I44" t="s">
         <v>22</v>
       </c>
       <c r="J44" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>124</v>
+      </c>
+      <c r="B45" t="s">
         <v>125</v>
       </c>
-      <c r="B45" t="s">
-        <v>126</v>
-      </c>
       <c r="C45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E45" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G45" t="s">
         <v>16</v>
       </c>
       <c r="H45" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I45" t="s">
         <v>22</v>
       </c>
       <c r="J45" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" t="s">
         <v>125</v>
       </c>
-      <c r="B46" t="s">
-        <v>126</v>
-      </c>
       <c r="C46" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D46" t="s">
+        <v>77</v>
+      </c>
+      <c r="E46" t="s">
         <v>78</v>
       </c>
-      <c r="E46" t="s">
-        <v>79</v>
-      </c>
       <c r="F46" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G46" t="s">
         <v>16</v>
       </c>
       <c r="H46" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I46" t="s">
         <v>22</v>
       </c>
       <c r="J46" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>124</v>
+      </c>
+      <c r="B47" t="s">
         <v>125</v>
       </c>
-      <c r="B47" t="s">
-        <v>126</v>
-      </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G47" t="s">
         <v>21</v>
       </c>
       <c r="H47" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I47" t="s">
         <v>22</v>
       </c>
       <c r="J47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" t="s">
         <v>140</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>141</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>142</v>
       </c>
-      <c r="D48" t="s">
-        <v>143</v>
-      </c>
       <c r="E48" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F48" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G48" t="s">
         <v>16</v>
       </c>
       <c r="H48" t="s">
+        <v>143</v>
+      </c>
+      <c r="I48" t="s">
+        <v>22</v>
+      </c>
+      <c r="J48" t="s">
         <v>144</v>
-      </c>
-      <c r="I48" t="s">
-        <v>22</v>
-      </c>
-      <c r="J48" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>139</v>
+      </c>
+      <c r="B49" t="s">
         <v>140</v>
       </c>
-      <c r="B49" t="s">
-        <v>141</v>
-      </c>
       <c r="C49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D49" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E49" t="s">
+        <v>127</v>
+      </c>
+      <c r="F49" t="s">
         <v>128</v>
-      </c>
-      <c r="F49" t="s">
-        <v>129</v>
       </c>
       <c r="G49" t="s">
         <v>16</v>
       </c>
       <c r="H49" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I49" t="s">
         <v>22</v>
@@ -2834,92 +2831,92 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>139</v>
+      </c>
+      <c r="B50" t="s">
         <v>140</v>
       </c>
-      <c r="B50" t="s">
-        <v>141</v>
-      </c>
       <c r="C50" t="s">
+        <v>146</v>
+      </c>
+      <c r="D50" t="s">
+        <v>142</v>
+      </c>
+      <c r="E50" t="s">
         <v>147</v>
       </c>
-      <c r="D50" t="s">
-        <v>143</v>
-      </c>
-      <c r="E50" t="s">
-        <v>148</v>
-      </c>
       <c r="F50" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G50" t="s">
         <v>21</v>
       </c>
       <c r="H50" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I50" t="s">
         <v>22</v>
       </c>
       <c r="J50" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>139</v>
+      </c>
+      <c r="B51" t="s">
         <v>140</v>
       </c>
-      <c r="B51" t="s">
-        <v>141</v>
-      </c>
       <c r="C51" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D51" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E51" t="s">
+        <v>127</v>
+      </c>
+      <c r="F51" t="s">
         <v>128</v>
-      </c>
-      <c r="F51" t="s">
-        <v>129</v>
       </c>
       <c r="G51" t="s">
         <v>21</v>
       </c>
       <c r="H51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I51" t="s">
         <v>22</v>
       </c>
       <c r="J51" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>139</v>
+      </c>
+      <c r="B52" t="s">
         <v>140</v>
       </c>
-      <c r="B52" t="s">
-        <v>141</v>
-      </c>
       <c r="C52" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D52" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E52" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52" t="s">
         <v>128</v>
-      </c>
-      <c r="F52" t="s">
-        <v>129</v>
       </c>
       <c r="G52" t="s">
         <v>21</v>
       </c>
       <c r="H52" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I52" t="s">
         <v>22</v>
@@ -2927,188 +2924,188 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>139</v>
+      </c>
+      <c r="B53" t="s">
         <v>140</v>
       </c>
-      <c r="B53" t="s">
-        <v>141</v>
-      </c>
       <c r="C53" t="s">
+        <v>152</v>
+      </c>
+      <c r="D53" t="s">
+        <v>142</v>
+      </c>
+      <c r="E53" t="s">
         <v>153</v>
       </c>
-      <c r="D53" t="s">
-        <v>143</v>
-      </c>
-      <c r="E53" t="s">
-        <v>154</v>
-      </c>
       <c r="F53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G53" t="s">
         <v>21</v>
       </c>
       <c r="H53" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I53" t="s">
         <v>22</v>
       </c>
       <c r="J53" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>139</v>
+      </c>
+      <c r="B54" t="s">
         <v>140</v>
       </c>
-      <c r="B54" t="s">
-        <v>141</v>
-      </c>
       <c r="C54" t="s">
+        <v>155</v>
+      </c>
+      <c r="D54" t="s">
+        <v>142</v>
+      </c>
+      <c r="E54" t="s">
+        <v>147</v>
+      </c>
+      <c r="F54" t="s">
+        <v>128</v>
+      </c>
+      <c r="G54" t="s">
+        <v>116</v>
+      </c>
+      <c r="H54" t="s">
+        <v>143</v>
+      </c>
+      <c r="I54" t="s">
+        <v>22</v>
+      </c>
+      <c r="J54" t="s">
         <v>156</v>
-      </c>
-      <c r="D54" t="s">
-        <v>143</v>
-      </c>
-      <c r="E54" t="s">
-        <v>148</v>
-      </c>
-      <c r="F54" t="s">
-        <v>129</v>
-      </c>
-      <c r="G54" t="s">
-        <v>117</v>
-      </c>
-      <c r="H54" t="s">
-        <v>144</v>
-      </c>
-      <c r="I54" t="s">
-        <v>22</v>
-      </c>
-      <c r="J54" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>139</v>
+      </c>
+      <c r="B55" t="s">
         <v>140</v>
       </c>
-      <c r="B55" t="s">
-        <v>141</v>
-      </c>
       <c r="C55" t="s">
+        <v>157</v>
+      </c>
+      <c r="D55" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" t="s">
+        <v>127</v>
+      </c>
+      <c r="F55" t="s">
+        <v>128</v>
+      </c>
+      <c r="G55" t="s">
+        <v>116</v>
+      </c>
+      <c r="H55" t="s">
+        <v>143</v>
+      </c>
+      <c r="I55" t="s">
+        <v>22</v>
+      </c>
+      <c r="J55" t="s">
         <v>158</v>
-      </c>
-      <c r="D55" t="s">
-        <v>74</v>
-      </c>
-      <c r="E55" t="s">
-        <v>128</v>
-      </c>
-      <c r="F55" t="s">
-        <v>129</v>
-      </c>
-      <c r="G55" t="s">
-        <v>117</v>
-      </c>
-      <c r="H55" t="s">
-        <v>144</v>
-      </c>
-      <c r="I55" t="s">
-        <v>22</v>
-      </c>
-      <c r="J55" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>139</v>
+      </c>
+      <c r="B56" t="s">
         <v>140</v>
       </c>
-      <c r="B56" t="s">
-        <v>141</v>
-      </c>
       <c r="C56" t="s">
+        <v>159</v>
+      </c>
+      <c r="D56" t="s">
+        <v>142</v>
+      </c>
+      <c r="E56" t="s">
+        <v>127</v>
+      </c>
+      <c r="F56" t="s">
+        <v>128</v>
+      </c>
+      <c r="G56" t="s">
+        <v>116</v>
+      </c>
+      <c r="H56" t="s">
+        <v>143</v>
+      </c>
+      <c r="I56" t="s">
+        <v>22</v>
+      </c>
+      <c r="J56" t="s">
         <v>160</v>
-      </c>
-      <c r="D56" t="s">
-        <v>143</v>
-      </c>
-      <c r="E56" t="s">
-        <v>128</v>
-      </c>
-      <c r="F56" t="s">
-        <v>129</v>
-      </c>
-      <c r="G56" t="s">
-        <v>117</v>
-      </c>
-      <c r="H56" t="s">
-        <v>144</v>
-      </c>
-      <c r="I56" t="s">
-        <v>22</v>
-      </c>
-      <c r="J56" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>161</v>
+      </c>
+      <c r="B57" t="s">
         <v>162</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>163</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
+        <v>103</v>
+      </c>
+      <c r="E57" t="s">
         <v>164</v>
       </c>
-      <c r="D57" t="s">
-        <v>104</v>
-      </c>
-      <c r="E57" t="s">
-        <v>165</v>
-      </c>
       <c r="F57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G57" t="s">
         <v>16</v>
       </c>
       <c r="H57" t="s">
+        <v>165</v>
+      </c>
+      <c r="I57" t="s">
+        <v>22</v>
+      </c>
+      <c r="J57" t="s">
         <v>166</v>
-      </c>
-      <c r="I57" t="s">
-        <v>22</v>
-      </c>
-      <c r="J57" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>161</v>
+      </c>
+      <c r="B58" t="s">
         <v>162</v>
       </c>
-      <c r="B58" t="s">
-        <v>163</v>
-      </c>
       <c r="C58" t="s">
+        <v>167</v>
+      </c>
+      <c r="D58" t="s">
         <v>168</v>
       </c>
-      <c r="D58" t="s">
-        <v>169</v>
-      </c>
       <c r="E58" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F58" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G58" t="s">
         <v>21</v>
       </c>
       <c r="H58" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I58" t="s">
         <v>22</v>
@@ -3116,124 +3113,124 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>161</v>
+      </c>
+      <c r="B59" t="s">
         <v>162</v>
       </c>
-      <c r="B59" t="s">
-        <v>163</v>
-      </c>
       <c r="C59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D59" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E59" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F59" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G59" t="s">
         <v>21</v>
       </c>
       <c r="H59" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I59" t="s">
         <v>22</v>
       </c>
       <c r="J59" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>161</v>
+      </c>
+      <c r="B60" t="s">
         <v>162</v>
       </c>
-      <c r="B60" t="s">
-        <v>163</v>
-      </c>
       <c r="C60" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D60" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E60" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F60" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G60" t="s">
         <v>21</v>
       </c>
       <c r="H60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I60" t="s">
         <v>22</v>
       </c>
       <c r="J60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>161</v>
+      </c>
+      <c r="B61" t="s">
         <v>162</v>
       </c>
-      <c r="B61" t="s">
-        <v>163</v>
-      </c>
       <c r="C61" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D61" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E61" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F61" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G61" t="s">
         <v>21</v>
       </c>
       <c r="H61" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I61" t="s">
         <v>22</v>
       </c>
       <c r="J61" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>161</v>
+      </c>
+      <c r="B62" t="s">
         <v>162</v>
       </c>
-      <c r="B62" t="s">
-        <v>163</v>
-      </c>
       <c r="C62" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E62" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G62" t="s">
         <v>21</v>
       </c>
       <c r="H62" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I62" t="s">
         <v>22</v>
@@ -3241,51 +3238,51 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>161</v>
+      </c>
+      <c r="B63" t="s">
         <v>162</v>
       </c>
-      <c r="B63" t="s">
-        <v>163</v>
-      </c>
       <c r="C63" t="s">
+        <v>176</v>
+      </c>
+      <c r="D63" t="s">
+        <v>142</v>
+      </c>
+      <c r="E63" t="s">
         <v>177</v>
       </c>
-      <c r="D63" t="s">
-        <v>143</v>
-      </c>
-      <c r="E63" t="s">
-        <v>178</v>
-      </c>
       <c r="F63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G63" t="s">
         <v>21</v>
       </c>
       <c r="H63" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I63" t="s">
         <v>22</v>
       </c>
       <c r="J63" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>161</v>
+      </c>
+      <c r="B64" t="s">
         <v>162</v>
       </c>
-      <c r="B64" t="s">
-        <v>163</v>
-      </c>
       <c r="C64" t="s">
+        <v>179</v>
+      </c>
+      <c r="D64" t="s">
+        <v>103</v>
+      </c>
+      <c r="E64" t="s">
         <v>180</v>
-      </c>
-      <c r="D64" t="s">
-        <v>104</v>
-      </c>
-      <c r="E64" t="s">
-        <v>181</v>
       </c>
       <c r="F64" t="s">
         <v>27</v>
@@ -3294,7 +3291,7 @@
         <v>21</v>
       </c>
       <c r="H64" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I64" t="s">
         <v>22</v>
@@ -3302,124 +3299,124 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>161</v>
+      </c>
+      <c r="B65" t="s">
         <v>162</v>
       </c>
-      <c r="B65" t="s">
-        <v>163</v>
-      </c>
       <c r="C65" t="s">
+        <v>181</v>
+      </c>
+      <c r="D65" t="s">
+        <v>53</v>
+      </c>
+      <c r="E65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F65" t="s">
+        <v>70</v>
+      </c>
+      <c r="G65" t="s">
+        <v>116</v>
+      </c>
+      <c r="H65" t="s">
+        <v>165</v>
+      </c>
+      <c r="I65" t="s">
+        <v>22</v>
+      </c>
+      <c r="J65" t="s">
         <v>182</v>
-      </c>
-      <c r="D65" t="s">
-        <v>54</v>
-      </c>
-      <c r="E65" t="s">
-        <v>128</v>
-      </c>
-      <c r="F65" t="s">
-        <v>71</v>
-      </c>
-      <c r="G65" t="s">
-        <v>117</v>
-      </c>
-      <c r="H65" t="s">
-        <v>166</v>
-      </c>
-      <c r="I65" t="s">
-        <v>22</v>
-      </c>
-      <c r="J65" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>161</v>
+      </c>
+      <c r="B66" t="s">
         <v>162</v>
       </c>
-      <c r="B66" t="s">
-        <v>163</v>
-      </c>
       <c r="C66" t="s">
+        <v>183</v>
+      </c>
+      <c r="D66" t="s">
+        <v>53</v>
+      </c>
+      <c r="E66" t="s">
+        <v>127</v>
+      </c>
+      <c r="F66" t="s">
+        <v>70</v>
+      </c>
+      <c r="G66" t="s">
+        <v>116</v>
+      </c>
+      <c r="H66" t="s">
+        <v>165</v>
+      </c>
+      <c r="I66" t="s">
+        <v>22</v>
+      </c>
+      <c r="J66" t="s">
         <v>184</v>
-      </c>
-      <c r="D66" t="s">
-        <v>54</v>
-      </c>
-      <c r="E66" t="s">
-        <v>128</v>
-      </c>
-      <c r="F66" t="s">
-        <v>71</v>
-      </c>
-      <c r="G66" t="s">
-        <v>117</v>
-      </c>
-      <c r="H66" t="s">
-        <v>166</v>
-      </c>
-      <c r="I66" t="s">
-        <v>22</v>
-      </c>
-      <c r="J66" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>161</v>
+      </c>
+      <c r="B67" t="s">
         <v>162</v>
       </c>
-      <c r="B67" t="s">
-        <v>163</v>
-      </c>
       <c r="C67" t="s">
+        <v>185</v>
+      </c>
+      <c r="D67" t="s">
+        <v>53</v>
+      </c>
+      <c r="E67" t="s">
+        <v>127</v>
+      </c>
+      <c r="F67" t="s">
+        <v>70</v>
+      </c>
+      <c r="G67" t="s">
+        <v>116</v>
+      </c>
+      <c r="H67" t="s">
+        <v>165</v>
+      </c>
+      <c r="I67" t="s">
+        <v>22</v>
+      </c>
+      <c r="J67" t="s">
         <v>186</v>
-      </c>
-      <c r="D67" t="s">
-        <v>54</v>
-      </c>
-      <c r="E67" t="s">
-        <v>128</v>
-      </c>
-      <c r="F67" t="s">
-        <v>71</v>
-      </c>
-      <c r="G67" t="s">
-        <v>117</v>
-      </c>
-      <c r="H67" t="s">
-        <v>166</v>
-      </c>
-      <c r="I67" t="s">
-        <v>22</v>
-      </c>
-      <c r="J67" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>161</v>
+      </c>
+      <c r="B68" t="s">
         <v>162</v>
       </c>
-      <c r="B68" t="s">
-        <v>163</v>
-      </c>
       <c r="C68" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D68" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E68" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G68" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H68" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I68" t="s">
         <v>22</v>
@@ -3427,28 +3424,28 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>161</v>
+      </c>
+      <c r="B69" t="s">
         <v>162</v>
       </c>
-      <c r="B69" t="s">
-        <v>163</v>
-      </c>
       <c r="C69" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D69" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E69" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H69" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I69" t="s">
         <v>22</v>
@@ -3456,92 +3453,92 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>161</v>
+      </c>
+      <c r="B70" t="s">
         <v>162</v>
       </c>
-      <c r="B70" t="s">
-        <v>163</v>
-      </c>
       <c r="C70" t="s">
+        <v>189</v>
+      </c>
+      <c r="D70" t="s">
+        <v>168</v>
+      </c>
+      <c r="E70" t="s">
+        <v>127</v>
+      </c>
+      <c r="F70" t="s">
+        <v>70</v>
+      </c>
+      <c r="G70" t="s">
+        <v>116</v>
+      </c>
+      <c r="H70" t="s">
+        <v>165</v>
+      </c>
+      <c r="I70" t="s">
+        <v>22</v>
+      </c>
+      <c r="J70" t="s">
         <v>190</v>
-      </c>
-      <c r="D70" t="s">
-        <v>169</v>
-      </c>
-      <c r="E70" t="s">
-        <v>128</v>
-      </c>
-      <c r="F70" t="s">
-        <v>71</v>
-      </c>
-      <c r="G70" t="s">
-        <v>117</v>
-      </c>
-      <c r="H70" t="s">
-        <v>166</v>
-      </c>
-      <c r="I70" t="s">
-        <v>22</v>
-      </c>
-      <c r="J70" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>161</v>
+      </c>
+      <c r="B71" t="s">
         <v>162</v>
       </c>
-      <c r="B71" t="s">
-        <v>163</v>
-      </c>
       <c r="C71" t="s">
+        <v>191</v>
+      </c>
+      <c r="D71" t="s">
+        <v>168</v>
+      </c>
+      <c r="E71" t="s">
+        <v>127</v>
+      </c>
+      <c r="F71" t="s">
+        <v>70</v>
+      </c>
+      <c r="G71" t="s">
+        <v>116</v>
+      </c>
+      <c r="H71" t="s">
+        <v>165</v>
+      </c>
+      <c r="I71" t="s">
+        <v>22</v>
+      </c>
+      <c r="J71" t="s">
         <v>192</v>
-      </c>
-      <c r="D71" t="s">
-        <v>169</v>
-      </c>
-      <c r="E71" t="s">
-        <v>128</v>
-      </c>
-      <c r="F71" t="s">
-        <v>71</v>
-      </c>
-      <c r="G71" t="s">
-        <v>117</v>
-      </c>
-      <c r="H71" t="s">
-        <v>166</v>
-      </c>
-      <c r="I71" t="s">
-        <v>22</v>
-      </c>
-      <c r="J71" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>161</v>
+      </c>
+      <c r="B72" t="s">
         <v>162</v>
       </c>
-      <c r="B72" t="s">
-        <v>163</v>
-      </c>
       <c r="C72" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D72" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F72" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G72" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H72" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I72" t="s">
         <v>22</v>
@@ -3549,28 +3546,28 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>194</v>
+      </c>
+      <c r="B73" t="s">
         <v>195</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>196</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>197</v>
       </c>
-      <c r="D73" t="s">
-        <v>198</v>
-      </c>
       <c r="E73" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F73" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G73" t="s">
         <v>21</v>
       </c>
       <c r="H73" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I73" t="s">
         <v>22</v>
@@ -3578,28 +3575,28 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>194</v>
+      </c>
+      <c r="B74" t="s">
         <v>195</v>
       </c>
-      <c r="B74" t="s">
-        <v>196</v>
-      </c>
       <c r="C74" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D74" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E74" t="s">
+        <v>127</v>
+      </c>
+      <c r="F74" t="s">
         <v>128</v>
-      </c>
-      <c r="F74" t="s">
-        <v>129</v>
       </c>
       <c r="G74" t="s">
         <v>21</v>
       </c>
       <c r="H74" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I74" t="s">
         <v>22</v>
@@ -3607,92 +3604,92 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>194</v>
+      </c>
+      <c r="B75" t="s">
         <v>195</v>
       </c>
-      <c r="B75" t="s">
-        <v>196</v>
-      </c>
       <c r="C75" t="s">
+        <v>200</v>
+      </c>
+      <c r="D75" t="s">
+        <v>168</v>
+      </c>
+      <c r="E75" t="s">
         <v>201</v>
       </c>
-      <c r="D75" t="s">
-        <v>169</v>
-      </c>
-      <c r="E75" t="s">
-        <v>202</v>
-      </c>
       <c r="F75" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G75" t="s">
         <v>21</v>
       </c>
       <c r="H75" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I75" t="s">
         <v>22</v>
       </c>
       <c r="J75" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>194</v>
+      </c>
+      <c r="B76" t="s">
         <v>195</v>
       </c>
-      <c r="B76" t="s">
-        <v>196</v>
-      </c>
       <c r="C76" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D76" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E76" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F76" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G76" t="s">
         <v>21</v>
       </c>
       <c r="H76" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I76" t="s">
         <v>22</v>
       </c>
       <c r="J76" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>194</v>
+      </c>
+      <c r="B77" t="s">
         <v>195</v>
       </c>
-      <c r="B77" t="s">
-        <v>196</v>
-      </c>
       <c r="C77" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D77" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E77" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F77" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G77" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H77" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I77" t="s">
         <v>22</v>
@@ -3700,188 +3697,188 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>194</v>
+      </c>
+      <c r="B78" t="s">
         <v>195</v>
       </c>
-      <c r="B78" t="s">
-        <v>196</v>
-      </c>
       <c r="C78" t="s">
+        <v>206</v>
+      </c>
+      <c r="D78" t="s">
         <v>207</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
+        <v>127</v>
+      </c>
+      <c r="F78" t="s">
+        <v>70</v>
+      </c>
+      <c r="G78" t="s">
+        <v>116</v>
+      </c>
+      <c r="H78" t="s">
+        <v>198</v>
+      </c>
+      <c r="I78" t="s">
+        <v>22</v>
+      </c>
+      <c r="J78" t="s">
         <v>208</v>
-      </c>
-      <c r="E78" t="s">
-        <v>128</v>
-      </c>
-      <c r="F78" t="s">
-        <v>71</v>
-      </c>
-      <c r="G78" t="s">
-        <v>117</v>
-      </c>
-      <c r="H78" t="s">
-        <v>199</v>
-      </c>
-      <c r="I78" t="s">
-        <v>22</v>
-      </c>
-      <c r="J78" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>194</v>
+      </c>
+      <c r="B79" t="s">
         <v>195</v>
       </c>
-      <c r="B79" t="s">
-        <v>196</v>
-      </c>
       <c r="C79" t="s">
+        <v>209</v>
+      </c>
+      <c r="D79" t="s">
+        <v>207</v>
+      </c>
+      <c r="E79" t="s">
+        <v>127</v>
+      </c>
+      <c r="F79" t="s">
+        <v>70</v>
+      </c>
+      <c r="G79" t="s">
+        <v>116</v>
+      </c>
+      <c r="H79" t="s">
+        <v>198</v>
+      </c>
+      <c r="I79" t="s">
+        <v>22</v>
+      </c>
+      <c r="J79" t="s">
         <v>210</v>
-      </c>
-      <c r="D79" t="s">
-        <v>208</v>
-      </c>
-      <c r="E79" t="s">
-        <v>128</v>
-      </c>
-      <c r="F79" t="s">
-        <v>71</v>
-      </c>
-      <c r="G79" t="s">
-        <v>117</v>
-      </c>
-      <c r="H79" t="s">
-        <v>199</v>
-      </c>
-      <c r="I79" t="s">
-        <v>22</v>
-      </c>
-      <c r="J79" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>194</v>
+      </c>
+      <c r="B80" t="s">
         <v>195</v>
       </c>
-      <c r="B80" t="s">
-        <v>196</v>
-      </c>
       <c r="C80" t="s">
+        <v>211</v>
+      </c>
+      <c r="D80" t="s">
+        <v>207</v>
+      </c>
+      <c r="E80" t="s">
+        <v>127</v>
+      </c>
+      <c r="F80" t="s">
+        <v>70</v>
+      </c>
+      <c r="G80" t="s">
+        <v>116</v>
+      </c>
+      <c r="H80" t="s">
+        <v>198</v>
+      </c>
+      <c r="I80" t="s">
+        <v>22</v>
+      </c>
+      <c r="J80" t="s">
         <v>212</v>
-      </c>
-      <c r="D80" t="s">
-        <v>208</v>
-      </c>
-      <c r="E80" t="s">
-        <v>128</v>
-      </c>
-      <c r="F80" t="s">
-        <v>71</v>
-      </c>
-      <c r="G80" t="s">
-        <v>117</v>
-      </c>
-      <c r="H80" t="s">
-        <v>199</v>
-      </c>
-      <c r="I80" t="s">
-        <v>22</v>
-      </c>
-      <c r="J80" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>213</v>
+      </c>
+      <c r="B81" t="s">
         <v>214</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>215</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
+        <v>48</v>
+      </c>
+      <c r="E81" t="s">
         <v>216</v>
-      </c>
-      <c r="D81" t="s">
-        <v>49</v>
-      </c>
-      <c r="E81" t="s">
-        <v>217</v>
       </c>
       <c r="F81" t="s">
         <v>27</v>
       </c>
       <c r="G81" t="s">
+        <v>217</v>
+      </c>
+      <c r="H81" t="s">
         <v>218</v>
       </c>
-      <c r="H81" t="s">
+      <c r="I81" t="s">
+        <v>22</v>
+      </c>
+      <c r="J81" t="s">
         <v>219</v>
-      </c>
-      <c r="I81" t="s">
-        <v>22</v>
-      </c>
-      <c r="J81" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>213</v>
+      </c>
+      <c r="B82" t="s">
         <v>214</v>
       </c>
-      <c r="B82" t="s">
-        <v>215</v>
-      </c>
       <c r="C82" t="s">
+        <v>220</v>
+      </c>
+      <c r="D82" t="s">
         <v>221</v>
       </c>
-      <c r="D82" t="s">
+      <c r="E82" t="s">
+        <v>147</v>
+      </c>
+      <c r="F82" t="s">
+        <v>70</v>
+      </c>
+      <c r="G82" t="s">
+        <v>217</v>
+      </c>
+      <c r="H82" t="s">
+        <v>218</v>
+      </c>
+      <c r="I82" t="s">
+        <v>22</v>
+      </c>
+      <c r="J82" t="s">
         <v>222</v>
-      </c>
-      <c r="E82" t="s">
-        <v>148</v>
-      </c>
-      <c r="F82" t="s">
-        <v>71</v>
-      </c>
-      <c r="G82" t="s">
-        <v>218</v>
-      </c>
-      <c r="H82" t="s">
-        <v>219</v>
-      </c>
-      <c r="I82" t="s">
-        <v>22</v>
-      </c>
-      <c r="J82" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>213</v>
+      </c>
+      <c r="B83" t="s">
         <v>214</v>
       </c>
-      <c r="B83" t="s">
-        <v>215</v>
-      </c>
       <c r="C83" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D83" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E83" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F83" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G83" t="s">
+        <v>217</v>
+      </c>
+      <c r="H83" t="s">
         <v>218</v>
-      </c>
-      <c r="H83" t="s">
-        <v>219</v>
       </c>
       <c r="I83" t="s">
         <v>22</v>
@@ -3889,252 +3886,252 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>213</v>
+      </c>
+      <c r="B84" t="s">
         <v>214</v>
       </c>
-      <c r="B84" t="s">
-        <v>215</v>
-      </c>
       <c r="C84" t="s">
+        <v>224</v>
+      </c>
+      <c r="D84" t="s">
+        <v>221</v>
+      </c>
+      <c r="E84" t="s">
+        <v>127</v>
+      </c>
+      <c r="F84" t="s">
+        <v>70</v>
+      </c>
+      <c r="G84" t="s">
+        <v>217</v>
+      </c>
+      <c r="H84" t="s">
+        <v>218</v>
+      </c>
+      <c r="I84" t="s">
+        <v>22</v>
+      </c>
+      <c r="J84" t="s">
         <v>225</v>
-      </c>
-      <c r="D84" t="s">
-        <v>222</v>
-      </c>
-      <c r="E84" t="s">
-        <v>128</v>
-      </c>
-      <c r="F84" t="s">
-        <v>71</v>
-      </c>
-      <c r="G84" t="s">
-        <v>218</v>
-      </c>
-      <c r="H84" t="s">
-        <v>219</v>
-      </c>
-      <c r="I84" t="s">
-        <v>22</v>
-      </c>
-      <c r="J84" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>213</v>
+      </c>
+      <c r="B85" t="s">
         <v>214</v>
       </c>
-      <c r="B85" t="s">
-        <v>215</v>
-      </c>
       <c r="C85" t="s">
+        <v>226</v>
+      </c>
+      <c r="D85" t="s">
+        <v>221</v>
+      </c>
+      <c r="E85" t="s">
+        <v>147</v>
+      </c>
+      <c r="F85" t="s">
+        <v>70</v>
+      </c>
+      <c r="G85" t="s">
+        <v>217</v>
+      </c>
+      <c r="H85" t="s">
+        <v>218</v>
+      </c>
+      <c r="I85" t="s">
+        <v>22</v>
+      </c>
+      <c r="J85" t="s">
         <v>227</v>
-      </c>
-      <c r="D85" t="s">
-        <v>222</v>
-      </c>
-      <c r="E85" t="s">
-        <v>148</v>
-      </c>
-      <c r="F85" t="s">
-        <v>71</v>
-      </c>
-      <c r="G85" t="s">
-        <v>218</v>
-      </c>
-      <c r="H85" t="s">
-        <v>219</v>
-      </c>
-      <c r="I85" t="s">
-        <v>22</v>
-      </c>
-      <c r="J85" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>213</v>
+      </c>
+      <c r="B86" t="s">
         <v>214</v>
       </c>
-      <c r="B86" t="s">
-        <v>215</v>
-      </c>
       <c r="C86" t="s">
+        <v>228</v>
+      </c>
+      <c r="D86" t="s">
+        <v>168</v>
+      </c>
+      <c r="E86" t="s">
+        <v>127</v>
+      </c>
+      <c r="F86" t="s">
+        <v>70</v>
+      </c>
+      <c r="G86" t="s">
+        <v>217</v>
+      </c>
+      <c r="H86" t="s">
+        <v>218</v>
+      </c>
+      <c r="I86" t="s">
+        <v>22</v>
+      </c>
+      <c r="J86" t="s">
         <v>229</v>
-      </c>
-      <c r="D86" t="s">
-        <v>169</v>
-      </c>
-      <c r="E86" t="s">
-        <v>128</v>
-      </c>
-      <c r="F86" t="s">
-        <v>71</v>
-      </c>
-      <c r="G86" t="s">
-        <v>218</v>
-      </c>
-      <c r="H86" t="s">
-        <v>219</v>
-      </c>
-      <c r="I86" t="s">
-        <v>22</v>
-      </c>
-      <c r="J86" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>213</v>
+      </c>
+      <c r="B87" t="s">
         <v>214</v>
       </c>
-      <c r="B87" t="s">
-        <v>215</v>
-      </c>
       <c r="C87" t="s">
+        <v>230</v>
+      </c>
+      <c r="D87" t="s">
+        <v>168</v>
+      </c>
+      <c r="E87" t="s">
+        <v>127</v>
+      </c>
+      <c r="F87" t="s">
+        <v>70</v>
+      </c>
+      <c r="G87" t="s">
+        <v>217</v>
+      </c>
+      <c r="H87" t="s">
+        <v>218</v>
+      </c>
+      <c r="I87" t="s">
+        <v>22</v>
+      </c>
+      <c r="J87" t="s">
         <v>231</v>
-      </c>
-      <c r="D87" t="s">
-        <v>169</v>
-      </c>
-      <c r="E87" t="s">
-        <v>128</v>
-      </c>
-      <c r="F87" t="s">
-        <v>71</v>
-      </c>
-      <c r="G87" t="s">
-        <v>218</v>
-      </c>
-      <c r="H87" t="s">
-        <v>219</v>
-      </c>
-      <c r="I87" t="s">
-        <v>22</v>
-      </c>
-      <c r="J87" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>213</v>
+      </c>
+      <c r="B88" t="s">
         <v>214</v>
       </c>
-      <c r="B88" t="s">
-        <v>215</v>
-      </c>
       <c r="C88" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D88" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E88" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G88" t="s">
+        <v>217</v>
+      </c>
+      <c r="H88" t="s">
         <v>218</v>
       </c>
-      <c r="H88" t="s">
-        <v>219</v>
-      </c>
       <c r="I88" t="s">
         <v>22</v>
       </c>
       <c r="J88" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>213</v>
+      </c>
+      <c r="B89" t="s">
         <v>214</v>
       </c>
-      <c r="B89" t="s">
-        <v>215</v>
-      </c>
       <c r="C89" t="s">
+        <v>233</v>
+      </c>
+      <c r="D89" t="s">
         <v>234</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
+        <v>127</v>
+      </c>
+      <c r="F89" t="s">
+        <v>70</v>
+      </c>
+      <c r="G89" t="s">
+        <v>217</v>
+      </c>
+      <c r="H89" t="s">
+        <v>218</v>
+      </c>
+      <c r="I89" t="s">
+        <v>22</v>
+      </c>
+      <c r="J89" t="s">
         <v>235</v>
-      </c>
-      <c r="E89" t="s">
-        <v>128</v>
-      </c>
-      <c r="F89" t="s">
-        <v>71</v>
-      </c>
-      <c r="G89" t="s">
-        <v>218</v>
-      </c>
-      <c r="H89" t="s">
-        <v>219</v>
-      </c>
-      <c r="I89" t="s">
-        <v>22</v>
-      </c>
-      <c r="J89" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>213</v>
+      </c>
+      <c r="B90" t="s">
         <v>214</v>
       </c>
-      <c r="B90" t="s">
-        <v>215</v>
-      </c>
       <c r="C90" t="s">
+        <v>236</v>
+      </c>
+      <c r="D90" t="s">
+        <v>234</v>
+      </c>
+      <c r="E90" t="s">
+        <v>127</v>
+      </c>
+      <c r="F90" t="s">
+        <v>70</v>
+      </c>
+      <c r="G90" t="s">
+        <v>217</v>
+      </c>
+      <c r="H90" t="s">
+        <v>218</v>
+      </c>
+      <c r="I90" t="s">
+        <v>22</v>
+      </c>
+      <c r="J90" t="s">
         <v>237</v>
-      </c>
-      <c r="D90" t="s">
-        <v>235</v>
-      </c>
-      <c r="E90" t="s">
-        <v>128</v>
-      </c>
-      <c r="F90" t="s">
-        <v>71</v>
-      </c>
-      <c r="G90" t="s">
-        <v>218</v>
-      </c>
-      <c r="H90" t="s">
-        <v>219</v>
-      </c>
-      <c r="I90" t="s">
-        <v>22</v>
-      </c>
-      <c r="J90" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>213</v>
+      </c>
+      <c r="B91" t="s">
         <v>214</v>
       </c>
-      <c r="B91" t="s">
-        <v>215</v>
-      </c>
       <c r="C91" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D91" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E91" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F91" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G91" t="s">
+        <v>217</v>
+      </c>
+      <c r="H91" t="s">
         <v>218</v>
-      </c>
-      <c r="H91" t="s">
-        <v>219</v>
       </c>
       <c r="I91" t="s">
         <v>22</v>
@@ -4142,60 +4139,60 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>213</v>
+      </c>
+      <c r="B92" t="s">
         <v>214</v>
       </c>
-      <c r="B92" t="s">
-        <v>215</v>
-      </c>
       <c r="C92" t="s">
+        <v>239</v>
+      </c>
+      <c r="D92" t="s">
+        <v>221</v>
+      </c>
+      <c r="E92" t="s">
+        <v>147</v>
+      </c>
+      <c r="F92" t="s">
+        <v>70</v>
+      </c>
+      <c r="G92" t="s">
+        <v>217</v>
+      </c>
+      <c r="H92" t="s">
+        <v>218</v>
+      </c>
+      <c r="I92" t="s">
+        <v>22</v>
+      </c>
+      <c r="J92" t="s">
         <v>240</v>
-      </c>
-      <c r="D92" t="s">
-        <v>222</v>
-      </c>
-      <c r="E92" t="s">
-        <v>148</v>
-      </c>
-      <c r="F92" t="s">
-        <v>71</v>
-      </c>
-      <c r="G92" t="s">
-        <v>218</v>
-      </c>
-      <c r="H92" t="s">
-        <v>219</v>
-      </c>
-      <c r="I92" t="s">
-        <v>22</v>
-      </c>
-      <c r="J92" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>213</v>
+      </c>
+      <c r="B93" t="s">
         <v>214</v>
       </c>
-      <c r="B93" t="s">
-        <v>215</v>
-      </c>
       <c r="C93" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D93" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E93" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F93" t="s">
         <v>33</v>
       </c>
       <c r="G93" t="s">
+        <v>217</v>
+      </c>
+      <c r="H93" t="s">
         <v>218</v>
-      </c>
-      <c r="H93" t="s">
-        <v>219</v>
       </c>
       <c r="I93" t="s">
         <v>22</v>
@@ -4203,51 +4200,51 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>213</v>
+      </c>
+      <c r="B94" t="s">
         <v>214</v>
       </c>
-      <c r="B94" t="s">
-        <v>215</v>
-      </c>
       <c r="C94" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D94" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E94" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F94" t="s">
         <v>33</v>
       </c>
       <c r="G94" t="s">
+        <v>217</v>
+      </c>
+      <c r="H94" t="s">
         <v>218</v>
       </c>
-      <c r="H94" t="s">
-        <v>219</v>
-      </c>
       <c r="I94" t="s">
         <v>22</v>
       </c>
       <c r="J94" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>244</v>
+      </c>
+      <c r="B95" t="s">
         <v>245</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C95" t="s">
         <v>246</v>
       </c>
-      <c r="C95" t="s">
+      <c r="D95" t="s">
+        <v>112</v>
+      </c>
+      <c r="E95" t="s">
         <v>247</v>
-      </c>
-      <c r="D95" t="s">
-        <v>113</v>
-      </c>
-      <c r="E95" t="s">
-        <v>248</v>
       </c>
       <c r="F95" t="s">
         <v>27</v>
@@ -4256,30 +4253,30 @@
         <v>16</v>
       </c>
       <c r="H95" t="s">
+        <v>248</v>
+      </c>
+      <c r="I95" t="s">
+        <v>22</v>
+      </c>
+      <c r="J95" t="s">
         <v>249</v>
-      </c>
-      <c r="I95" t="s">
-        <v>22</v>
-      </c>
-      <c r="J95" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>244</v>
+      </c>
+      <c r="B96" t="s">
         <v>245</v>
       </c>
-      <c r="B96" t="s">
-        <v>246</v>
-      </c>
       <c r="C96" t="s">
+        <v>250</v>
+      </c>
+      <c r="D96" t="s">
+        <v>112</v>
+      </c>
+      <c r="E96" t="s">
         <v>251</v>
-      </c>
-      <c r="D96" t="s">
-        <v>113</v>
-      </c>
-      <c r="E96" t="s">
-        <v>252</v>
       </c>
       <c r="F96" t="s">
         <v>27</v>
@@ -4288,30 +4285,30 @@
         <v>16</v>
       </c>
       <c r="H96" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I96" t="s">
         <v>22</v>
       </c>
       <c r="J96" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>244</v>
+      </c>
+      <c r="B97" t="s">
         <v>245</v>
       </c>
-      <c r="B97" t="s">
-        <v>246</v>
-      </c>
       <c r="C97" t="s">
+        <v>253</v>
+      </c>
+      <c r="D97" t="s">
+        <v>57</v>
+      </c>
+      <c r="E97" t="s">
         <v>254</v>
-      </c>
-      <c r="D97" t="s">
-        <v>58</v>
-      </c>
-      <c r="E97" t="s">
-        <v>255</v>
       </c>
       <c r="F97" t="s">
         <v>27</v>
@@ -4320,30 +4317,30 @@
         <v>16</v>
       </c>
       <c r="H97" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I97" t="s">
         <v>22</v>
       </c>
       <c r="J97" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>244</v>
+      </c>
+      <c r="B98" t="s">
         <v>245</v>
       </c>
-      <c r="B98" t="s">
-        <v>246</v>
-      </c>
       <c r="C98" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D98" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E98" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F98" t="s">
         <v>27</v>
@@ -4352,30 +4349,30 @@
         <v>21</v>
       </c>
       <c r="H98" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I98" t="s">
         <v>22</v>
       </c>
       <c r="J98" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>244</v>
+      </c>
+      <c r="B99" t="s">
         <v>245</v>
       </c>
-      <c r="B99" t="s">
-        <v>246</v>
-      </c>
       <c r="C99" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D99" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E99" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F99" t="s">
         <v>27</v>
@@ -4384,7 +4381,7 @@
         <v>21</v>
       </c>
       <c r="H99" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I99" t="s">
         <v>22</v>
@@ -4392,19 +4389,19 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>244</v>
+      </c>
+      <c r="B100" t="s">
         <v>245</v>
       </c>
-      <c r="B100" t="s">
-        <v>246</v>
-      </c>
       <c r="C100" t="s">
+        <v>259</v>
+      </c>
+      <c r="D100" t="s">
+        <v>57</v>
+      </c>
+      <c r="E100" t="s">
         <v>260</v>
-      </c>
-      <c r="D100" t="s">
-        <v>58</v>
-      </c>
-      <c r="E100" t="s">
-        <v>261</v>
       </c>
       <c r="F100" t="s">
         <v>27</v>
@@ -4413,7 +4410,7 @@
         <v>21</v>
       </c>
       <c r="H100" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I100" t="s">
         <v>22</v>
@@ -4421,19 +4418,19 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>244</v>
+      </c>
+      <c r="B101" t="s">
         <v>245</v>
       </c>
-      <c r="B101" t="s">
-        <v>246</v>
-      </c>
       <c r="C101" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D101" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E101" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F101" t="s">
         <v>27</v>
@@ -4442,7 +4439,7 @@
         <v>21</v>
       </c>
       <c r="H101" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I101" t="s">
         <v>22</v>
@@ -4450,19 +4447,19 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
+        <v>244</v>
+      </c>
+      <c r="B102" t="s">
         <v>245</v>
       </c>
-      <c r="B102" t="s">
-        <v>246</v>
-      </c>
       <c r="C102" t="s">
+        <v>262</v>
+      </c>
+      <c r="D102" t="s">
+        <v>57</v>
+      </c>
+      <c r="E102" t="s">
         <v>263</v>
-      </c>
-      <c r="D102" t="s">
-        <v>58</v>
-      </c>
-      <c r="E102" t="s">
-        <v>264</v>
       </c>
       <c r="F102" t="s">
         <v>27</v>
@@ -4471,103 +4468,103 @@
         <v>21</v>
       </c>
       <c r="H102" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I102" t="s">
         <v>22</v>
       </c>
       <c r="J102" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>244</v>
+      </c>
+      <c r="B103" t="s">
         <v>245</v>
       </c>
-      <c r="B103" t="s">
-        <v>246</v>
-      </c>
       <c r="C103" t="s">
+        <v>265</v>
+      </c>
+      <c r="D103" t="s">
+        <v>197</v>
+      </c>
+      <c r="E103" t="s">
         <v>266</v>
-      </c>
-      <c r="D103" t="s">
-        <v>198</v>
-      </c>
-      <c r="E103" t="s">
-        <v>267</v>
       </c>
       <c r="F103" t="s">
         <v>27</v>
       </c>
       <c r="G103" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H103" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I103" t="s">
         <v>22</v>
       </c>
       <c r="J103" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>244</v>
+      </c>
+      <c r="B104" t="s">
         <v>245</v>
       </c>
-      <c r="B104" t="s">
-        <v>246</v>
-      </c>
       <c r="C104" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D104" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E104" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F104" t="s">
         <v>27</v>
       </c>
       <c r="G104" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H104" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I104" t="s">
         <v>22</v>
       </c>
       <c r="J104" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>244</v>
+      </c>
+      <c r="B105" t="s">
         <v>245</v>
       </c>
-      <c r="B105" t="s">
-        <v>246</v>
-      </c>
       <c r="C105" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D105" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E105" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F105" t="s">
         <v>27</v>
       </c>
       <c r="G105" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H105" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I105" t="s">
         <v>22</v>
@@ -4575,28 +4572,28 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
+        <v>244</v>
+      </c>
+      <c r="B106" t="s">
         <v>245</v>
       </c>
-      <c r="B106" t="s">
-        <v>246</v>
-      </c>
       <c r="C106" t="s">
+        <v>271</v>
+      </c>
+      <c r="D106" t="s">
+        <v>197</v>
+      </c>
+      <c r="E106" t="s">
         <v>272</v>
-      </c>
-      <c r="D106" t="s">
-        <v>198</v>
-      </c>
-      <c r="E106" t="s">
-        <v>273</v>
       </c>
       <c r="F106" t="s">
         <v>27</v>
       </c>
       <c r="G106" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H106" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I106" t="s">
         <v>22</v>
@@ -4604,34 +4601,34 @@
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
+        <v>273</v>
+      </c>
+      <c r="B107" t="s">
         <v>274</v>
       </c>
-      <c r="B107" t="s">
+      <c r="C107" t="s">
         <v>275</v>
       </c>
-      <c r="C107" t="s">
+      <c r="D107" t="s">
         <v>276</v>
       </c>
-      <c r="D107" t="s">
+      <c r="E107" t="s">
+        <v>147</v>
+      </c>
+      <c r="F107" t="s">
         <v>277</v>
       </c>
-      <c r="E107" t="s">
-        <v>148</v>
-      </c>
-      <c r="F107" t="s">
+      <c r="G107" t="s">
+        <v>277</v>
+      </c>
+      <c r="H107" t="s">
+        <v>277</v>
+      </c>
+      <c r="I107" t="s">
+        <v>22</v>
+      </c>
+      <c r="J107" t="s">
         <v>278</v>
-      </c>
-      <c r="G107" t="s">
-        <v>278</v>
-      </c>
-      <c r="H107" t="s">
-        <v>278</v>
-      </c>
-      <c r="I107" t="s">
-        <v>22</v>
-      </c>
-      <c r="J107" t="s">
-        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -4657,19 +4654,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E1" t="s">
         <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G1" t="s">
         <v>16</v>
@@ -4678,10 +4675,10 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4695,10 +4692,10 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E2" t="s">
         <v>283</v>
-      </c>
-      <c r="E2" t="s">
-        <v>284</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -4718,19 +4715,19 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
         <v>46</v>
       </c>
-      <c r="B3" t="s">
-        <v>47</v>
-      </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E3" t="s">
         <v>285</v>
-      </c>
-      <c r="E3" t="s">
-        <v>286</v>
       </c>
       <c r="F3">
         <v>11</v>
@@ -4750,19 +4747,19 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
         <v>87</v>
       </c>
-      <c r="B4" t="s">
-        <v>88</v>
-      </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D4" t="s">
+        <v>286</v>
+      </c>
+      <c r="E4" t="s">
         <v>287</v>
-      </c>
-      <c r="E4" t="s">
-        <v>288</v>
       </c>
       <c r="F4">
         <v>20</v>
@@ -4782,19 +4779,19 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" t="s">
         <v>125</v>
       </c>
-      <c r="B5" t="s">
-        <v>126</v>
-      </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E5" t="s">
         <v>289</v>
-      </c>
-      <c r="E5" t="s">
-        <v>290</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -4814,19 +4811,19 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" t="s">
         <v>140</v>
       </c>
-      <c r="B6" t="s">
-        <v>141</v>
-      </c>
       <c r="C6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -4846,19 +4843,19 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B7" t="s">
         <v>162</v>
       </c>
-      <c r="B7" t="s">
-        <v>163</v>
-      </c>
       <c r="C7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D7" t="s">
+        <v>291</v>
+      </c>
+      <c r="E7" t="s">
         <v>292</v>
-      </c>
-      <c r="E7" t="s">
-        <v>293</v>
       </c>
       <c r="F7">
         <v>16</v>
@@ -4878,19 +4875,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B8" t="s">
         <v>195</v>
       </c>
-      <c r="B8" t="s">
-        <v>196</v>
-      </c>
       <c r="C8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D8" t="s">
+        <v>293</v>
+      </c>
+      <c r="E8" t="s">
         <v>294</v>
-      </c>
-      <c r="E8" t="s">
-        <v>295</v>
       </c>
       <c r="F8">
         <v>8</v>
@@ -4910,19 +4907,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" t="s">
         <v>214</v>
       </c>
-      <c r="B9" t="s">
-        <v>215</v>
-      </c>
       <c r="C9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F9">
         <v>14</v>
@@ -4942,19 +4939,19 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" t="s">
         <v>245</v>
       </c>
-      <c r="B10" t="s">
-        <v>246</v>
-      </c>
       <c r="C10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F10">
         <v>12</v>
@@ -4974,19 +4971,19 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B11" t="s">
         <v>274</v>
       </c>
-      <c r="B11" t="s">
-        <v>275</v>
-      </c>
       <c r="C11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F11">
         <v>1</v>

</xml_diff>

<commit_message>
Decide repo-consolidation question: not needed right now
No other developers are working on the application at the moment, so
there's no collaborator-access-management need driving a move to a
GitHub Organization -- the entire benefit it would add. Revisit if/when
a freelancer or team member joins.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="298">
   <si>
     <t>Phase</t>
   </si>
@@ -83,13 +83,16 @@
     <t>Should</t>
   </si>
   <si>
+    <t>Postponed</t>
+  </si>
+  <si>
+    <t>Only worth doing for cleaner team/collaborator access management going forward — ownership risk itself is already resolved. Decided 2026-08-23: not needed right now. No other developers are working on this application at the moment, so there's no collaborator-access-management need driving it -- the entire benefit an Organization would add. Revisit if/when a freelancer or team member joins. Real migration cost if done: every Vercel project's git integration would need manually reconnecting after any repo transfer.</t>
+  </si>
+  <si>
+    <t>Transfer or mirror the 3 repos to their final home</t>
+  </si>
+  <si>
     <t>Not started</t>
-  </si>
-  <si>
-    <t>Only worth doing for cleaner team/collaborator access management going forward — ownership risk itself is already resolved.</t>
-  </si>
-  <si>
-    <t>Transfer or mirror the 3 repos to their final home</t>
   </si>
   <si>
     <t>Depends on decision above. GitHub 'Transfer ownership' preserves history + auto-redirects; manual mirror (git push --mirror) only needed for a brand-new repo identity.</t>
@@ -1419,10 +1422,10 @@
         <v>17</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1433,7 +1436,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -1442,7 +1445,7 @@
         <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
         <v>16</v>
@@ -1451,10 +1454,10 @@
         <v>17</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -1465,10 +1468,10 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -1486,7 +1489,7 @@
         <v>18</v>
       </c>
       <c r="J6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -1497,7 +1500,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
@@ -1506,7 +1509,7 @@
         <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G7" t="s">
         <v>16</v>
@@ -1518,7 +1521,7 @@
         <v>18</v>
       </c>
       <c r="J7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -1529,16 +1532,16 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
         <v>16</v>
@@ -1550,7 +1553,7 @@
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -1561,7 +1564,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
@@ -1582,7 +1585,7 @@
         <v>18</v>
       </c>
       <c r="J9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1593,16 +1596,16 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G10" t="s">
         <v>16</v>
@@ -1614,7 +1617,7 @@
         <v>18</v>
       </c>
       <c r="J10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1625,10 +1628,10 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
         <v>14</v>
@@ -1646,2989 +1649,2989 @@
         <v>18</v>
       </c>
       <c r="J11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G12" t="s">
         <v>16</v>
       </c>
       <c r="H12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I12" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G13" t="s">
         <v>16</v>
       </c>
       <c r="H13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I13" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G14" t="s">
         <v>16</v>
       </c>
       <c r="H14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I14" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G15" t="s">
         <v>16</v>
       </c>
       <c r="H15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G16" t="s">
         <v>16</v>
       </c>
       <c r="H16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I16" t="s">
         <v>18</v>
       </c>
       <c r="J16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G17" t="s">
         <v>16</v>
       </c>
       <c r="H17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I17" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G18" t="s">
         <v>16</v>
       </c>
       <c r="H18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I18" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G19" t="s">
         <v>16</v>
       </c>
       <c r="H19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I19" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G20" t="s">
         <v>16</v>
       </c>
       <c r="H20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I20" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G21" t="s">
         <v>21</v>
       </c>
       <c r="H21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I21" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G22" t="s">
         <v>21</v>
       </c>
       <c r="H22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I22" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G23" t="s">
         <v>16</v>
       </c>
       <c r="H23" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I23" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G24" t="s">
         <v>16</v>
       </c>
       <c r="H24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I24" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G25" t="s">
         <v>16</v>
       </c>
       <c r="H25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I25" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J25" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F26" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G26" t="s">
         <v>21</v>
       </c>
       <c r="H26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I26" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G27" t="s">
         <v>21</v>
       </c>
       <c r="H27" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I27" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F28" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G28" t="s">
         <v>21</v>
       </c>
       <c r="H28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I28" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E29" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G29" t="s">
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I29" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J29" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F30" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G30" t="s">
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I30" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D31" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F31" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G31" t="s">
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I31" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G32" t="s">
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I32" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D33" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F33" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G33" t="s">
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I33" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C34" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D34" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F34" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G34" t="s">
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I34" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J34" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B35" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D35" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F35" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G35" t="s">
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I35" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D36" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F36" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G36" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H36" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I36" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C37" t="s">
+        <v>118</v>
+      </c>
+      <c r="D37" t="s">
+        <v>90</v>
+      </c>
+      <c r="E37" t="s">
+        <v>91</v>
+      </c>
+      <c r="F37" t="s">
+        <v>28</v>
+      </c>
+      <c r="G37" t="s">
         <v>117</v>
       </c>
-      <c r="D37" t="s">
-        <v>89</v>
-      </c>
-      <c r="E37" t="s">
-        <v>90</v>
-      </c>
-      <c r="F37" t="s">
-        <v>27</v>
-      </c>
-      <c r="G37" t="s">
-        <v>116</v>
-      </c>
       <c r="H37" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I37" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F38" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G38" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H38" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I38" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D39" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F39" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G39" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H39" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I39" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J39" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C40" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D40" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F40" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G40" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H40" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I40" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C41" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D41" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F41" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G41" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H41" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I41" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C42" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D42" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F42" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G42" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H42" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I42" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B43" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C43" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D43" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E43" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F43" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G43" t="s">
         <v>16</v>
       </c>
       <c r="H43" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I43" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D44" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F44" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G44" t="s">
         <v>16</v>
       </c>
       <c r="H44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I44" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J44" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B45" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C45" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E45" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F45" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G45" t="s">
         <v>16</v>
       </c>
       <c r="H45" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I45" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J45" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B46" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C46" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D46" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E46" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F46" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G46" t="s">
         <v>16</v>
       </c>
       <c r="H46" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I46" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J46" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E47" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F47" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G47" t="s">
         <v>21</v>
       </c>
       <c r="H47" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I47" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J47" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E48" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F48" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G48" t="s">
         <v>16</v>
       </c>
       <c r="H48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I48" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B49" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E49" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G49" t="s">
         <v>16</v>
       </c>
       <c r="H49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I49" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B50" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F50" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G50" t="s">
         <v>21</v>
       </c>
       <c r="H50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I50" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D51" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E51" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F51" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G51" t="s">
         <v>21</v>
       </c>
       <c r="H51" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I51" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B52" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C52" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D52" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E52" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F52" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G52" t="s">
         <v>21</v>
       </c>
       <c r="H52" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I52" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B53" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D53" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E53" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F53" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G53" t="s">
         <v>21</v>
       </c>
       <c r="H53" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I53" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B54" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F54" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G54" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H54" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I54" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B55" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D55" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E55" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F55" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H55" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I55" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J55" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B56" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C56" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D56" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E56" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F56" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G56" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H56" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I56" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B57" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C57" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D57" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E57" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F57" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G57" t="s">
         <v>16</v>
       </c>
       <c r="H57" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I57" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J57" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B58" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C58" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E58" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F58" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G58" t="s">
         <v>21</v>
       </c>
       <c r="H58" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I58" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B59" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C59" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D59" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E59" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F59" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G59" t="s">
         <v>21</v>
       </c>
       <c r="H59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I59" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J59" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C60" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D60" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E60" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F60" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G60" t="s">
         <v>21</v>
       </c>
       <c r="H60" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I60" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J60" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C61" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D61" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E61" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F61" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G61" t="s">
         <v>21</v>
       </c>
       <c r="H61" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I61" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J61" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B62" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C62" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D62" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E62" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F62" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G62" t="s">
         <v>21</v>
       </c>
       <c r="H62" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I62" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C63" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D63" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E63" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F63" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G63" t="s">
         <v>21</v>
       </c>
       <c r="H63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I63" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J63" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C64" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D64" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E64" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F64" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G64" t="s">
         <v>21</v>
       </c>
       <c r="H64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I64" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C65" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D65" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E65" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G65" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H65" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I65" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J65" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C66" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D66" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E66" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F66" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G66" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H66" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I66" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J66" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C67" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D67" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F67" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G67" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I67" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J67" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B68" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C68" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D68" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E68" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F68" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G68" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I68" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C69" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D69" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E69" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F69" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G69" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H69" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I69" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C70" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E70" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F70" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H70" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I70" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J70" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C71" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E71" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F71" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G71" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H71" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I71" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J71" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B72" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C72" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D72" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E72" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F72" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G72" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H72" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I72" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B73" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C73" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D73" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E73" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F73" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G73" t="s">
         <v>21</v>
       </c>
       <c r="H73" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I73" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B74" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C74" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D74" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E74" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F74" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G74" t="s">
         <v>21</v>
       </c>
       <c r="H74" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I74" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B75" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C75" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D75" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E75" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F75" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G75" t="s">
         <v>21</v>
       </c>
       <c r="H75" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I75" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J75" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B76" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C76" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D76" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E76" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F76" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G76" t="s">
         <v>21</v>
       </c>
       <c r="H76" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I76" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J76" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B77" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C77" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D77" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E77" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F77" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G77" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H77" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I77" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C78" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D78" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E78" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F78" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G78" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H78" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I78" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J78" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B79" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C79" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D79" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E79" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F79" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G79" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H79" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I79" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J79" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B80" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C80" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D80" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E80" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F80" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G80" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H80" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I80" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J80" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B81" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C81" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D81" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E81" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F81" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G81" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H81" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I81" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J81" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B82" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C82" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D82" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E82" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F82" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G82" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H82" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I82" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J82" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B83" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C83" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D83" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E83" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F83" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G83" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H83" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I83" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B84" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C84" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D84" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E84" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F84" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G84" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H84" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I84" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J84" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B85" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C85" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D85" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E85" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F85" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G85" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H85" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I85" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J85" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B86" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C86" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D86" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E86" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F86" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G86" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H86" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I86" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J86" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B87" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C87" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D87" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E87" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F87" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G87" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H87" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I87" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J87" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B88" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C88" t="s">
+        <v>233</v>
+      </c>
+      <c r="D88" t="s">
+        <v>169</v>
+      </c>
+      <c r="E88" t="s">
+        <v>128</v>
+      </c>
+      <c r="F88" t="s">
+        <v>71</v>
+      </c>
+      <c r="G88" t="s">
+        <v>218</v>
+      </c>
+      <c r="H88" t="s">
+        <v>219</v>
+      </c>
+      <c r="I88" t="s">
+        <v>25</v>
+      </c>
+      <c r="J88" t="s">
         <v>232</v>
-      </c>
-      <c r="D88" t="s">
-        <v>168</v>
-      </c>
-      <c r="E88" t="s">
-        <v>127</v>
-      </c>
-      <c r="F88" t="s">
-        <v>70</v>
-      </c>
-      <c r="G88" t="s">
-        <v>217</v>
-      </c>
-      <c r="H88" t="s">
-        <v>218</v>
-      </c>
-      <c r="I88" t="s">
-        <v>22</v>
-      </c>
-      <c r="J88" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B89" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C89" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D89" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E89" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F89" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G89" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H89" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I89" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J89" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B90" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C90" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D90" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E90" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F90" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G90" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H90" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I90" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J90" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B91" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C91" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D91" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E91" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F91" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G91" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H91" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I91" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B92" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C92" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D92" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E92" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F92" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G92" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H92" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I92" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J92" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B93" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C93" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D93" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E93" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F93" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G93" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H93" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I93" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B94" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C94" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D94" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E94" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F94" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G94" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H94" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I94" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J94" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B95" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C95" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D95" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E95" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F95" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G95" t="s">
         <v>16</v>
       </c>
       <c r="H95" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I95" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J95" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B96" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C96" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D96" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E96" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F96" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G96" t="s">
         <v>16</v>
       </c>
       <c r="H96" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I96" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J96" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B97" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C97" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D97" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E97" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F97" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G97" t="s">
         <v>16</v>
       </c>
       <c r="H97" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I97" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J97" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B98" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C98" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D98" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E98" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F98" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G98" t="s">
         <v>21</v>
       </c>
       <c r="H98" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I98" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J98" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B99" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C99" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D99" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E99" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F99" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G99" t="s">
         <v>21</v>
       </c>
       <c r="H99" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I99" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B100" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C100" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D100" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E100" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F100" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G100" t="s">
         <v>21</v>
       </c>
       <c r="H100" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I100" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B101" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C101" t="s">
+        <v>262</v>
+      </c>
+      <c r="D101" t="s">
+        <v>58</v>
+      </c>
+      <c r="E101" t="s">
         <v>261</v>
       </c>
-      <c r="D101" t="s">
-        <v>57</v>
-      </c>
-      <c r="E101" t="s">
-        <v>260</v>
-      </c>
       <c r="F101" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G101" t="s">
         <v>21</v>
       </c>
       <c r="H101" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I101" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B102" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C102" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D102" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E102" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F102" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G102" t="s">
         <v>21</v>
       </c>
       <c r="H102" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I102" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J102" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B103" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C103" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D103" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E103" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F103" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G103" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H103" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I103" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J103" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B104" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C104" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D104" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E104" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F104" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G104" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H104" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I104" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J104" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B105" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C105" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D105" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E105" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F105" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G105" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H105" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I105" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B106" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C106" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D106" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E106" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F106" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G106" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H106" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I106" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B107" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C107" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D107" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E107" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I107" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J107" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -4654,19 +4657,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E1" t="s">
         <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G1" t="s">
         <v>16</v>
@@ -4675,10 +4678,10 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4692,10 +4695,10 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -4715,19 +4718,19 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F3">
         <v>11</v>
@@ -4747,19 +4750,19 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F4">
         <v>20</v>
@@ -4779,19 +4782,19 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -4811,19 +4814,19 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
+        <v>291</v>
+      </c>
+      <c r="E6" t="s">
         <v>290</v>
-      </c>
-      <c r="E6" t="s">
-        <v>289</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -4843,19 +4846,19 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F7">
         <v>16</v>
@@ -4875,19 +4878,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F8">
         <v>8</v>
@@ -4907,19 +4910,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D9" t="s">
+        <v>296</v>
+      </c>
+      <c r="E9" t="s">
         <v>295</v>
-      </c>
-      <c r="E9" t="s">
-        <v>294</v>
       </c>
       <c r="F9">
         <v>14</v>
@@ -4939,19 +4942,19 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F10">
         <v>12</v>
@@ -4971,19 +4974,19 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F11">
         <v>1</v>

</xml_diff>

<commit_message>
Close out env-var gaps: weather/map done, Support Link + Stripe on hold
Confirmed WEATHER_API_KEY2 and the 4 CARTO_WRI_MAP_TILE_URL vars are
already set in swales-services/.env.local -- nothing further needed
there. NEXT_PUBLIC_SUPPORT_LINK and the Stripe donation links
(designer + services) stay open, explicitly on hold per Omar until a
real business bank account exists to back them.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -125,10 +125,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -160,10 +160,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -636,7 +636,7 @@
         <v>Done</v>
       </c>
       <c r="J7" t="str">
-        <v>Prompted by finding the local Postgres port mismatch (app config assumes 5432, actual local Postgres is 5433) and DATABASE_URL silently overriding local dev intent. Done 2026-08-23. Added .env.example to all 3 repos (backend/designer/services), documenting every process.env.* var actually referenced in code. Found and flagged (not removed): backend's DB_HOST/DB_NAME/DB_USER/DB_PASS + config/database.js are dead code (DATABASE_URL always wins); EMAIL_USER/EMAIL_PASS/Password_Reset_Url/Email_verify_Url/AllowedOrigins are unused leftovers. designer + services were both missing NEXT_PUBLIC_STRIPE_LINK_3/_5/_10 locally (only _CUSTOM set). services was also missing WEATHER_API_KEY2, NEXT_PUBLIC_SUPPORT_LINK, and 4 CARTO_WRI_MAP_TILE_URL vars. Confirmed no .env/.env.local currently tracked in any repo. Historical finding: services had a real .env.local committed to git history on 2025-04-23 (c6ae545) -- every secret in it has since been rotated, no live exposure, left history as-is. See status.md for full detail.</v>
+        <v>Prompted by finding the local Postgres port mismatch (app config assumes 5432, actual local Postgres is 5433) and DATABASE_URL silently overriding local dev intent. Done 2026-08-23. Added .env.example to all 3 repos (backend/designer/services), documenting every process.env.* var actually referenced in code. Found and flagged (not removed): backend's DB_HOST/DB_NAME/DB_USER/DB_PASS + config/database.js are dead code (DATABASE_URL always wins); EMAIL_USER/EMAIL_PASS/Password_Reset_Url/Email_verify_Url/AllowedOrigins are unused leftovers. designer + services were both missing NEXT_PUBLIC_STRIPE_LINK_3/_5/_10 locally (only _CUSTOM set). services was also missing WEATHER_API_KEY2, NEXT_PUBLIC_SUPPORT_LINK, and 4 CARTO_WRI_MAP_TILE_URL vars. Confirmed no .env/.env.local currently tracked in any repo. Historical finding: services had a real .env.local committed to git history on 2025-04-23 (c6ae545) -- every secret in it has since been rotated, no live exposure, left history as-is. See status.md for full detail. Follow-up (2026-08-23): weather/map gaps confirmed resolved -- WEATHER_API_KEY2 (deliberate second OWM key, isolated rate-limit budget for the box-weather endpoint) and all 4 NEXT_PUBLIC_CARTO_WRI_MAP_TILE_URL1-4 (CARTO/WRI water-stress layer) now set in swales-services/.env.local. Support Link + Stripe donation links (NEXT_PUBLIC_SUPPORT_LINK, NEXT_PUBLIC_STRIPE_LINK_3/_5/_10/_CUSTOM across designer+services) remain ON HOLD until Omar opens a real business bank account -- code on both sides already reads identical env-var names, just needs real values once available.</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Correct production-repo claim in CLAUDE.md; flag mobile stack proposal for review
CLAUDE.md previously said this repo was live production; api.swales.app/
SwalesApp\back is. Also records the proposed React Native + Expo mobile
stack as pending sign-off before Phase B starts.
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J108"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="6.83203125"/>
     <col min="2" max="2" customWidth="1" width="28.83203125"/>
@@ -1063,28 +1063,28 @@
         <v>Finish &amp; Connect the Core</v>
       </c>
       <c r="C21" t="str">
-        <v>Decide whether wind turbine sizing should use real wind speed</v>
+        <v>Decide the mobile app tech stack (React Native + Expo proposed)</v>
       </c>
       <c r="D21" t="str">
         <v>Product decision</v>
       </c>
       <c r="E21" t="str">
-        <v>Codebase audit — Section A</v>
+        <v>New (mobile ask)</v>
       </c>
       <c r="F21" t="str">
-        <v>web</v>
+        <v>mobile</v>
       </c>
       <c r="G21" t="str">
-        <v>Should</v>
+        <v>Must</v>
       </c>
       <c r="H21" t="str">
         <v>Weeks 1-4</v>
       </c>
       <c r="I21" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="J21" t="str">
-        <v>Currently matches your own wind.txt spec verbatim, including an unused meanWindSpeed parameter — deliberately not changed until you confirm intent. A product decision, not a bug.</v>
+        <v>Proposed 2026-08-24, pending Omar's review — do not start Phase B build work until confirmed: React Native + Expo (managed, TypeScript) to match the web stack's Next.js/TypeScript; offline-first local store (WatermelonDB/SQLite) with a sync queue for field capture with no signal; auth reused from shared_backend once built, not a second auth system; external vision API for photo/plant ID at MVP, on-device model only if cost/latency demands it later; Expo push for notifications. Full reasoning in roadmap.md's "First 2 weeks" item 5 and status.md's "Next up" item 1.</v>
       </c>
     </row>
     <row r="22">
@@ -1095,16 +1095,16 @@
         <v>Finish &amp; Connect the Core</v>
       </c>
       <c r="C22" t="str">
-        <v>Reconcile plant/element schema with the long-term relationships knowledge-graph vision</v>
+        <v>Decide whether wind turbine sizing should use real wind speed</v>
       </c>
       <c r="D22" t="str">
-        <v>Core data</v>
+        <v>Product decision</v>
       </c>
       <c r="E22" t="str">
-        <v>Codebase audit — Section C</v>
+        <v>Codebase audit — Section A</v>
       </c>
       <c r="F22" t="str">
-        <v>backend</v>
+        <v>web</v>
       </c>
       <c r="G22" t="str">
         <v>Should</v>
@@ -1116,39 +1116,39 @@
         <v>Not started</v>
       </c>
       <c r="J22" t="str">
-        <v>The delivered 22-field flat schema (good_companions/avoid_near as strings) is a deliberate MVP. Your long-term vision is a ~50-field plant schema plus dozens of linked entity types (guilds, pests, diseases, cover crops...) tied together by a real relationships graph. Not a conflict — but worth a short pass now so early seed data doesn't need re-keying once the graph structure gets built, since that's explicitly a 2-3 year vision per your own notes, not this sprint.</v>
+        <v>Currently matches your own wind.txt spec verbatim, including an unused meanWindSpeed parameter — deliberately not changed until you confirm intent. A product decision, not a bug.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>A2</v>
+        <v>A</v>
       </c>
       <c r="B23" t="str">
-        <v>Analysis Engine Quick Wins (parallel)</v>
+        <v>Finish &amp; Connect the Core</v>
       </c>
       <c r="C23" t="str">
-        <v>Site comparison (two locations side-by-side: wind/solar/soil)</v>
+        <v>Reconcile plant/element schema with the long-term relationships knowledge-graph vision</v>
       </c>
       <c r="D23" t="str">
-        <v>Analysis cards</v>
+        <v>Core data</v>
       </c>
       <c r="E23" t="str">
-        <v>Codebase audit — Section B</v>
+        <v>Codebase audit — Section C</v>
       </c>
       <c r="F23" t="str">
-        <v>web</v>
+        <v>backend</v>
       </c>
       <c r="G23" t="str">
-        <v>Must</v>
+        <v>Should</v>
       </c>
       <c r="H23" t="str">
-        <v>Weeks 1-10, parallel to A/B</v>
+        <v>Weeks 1-4</v>
       </c>
       <c r="I23" t="str">
         <v>Not started</v>
       </c>
       <c r="J23" t="str">
-        <v>Split-panel layout; data's already fetched — a fast win.</v>
+        <v>The delivered 22-field flat schema (good_companions/avoid_near as strings) is a deliberate MVP. Your long-term vision is a ~50-field plant schema plus dozens of linked entity types (guilds, pests, diseases, cover crops...) tied together by a real relationships graph. Not a conflict — but worth a short pass now so early seed data doesn't need re-keying once the graph structure gets built, since that's explicitly a 2-3 year vision per your own notes, not this sprint.</v>
       </c>
     </row>
     <row r="24">
@@ -1159,7 +1159,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C24" t="str">
-        <v>Shareable link (encode lat/lng + active layer in the URL)</v>
+        <v>Site comparison (two locations side-by-side: wind/solar/soil)</v>
       </c>
       <c r="D24" t="str">
         <v>Analysis cards</v>
@@ -1180,7 +1180,7 @@
         <v>Not started</v>
       </c>
       <c r="J24" t="str">
-        <v>One-line param change — near-zero cost, ship immediately.</v>
+        <v>Split-panel layout; data's already fetched — a fast win.</v>
       </c>
     </row>
     <row r="25">
@@ -1191,7 +1191,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C25" t="str">
-        <v>PDF site report (wind + solar + soil analysis export)</v>
+        <v>Shareable link (encode lat/lng + active layer in the URL)</v>
       </c>
       <c r="D25" t="str">
         <v>Analysis cards</v>
@@ -1212,7 +1212,7 @@
         <v>Not started</v>
       </c>
       <c r="J25" t="str">
-        <v>Distinct from the design-canvas PDF export in Phase A — this is the energy/soil analysis report. The pdf skill handles generation. Also the thing monetization_framework needs to decide how to gate.</v>
+        <v>One-line param change — near-zero cost, ship immediately.</v>
       </c>
     </row>
     <row r="26">
@@ -1223,7 +1223,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C26" t="str">
-        <v>Combined renewable score (single energy-potential badge: wind + solar)</v>
+        <v>PDF site report (wind + solar + soil analysis export)</v>
       </c>
       <c r="D26" t="str">
         <v>Analysis cards</v>
@@ -1235,13 +1235,16 @@
         <v>web</v>
       </c>
       <c r="G26" t="str">
-        <v>Should</v>
+        <v>Must</v>
       </c>
       <c r="H26" t="str">
         <v>Weeks 1-10, parallel to A/B</v>
       </c>
       <c r="I26" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Distinct from the design-canvas PDF export in Phase A — this is the energy/soil analysis report. The pdf skill handles generation. Also the thing monetization_framework needs to decide how to gate.</v>
       </c>
     </row>
     <row r="27">
@@ -1252,7 +1255,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C27" t="str">
-        <v>ROI/payback calculator (electricity bill + budget -&gt; payback years)</v>
+        <v>Combined renewable score (single energy-potential badge: wind + solar)</v>
       </c>
       <c r="D27" t="str">
         <v>Analysis cards</v>
@@ -1271,9 +1274,6 @@
       </c>
       <c r="I27" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J27" t="str">
-        <v>Uses existing wind/solar data — pairs naturally with bankability in the W track.</v>
       </c>
     </row>
     <row r="28">
@@ -1284,7 +1284,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C28" t="str">
-        <v>Optimal install month recommender (seasonal solar + wind data)</v>
+        <v>ROI/payback calculator (electricity bill + budget -&gt; payback years)</v>
       </c>
       <c r="D28" t="str">
         <v>Analysis cards</v>
@@ -1305,7 +1305,7 @@
         <v>Not started</v>
       </c>
       <c r="J28" t="str">
-        <v>Built on SmartSolarAdvisor's existing seasonal data.</v>
+        <v>Uses existing wind/solar data — pairs naturally with bankability in the W track.</v>
       </c>
     </row>
     <row r="29">
@@ -1316,10 +1316,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C29" t="str">
-        <v>Onboarding tooltip tour (4-step walkthrough)</v>
+        <v>Optimal install month recommender (seasonal solar + wind data)</v>
       </c>
       <c r="D29" t="str">
-        <v>Onboarding</v>
+        <v>Analysis cards</v>
       </c>
       <c r="E29" t="str">
         <v>Codebase audit — Section B</v>
@@ -1337,7 +1337,7 @@
         <v>Not started</v>
       </c>
       <c r="J29" t="str">
-        <v>Distinct from the broader 'onboarding' beginner-mode item in Phase D — this is a lightweight tour for the existing analysis-card UI, shippable now.</v>
+        <v>Built on SmartSolarAdvisor's existing seasonal data.</v>
       </c>
     </row>
     <row r="30">
@@ -1348,10 +1348,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C30" t="str">
-        <v>Precipitation card — Option A (static: intensity badge, rainfall chart, guidance, soil-saturation estimate)</v>
+        <v>Onboarding tooltip tour (4-step walkthrough)</v>
       </c>
       <c r="D30" t="str">
-        <v>Analysis cards</v>
+        <v>Onboarding</v>
       </c>
       <c r="E30" t="str">
         <v>Codebase audit — Section B</v>
@@ -1369,7 +1369,7 @@
         <v>Not started</v>
       </c>
       <c r="J30" t="str">
-        <v>Ship this static version first (matches the SolarCard/WindDashboard pattern), per your own recommendation.</v>
+        <v>Distinct from the broader 'onboarding' beginner-mode item in Phase D — this is a lightweight tour for the existing analysis-card UI, shippable now.</v>
       </c>
     </row>
     <row r="31">
@@ -1380,7 +1380,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C31" t="str">
-        <v>Composite soil health score (0-100, weighted, with trend indicator)</v>
+        <v>Precipitation card — Option A (static: intensity badge, rainfall chart, guidance, soil-saturation estimate)</v>
       </c>
       <c r="D31" t="str">
         <v>Analysis cards</v>
@@ -1399,6 +1399,9 @@
       </c>
       <c r="I31" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Ship this static version first (matches the SolarCard/WindDashboard pattern), per your own recommendation.</v>
       </c>
     </row>
     <row r="32">
@@ -1409,7 +1412,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C32" t="str">
-        <v>Crop suitability engine (ranks wheat/maize/legumes/vegetables/fruit trees with reasons)</v>
+        <v>Composite soil health score (0-100, weighted, with trend indicator)</v>
       </c>
       <c r="D32" t="str">
         <v>Analysis cards</v>
@@ -1438,10 +1441,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C33" t="str">
-        <v>Amendment calculator (exact kg/hectare dosing)</v>
+        <v>Crop suitability engine (ranks wheat/maize/legumes/vegetables/fruit trees with reasons)</v>
       </c>
       <c r="D33" t="str">
-        <v>Calculators</v>
+        <v>Analysis cards</v>
       </c>
       <c r="E33" t="str">
         <v>Codebase audit — Section B</v>
@@ -1467,10 +1470,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C34" t="str">
-        <v>Cross-layer integration (soil x precipitation x sun x wind unified farm advisory)</v>
+        <v>Amendment calculator (exact kg/hectare dosing)</v>
       </c>
       <c r="D34" t="str">
-        <v>AI assist</v>
+        <v>Calculators</v>
       </c>
       <c r="E34" t="str">
         <v>Codebase audit — Section B</v>
@@ -1486,9 +1489,6 @@
       </c>
       <c r="I34" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J34" t="str">
-        <v>Overlaps ai_advisor/decision_layer conceptually — likely the same underlying advisory engine applied to the analysis cards instead of the design canvas. Worth deciding if these converge into one engine.</v>
       </c>
     </row>
     <row r="35">
@@ -1499,10 +1499,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C35" t="str">
-        <v>UI consistency pass (spacing, tooltips, blog-post links, subtle animation across cards)</v>
+        <v>Cross-layer integration (soil x precipitation x sun x wind unified farm advisory)</v>
       </c>
       <c r="D35" t="str">
-        <v>Onboarding</v>
+        <v>AI assist</v>
       </c>
       <c r="E35" t="str">
         <v>Codebase audit — Section B</v>
@@ -1518,6 +1518,9 @@
       </c>
       <c r="I35" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Overlaps ai_advisor/decision_layer conceptually — likely the same underlying advisory engine applied to the analysis cards instead of the design canvas. Worth deciding if these converge into one engine.</v>
       </c>
     </row>
     <row r="36">
@@ -1528,10 +1531,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C36" t="str">
-        <v>"Find best spot nearby" (draw a radius, rank top 3 solar/wind locations)</v>
+        <v>UI consistency pass (spacing, tooltips, blog-post links, subtle animation across cards)</v>
       </c>
       <c r="D36" t="str">
-        <v>Analysis cards</v>
+        <v>Onboarding</v>
       </c>
       <c r="E36" t="str">
         <v>Codebase audit — Section B</v>
@@ -1540,7 +1543,7 @@
         <v>web</v>
       </c>
       <c r="G36" t="str">
-        <v>Could</v>
+        <v>Should</v>
       </c>
       <c r="H36" t="str">
         <v>Weeks 1-10, parallel to A/B</v>
@@ -1557,7 +1560,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C37" t="str">
-        <v>Shadow/obstruction input (mark trees/buildings to adjust solar estimate)</v>
+        <v>"Find best spot nearby" (draw a radius, rank top 3 solar/wind locations)</v>
       </c>
       <c r="D37" t="str">
         <v>Analysis cards</v>
@@ -1586,7 +1589,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C38" t="str">
-        <v>Saved pins with notes (localStorage OK for v1)</v>
+        <v>Shadow/obstruction input (mark trees/buildings to adjust solar estimate)</v>
       </c>
       <c r="D38" t="str">
         <v>Analysis cards</v>
@@ -1615,10 +1618,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C39" t="str">
-        <v>RainAdvisor service — Option B (irrigation decisions, flood/runoff risk, swale/water-harvesting sizing)</v>
+        <v>Saved pins with notes (localStorage OK for v1)</v>
       </c>
       <c r="D39" t="str">
-        <v>AI assist</v>
+        <v>Analysis cards</v>
       </c>
       <c r="E39" t="str">
         <v>Codebase audit — Section B</v>
@@ -1634,9 +1637,6 @@
       </c>
       <c r="I39" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J39" t="str">
-        <v>Layer in after precipitation_card ships, the same way SmartSolarAdvisor was bolted onto the sun tracker — don't build both at once.</v>
       </c>
     </row>
     <row r="40">
@@ -1647,10 +1647,10 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C40" t="str">
-        <v>Soil depth profile visualization (SoilGrids 0-100cm)</v>
+        <v>RainAdvisor service — Option B (irrigation decisions, flood/runoff risk, swale/water-harvesting sizing)</v>
       </c>
       <c r="D40" t="str">
-        <v>Analysis cards</v>
+        <v>AI assist</v>
       </c>
       <c r="E40" t="str">
         <v>Codebase audit — Section B</v>
@@ -1666,6 +1666,9 @@
       </c>
       <c r="I40" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Layer in after precipitation_card ships, the same way SmartSolarAdvisor was bolted onto the sun tracker — don't build both at once.</v>
       </c>
     </row>
     <row r="41">
@@ -1676,7 +1679,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C41" t="str">
-        <v>Carbon sequestration estimate (tonnes/hectare/year, linked to carbon credit schemes)</v>
+        <v>Soil depth profile visualization (SoilGrids 0-100cm)</v>
       </c>
       <c r="D41" t="str">
         <v>Analysis cards</v>
@@ -1705,7 +1708,7 @@
         <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C42" t="str">
-        <v>Erosion risk score (texture + bulk density + slope + rainfall intensity)</v>
+        <v>Carbon sequestration estimate (tonnes/hectare/year, linked to carbon credit schemes)</v>
       </c>
       <c r="D42" t="str">
         <v>Analysis cards</v>
@@ -1728,34 +1731,31 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>B</v>
+        <v>A2</v>
       </c>
       <c r="B43" t="str">
-        <v>Mobile MVP — Capture &amp; Identify</v>
+        <v>Analysis Engine Quick Wins (parallel)</v>
       </c>
       <c r="C43" t="str">
-        <v>Photo recognition AI (trees, plants, flowers, mushrooms)</v>
+        <v>Erosion risk score (texture + bulk density + slope + rainfall intensity)</v>
       </c>
       <c r="D43" t="str">
-        <v>AI assist</v>
+        <v>Analysis cards</v>
       </c>
       <c r="E43" t="str">
-        <v>List B</v>
+        <v>Codebase audit — Section B</v>
       </c>
       <c r="F43" t="str">
-        <v>mobile</v>
+        <v>web</v>
       </c>
       <c r="G43" t="str">
-        <v>Must</v>
+        <v>Could</v>
       </c>
       <c r="H43" t="str">
-        <v>Weeks 5-12</v>
+        <v>Weeks 1-10, parallel to A/B</v>
       </c>
       <c r="I43" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J43" t="str">
-        <v>Merge with 'Natural identifier' below — same feature. This is the single best reason to install the mobile app.</v>
       </c>
     </row>
     <row r="44">
@@ -1766,7 +1766,7 @@
         <v>Mobile MVP — Capture &amp; Identify</v>
       </c>
       <c r="C44" t="str">
-        <v>Natural identifier</v>
+        <v>Photo recognition AI (trees, plants, flowers, mushrooms)</v>
       </c>
       <c r="D44" t="str">
         <v>AI assist</v>
@@ -1787,7 +1787,7 @@
         <v>Not started</v>
       </c>
       <c r="J44" t="str">
-        <v>Duplicate of photo_recognition — ship as one feature, not two.</v>
+        <v>Merge with 'Natural identifier' below — same feature. This is the single best reason to install the mobile app.</v>
       </c>
     </row>
     <row r="45">
@@ -1798,13 +1798,13 @@
         <v>Mobile MVP — Capture &amp; Identify</v>
       </c>
       <c r="C45" t="str">
-        <v>Location-based site/observation logging (GPS pins)</v>
+        <v>Natural identifier</v>
       </c>
       <c r="D45" t="str">
-        <v>Real-world data</v>
+        <v>AI assist</v>
       </c>
       <c r="E45" t="str">
-        <v>New (mobile ask)</v>
+        <v>List B</v>
       </c>
       <c r="F45" t="str">
         <v>mobile</v>
@@ -1819,7 +1819,7 @@
         <v>Not started</v>
       </c>
       <c r="J45" t="str">
-        <v>Foundation for biodiversity tool, mushroom map, and community map — build the pin system once, reuse everywhere.</v>
+        <v>Duplicate of photo_recognition — ship as one feature, not two.</v>
       </c>
     </row>
     <row r="46">
@@ -1830,10 +1830,10 @@
         <v>Mobile MVP — Capture &amp; Identify</v>
       </c>
       <c r="C46" t="str">
-        <v>"My Sites/Designs" synced view from web account</v>
+        <v>Location-based site/observation logging (GPS pins)</v>
       </c>
       <c r="D46" t="str">
-        <v>Infrastructure</v>
+        <v>Real-world data</v>
       </c>
       <c r="E46" t="str">
         <v>New (mobile ask)</v>
@@ -1851,7 +1851,7 @@
         <v>Not started</v>
       </c>
       <c r="J46" t="str">
-        <v>Read-only on mobile at first — don't try to rebuild the design canvas on a phone screen. Confirmed there's no existing native app to build on — this is a genuine fresh build.</v>
+        <v>Foundation for biodiversity tool, mushroom map, and community map — build the pin system once, reuse everywhere.</v>
       </c>
     </row>
     <row r="47">
@@ -1862,19 +1862,19 @@
         <v>Mobile MVP — Capture &amp; Identify</v>
       </c>
       <c r="C47" t="str">
-        <v>Weather integration</v>
+        <v>"My Sites/Designs" synced view from web account</v>
       </c>
       <c r="D47" t="str">
-        <v>Real-world data</v>
+        <v>Infrastructure</v>
       </c>
       <c r="E47" t="str">
-        <v>List B</v>
+        <v>New (mobile ask)</v>
       </c>
       <c r="F47" t="str">
-        <v>both</v>
+        <v>mobile</v>
       </c>
       <c r="G47" t="str">
-        <v>Should</v>
+        <v>Must</v>
       </c>
       <c r="H47" t="str">
         <v>Weeks 5-12</v>
@@ -1883,39 +1883,39 @@
         <v>Not started</v>
       </c>
       <c r="J47" t="str">
-        <v>Useful context for field capture; relatively cheap via a weather API.</v>
+        <v>Read-only on mobile at first — don't try to rebuild the design canvas on a phone screen. Confirmed there's no existing native app to build on — this is a genuine fresh build.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="B48" t="str">
-        <v>Mobile Social Layer</v>
+        <v>Mobile MVP — Capture &amp; Identify</v>
       </c>
       <c r="C48" t="str">
-        <v>Core social mechanics: comments, likes, sharing</v>
+        <v>Weather integration</v>
       </c>
       <c r="D48" t="str">
-        <v>Social</v>
+        <v>Real-world data</v>
       </c>
       <c r="E48" t="str">
-        <v>New (mobile ask)</v>
+        <v>List B</v>
       </c>
       <c r="F48" t="str">
-        <v>mobile</v>
+        <v>both</v>
       </c>
       <c r="G48" t="str">
-        <v>Must</v>
+        <v>Should</v>
       </c>
       <c r="H48" t="str">
-        <v>Weeks 13-19</v>
+        <v>Weeks 5-12</v>
       </c>
       <c r="I48" t="str">
         <v>Not started</v>
       </c>
       <c r="J48" t="str">
-        <v>Build once as shared infrastructure — every social feature below (community, success stories, etc.) sits on top of this.</v>
+        <v>Useful context for field capture; relatively cheap via a weather API.</v>
       </c>
     </row>
     <row r="49">
@@ -1926,13 +1926,13 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C49" t="str">
-        <v>Community (feed of designs/observations)</v>
+        <v>Core social mechanics: comments, likes, sharing</v>
       </c>
       <c r="D49" t="str">
         <v>Social</v>
       </c>
       <c r="E49" t="str">
-        <v>List B</v>
+        <v>New (mobile ask)</v>
       </c>
       <c r="F49" t="str">
         <v>mobile</v>
@@ -1945,6 +1945,9 @@
       </c>
       <c r="I49" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Build once as shared infrastructure — every social feature below (community, success stories, etc.) sits on top of this.</v>
       </c>
     </row>
     <row r="50">
@@ -1955,28 +1958,25 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C50" t="str">
-        <v>Community map + Quora-style Q&amp;A</v>
+        <v>Community (feed of designs/observations)</v>
       </c>
       <c r="D50" t="str">
         <v>Social</v>
       </c>
       <c r="E50" t="str">
-        <v>List C</v>
+        <v>List B</v>
       </c>
       <c r="F50" t="str">
         <v>mobile</v>
       </c>
       <c r="G50" t="str">
-        <v>Should</v>
+        <v>Must</v>
       </c>
       <c r="H50" t="str">
         <v>Weeks 13-19</v>
       </c>
       <c r="I50" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J50" t="str">
-        <v>Q&amp;A layer can start simple — threaded comments on map pins.</v>
       </c>
     </row>
     <row r="51">
@@ -1987,13 +1987,13 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C51" t="str">
-        <v>Biodiversity observation tool</v>
+        <v>Community map + Quora-style Q&amp;A</v>
       </c>
       <c r="D51" t="str">
-        <v>Real-world data</v>
+        <v>Social</v>
       </c>
       <c r="E51" t="str">
-        <v>List B</v>
+        <v>List C</v>
       </c>
       <c r="F51" t="str">
         <v>mobile</v>
@@ -2008,7 +2008,7 @@
         <v>Not started</v>
       </c>
       <c r="J51" t="str">
-        <v>Reuses the location_logging pin system from Phase B.</v>
+        <v>Q&amp;A layer can start simple — threaded comments on map pins.</v>
       </c>
     </row>
     <row r="52">
@@ -2019,10 +2019,10 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C52" t="str">
-        <v>Success Stories</v>
+        <v>Biodiversity observation tool</v>
       </c>
       <c r="D52" t="str">
-        <v>Social</v>
+        <v>Real-world data</v>
       </c>
       <c r="E52" t="str">
         <v>List B</v>
@@ -2038,6 +2038,9 @@
       </c>
       <c r="I52" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Reuses the location_logging pin system from Phase B.</v>
       </c>
     </row>
     <row r="53">
@@ -2048,13 +2051,13 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C53" t="str">
-        <v>Decide the social/engagement layer's style (Twitter-like vs Instagram-like vs other)</v>
+        <v>Success Stories</v>
       </c>
       <c r="D53" t="str">
         <v>Social</v>
       </c>
       <c r="E53" t="str">
-        <v>Codebase audit — Section F</v>
+        <v>List B</v>
       </c>
       <c r="F53" t="str">
         <v>mobile</v>
@@ -2067,9 +2070,6 @@
       </c>
       <c r="I53" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J53" t="str">
-        <v>Open question from your own notes — decide before building out social_engine/community_feed in detail, since it shapes the UI pattern (feed vs. grid, text-first vs. photo-first).</v>
       </c>
     </row>
     <row r="54">
@@ -2080,19 +2080,19 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C54" t="str">
-        <v>Perma app map (gamified exploration, like Yusuf's map game)</v>
+        <v>Decide the social/engagement layer's style (Twitter-like vs Instagram-like vs other)</v>
       </c>
       <c r="D54" t="str">
         <v>Social</v>
       </c>
       <c r="E54" t="str">
-        <v>List C</v>
+        <v>Codebase audit — Section F</v>
       </c>
       <c r="F54" t="str">
         <v>mobile</v>
       </c>
       <c r="G54" t="str">
-        <v>Could</v>
+        <v>Should</v>
       </c>
       <c r="H54" t="str">
         <v>Weeks 13-19</v>
@@ -2101,7 +2101,7 @@
         <v>Not started</v>
       </c>
       <c r="J54" t="str">
-        <v>Builds on community_map — sequence after the base map has real content.</v>
+        <v>Open question from your own notes — decide before building out social_engine/community_feed in detail, since it shapes the UI pattern (feed vs. grid, text-first vs. photo-first).</v>
       </c>
     </row>
     <row r="55">
@@ -2112,13 +2112,13 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C55" t="str">
-        <v>Mushroom map</v>
+        <v>Perma app map (gamified exploration, like Yusuf's map game)</v>
       </c>
       <c r="D55" t="str">
-        <v>Real-world data</v>
+        <v>Social</v>
       </c>
       <c r="E55" t="str">
-        <v>List B</v>
+        <v>List C</v>
       </c>
       <c r="F55" t="str">
         <v>mobile</v>
@@ -2133,7 +2133,7 @@
         <v>Not started</v>
       </c>
       <c r="J55" t="str">
-        <v>A filtered view of the same pin system, not a separate build.</v>
+        <v>Builds on community_map — sequence after the base map has real content.</v>
       </c>
     </row>
     <row r="56">
@@ -2144,10 +2144,10 @@
         <v>Mobile Social Layer</v>
       </c>
       <c r="C56" t="str">
-        <v>Messaging app (DMs)</v>
+        <v>Mushroom map</v>
       </c>
       <c r="D56" t="str">
-        <v>Social</v>
+        <v>Real-world data</v>
       </c>
       <c r="E56" t="str">
         <v>List B</v>
@@ -2165,39 +2165,39 @@
         <v>Not started</v>
       </c>
       <c r="J56" t="str">
-        <v>Real engineering + moderation surface — confirm it's worth it before/instead of just comments+DM-via-email.</v>
+        <v>A filtered view of the same pin system, not a separate build.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="B57" t="str">
-        <v>Reference &amp; Content Layer</v>
+        <v>Mobile Social Layer</v>
       </c>
       <c r="C57" t="str">
-        <v>Usability &amp; onboarding (beginner mode)</v>
+        <v>Messaging app (DMs)</v>
       </c>
       <c r="D57" t="str">
-        <v>Onboarding</v>
+        <v>Social</v>
       </c>
       <c r="E57" t="str">
-        <v>List A – #8</v>
+        <v>List B</v>
       </c>
       <c r="F57" t="str">
-        <v>both</v>
+        <v>mobile</v>
       </c>
       <c r="G57" t="str">
-        <v>Must</v>
+        <v>Could</v>
       </c>
       <c r="H57" t="str">
-        <v>Weeks 20-27</v>
+        <v>Weeks 13-19</v>
       </c>
       <c r="I57" t="str">
         <v>Not started</v>
       </c>
       <c r="J57" t="str">
-        <v>Don't skip this — it's explicitly why MyPermagarden beats Swales today on ease of entry.</v>
+        <v>Real engineering + moderation surface — confirm it's worth it before/instead of just comments+DM-via-email.</v>
       </c>
     </row>
     <row r="58">
@@ -2208,25 +2208,28 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C58" t="str">
-        <v>Wiki</v>
+        <v>Usability &amp; onboarding (beginner mode)</v>
       </c>
       <c r="D58" t="str">
-        <v>Learning</v>
+        <v>Onboarding</v>
       </c>
       <c r="E58" t="str">
-        <v>List B</v>
+        <v>List A – #8</v>
       </c>
       <c r="F58" t="str">
         <v>both</v>
       </c>
       <c r="G58" t="str">
-        <v>Should</v>
+        <v>Must</v>
       </c>
       <c r="H58" t="str">
         <v>Weeks 20-27</v>
       </c>
       <c r="I58" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Don't skip this — it's explicitly why MyPermagarden beats Swales today on ease of entry.</v>
       </c>
     </row>
     <row r="59">
@@ -2237,10 +2240,10 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C59" t="str">
-        <v>Trees reference pages</v>
+        <v>Wiki</v>
       </c>
       <c r="D59" t="str">
-        <v>Core data</v>
+        <v>Learning</v>
       </c>
       <c r="E59" t="str">
         <v>List B</v>
@@ -2256,9 +2259,6 @@
       </c>
       <c r="I59" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J59" t="str">
-        <v>Pulls from the same plant_database schema — content expansion, not new architecture.</v>
       </c>
     </row>
     <row r="60">
@@ -2269,7 +2269,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C60" t="str">
-        <v>Plants reference pages</v>
+        <v>Trees reference pages</v>
       </c>
       <c r="D60" t="str">
         <v>Core data</v>
@@ -2290,7 +2290,7 @@
         <v>Not started</v>
       </c>
       <c r="J60" t="str">
-        <v>Same as above.</v>
+        <v>Pulls from the same plant_database schema — content expansion, not new architecture.</v>
       </c>
     </row>
     <row r="61">
@@ -2301,10 +2301,10 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C61" t="str">
-        <v>Energy Calculators</v>
+        <v>Plants reference pages</v>
       </c>
       <c r="D61" t="str">
-        <v>Calculators</v>
+        <v>Core data</v>
       </c>
       <c r="E61" t="str">
         <v>List B</v>
@@ -2322,7 +2322,7 @@
         <v>Not started</v>
       </c>
       <c r="J61" t="str">
-        <v>Contained scope, good quick win once content team has capacity.</v>
+        <v>Same as above.</v>
       </c>
     </row>
     <row r="62">
@@ -2333,7 +2333,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C62" t="str">
-        <v>Field Calculators</v>
+        <v>Energy Calculators</v>
       </c>
       <c r="D62" t="str">
         <v>Calculators</v>
@@ -2352,6 +2352,9 @@
       </c>
       <c r="I62" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Contained scope, good quick win once content team has capacity.</v>
       </c>
     </row>
     <row r="63">
@@ -2362,13 +2365,13 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C63" t="str">
-        <v>Design library / public gallery</v>
+        <v>Field Calculators</v>
       </c>
       <c r="D63" t="str">
-        <v>Social</v>
+        <v>Calculators</v>
       </c>
       <c r="E63" t="str">
-        <v>List A – Phase 5 / List B – Design</v>
+        <v>List B</v>
       </c>
       <c r="F63" t="str">
         <v>both</v>
@@ -2381,9 +2384,6 @@
       </c>
       <c r="I63" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J63" t="str">
-        <v>Needs real user designs to populate — sequence after Phase B/C produce some.</v>
       </c>
     </row>
     <row r="64">
@@ -2394,16 +2394,16 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C64" t="str">
-        <v>Templates (UK garden, homestead, agroforestry)</v>
+        <v>Design library / public gallery</v>
       </c>
       <c r="D64" t="str">
-        <v>Onboarding</v>
+        <v>Social</v>
       </c>
       <c r="E64" t="str">
-        <v>List A – Phase 5</v>
+        <v>List A – Phase 5 / List B – Design</v>
       </c>
       <c r="F64" t="str">
-        <v>web</v>
+        <v>both</v>
       </c>
       <c r="G64" t="str">
         <v>Should</v>
@@ -2413,6 +2413,9 @@
       </c>
       <c r="I64" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Needs real user designs to populate — sequence after Phase B/C produce some.</v>
       </c>
     </row>
     <row r="65">
@@ -2423,28 +2426,25 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C65" t="str">
-        <v>Flowers reference pages</v>
+        <v>Templates (UK garden, homestead, agroforestry)</v>
       </c>
       <c r="D65" t="str">
-        <v>Core data</v>
+        <v>Onboarding</v>
       </c>
       <c r="E65" t="str">
-        <v>List B</v>
+        <v>List A – Phase 5</v>
       </c>
       <c r="F65" t="str">
-        <v>both</v>
+        <v>web</v>
       </c>
       <c r="G65" t="str">
-        <v>Could</v>
+        <v>Should</v>
       </c>
       <c r="H65" t="str">
         <v>Weeks 20-27</v>
       </c>
       <c r="I65" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J65" t="str">
-        <v>Same schema, lower priority content set.</v>
       </c>
     </row>
     <row r="66">
@@ -2455,7 +2455,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C66" t="str">
-        <v>Animals reference pages</v>
+        <v>Flowers reference pages</v>
       </c>
       <c r="D66" t="str">
         <v>Core data</v>
@@ -2476,7 +2476,7 @@
         <v>Not started</v>
       </c>
       <c r="J66" t="str">
-        <v>Same schema, extends the animal_system category already in the seed data.</v>
+        <v>Same schema, lower priority content set.</v>
       </c>
     </row>
     <row r="67">
@@ -2487,7 +2487,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C67" t="str">
-        <v>Mushrooms reference pages</v>
+        <v>Animals reference pages</v>
       </c>
       <c r="D67" t="str">
         <v>Core data</v>
@@ -2508,7 +2508,7 @@
         <v>Not started</v>
       </c>
       <c r="J67" t="str">
-        <v>Same schema.</v>
+        <v>Same schema, extends the animal_system category already in the seed data.</v>
       </c>
     </row>
     <row r="68">
@@ -2519,7 +2519,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C68" t="str">
-        <v>Materials reference/catalog</v>
+        <v>Mushrooms reference pages</v>
       </c>
       <c r="D68" t="str">
         <v>Core data</v>
@@ -2538,6 +2538,9 @@
       </c>
       <c r="I68" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J68" t="str">
+        <v>Same schema.</v>
       </c>
     </row>
     <row r="69">
@@ -2548,10 +2551,10 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C69" t="str">
-        <v>Books and magazines library</v>
+        <v>Materials reference/catalog</v>
       </c>
       <c r="D69" t="str">
-        <v>Learning</v>
+        <v>Core data</v>
       </c>
       <c r="E69" t="str">
         <v>List B</v>
@@ -2577,7 +2580,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C70" t="str">
-        <v>Resources library</v>
+        <v>Books and magazines library</v>
       </c>
       <c r="D70" t="str">
         <v>Learning</v>
@@ -2596,9 +2599,6 @@
       </c>
       <c r="I70" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J70" t="str">
-        <v>Overlaps books_magazines — consider one unified library section.</v>
       </c>
     </row>
     <row r="71">
@@ -2609,7 +2609,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C71" t="str">
-        <v>Ideas (inspiration gallery)</v>
+        <v>Resources library</v>
       </c>
       <c r="D71" t="str">
         <v>Learning</v>
@@ -2630,7 +2630,7 @@
         <v>Not started</v>
       </c>
       <c r="J71" t="str">
-        <v>Overlaps design_gallery below — merge if possible.</v>
+        <v>Overlaps books_magazines — consider one unified library section.</v>
       </c>
     </row>
     <row r="72">
@@ -2641,7 +2641,7 @@
         <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C72" t="str">
-        <v>"Permaculture" content hub / landing page</v>
+        <v>Ideas (inspiration gallery)</v>
       </c>
       <c r="D72" t="str">
         <v>Learning</v>
@@ -2661,19 +2661,22 @@
       <c r="I72" t="str">
         <v>Not started</v>
       </c>
+      <c r="J72" t="str">
+        <v>Overlaps design_gallery below — merge if possible.</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>E</v>
+        <v>D</v>
       </c>
       <c r="B73" t="str">
-        <v>Education &amp; Gamification</v>
+        <v>Reference &amp; Content Layer</v>
       </c>
       <c r="C73" t="str">
-        <v>Yield planner</v>
+        <v>"Permaculture" content hub / landing page</v>
       </c>
       <c r="D73" t="str">
-        <v>Time/succession</v>
+        <v>Learning</v>
       </c>
       <c r="E73" t="str">
         <v>List B</v>
@@ -2682,10 +2685,10 @@
         <v>both</v>
       </c>
       <c r="G73" t="str">
-        <v>Should</v>
+        <v>Could</v>
       </c>
       <c r="H73" t="str">
-        <v>Weeks 28-34</v>
+        <v>Weeks 20-27</v>
       </c>
       <c r="I73" t="str">
         <v>Not started</v>
@@ -2699,7 +2702,7 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C74" t="str">
-        <v>Planner / Tips / To-do list</v>
+        <v>Yield planner</v>
       </c>
       <c r="D74" t="str">
         <v>Time/succession</v>
@@ -2708,7 +2711,7 @@
         <v>List B</v>
       </c>
       <c r="F74" t="str">
-        <v>mobile</v>
+        <v>both</v>
       </c>
       <c r="G74" t="str">
         <v>Should</v>
@@ -2728,16 +2731,16 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C75" t="str">
-        <v>Quiz / SwalesQuiz</v>
+        <v>Planner / Tips / To-do list</v>
       </c>
       <c r="D75" t="str">
-        <v>Learning</v>
+        <v>Time/succession</v>
       </c>
       <c r="E75" t="str">
-        <v>List B / List C</v>
+        <v>List B</v>
       </c>
       <c r="F75" t="str">
-        <v>both</v>
+        <v>mobile</v>
       </c>
       <c r="G75" t="str">
         <v>Should</v>
@@ -2747,9 +2750,6 @@
       </c>
       <c r="I75" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J75" t="str">
-        <v>Merge Quiz + SwalesQuiz + 'Test your knowledge' into one feature.</v>
       </c>
     </row>
     <row r="76">
@@ -2760,13 +2760,13 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C76" t="str">
-        <v>Test your knowledge</v>
+        <v>Quiz / SwalesQuiz</v>
       </c>
       <c r="D76" t="str">
         <v>Learning</v>
       </c>
       <c r="E76" t="str">
-        <v>List B</v>
+        <v>List B / List C</v>
       </c>
       <c r="F76" t="str">
         <v>both</v>
@@ -2781,7 +2781,7 @@
         <v>Not started</v>
       </c>
       <c r="J76" t="str">
-        <v>Duplicate of quiz — don't build twice.</v>
+        <v>Merge Quiz + SwalesQuiz + 'Test your knowledge' into one feature.</v>
       </c>
     </row>
     <row r="77">
@@ -2792,10 +2792,10 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C77" t="str">
-        <v>Events calendar</v>
+        <v>Test your knowledge</v>
       </c>
       <c r="D77" t="str">
-        <v>Social</v>
+        <v>Learning</v>
       </c>
       <c r="E77" t="str">
         <v>List B</v>
@@ -2804,13 +2804,16 @@
         <v>both</v>
       </c>
       <c r="G77" t="str">
-        <v>Could</v>
+        <v>Should</v>
       </c>
       <c r="H77" t="str">
         <v>Weeks 28-34</v>
       </c>
       <c r="I77" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J77" t="str">
+        <v>Duplicate of quiz — don't build twice.</v>
       </c>
     </row>
     <row r="78">
@@ -2821,10 +2824,10 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C78" t="str">
-        <v>Competitions / challenges / tests</v>
+        <v>Events calendar</v>
       </c>
       <c r="D78" t="str">
-        <v>Gamification</v>
+        <v>Social</v>
       </c>
       <c r="E78" t="str">
         <v>List B</v>
@@ -2840,9 +2843,6 @@
       </c>
       <c r="I78" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J78" t="str">
-        <v>Needs an active user base to have anyone to compete against — correctly gated here, not earlier.</v>
       </c>
     </row>
     <row r="79">
@@ -2853,7 +2853,7 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C79" t="str">
-        <v>Coins / earnings or similar</v>
+        <v>Competitions / challenges / tests</v>
       </c>
       <c r="D79" t="str">
         <v>Gamification</v>
@@ -2874,7 +2874,7 @@
         <v>Not started</v>
       </c>
       <c r="J79" t="str">
-        <v>Merge with 'Rewards using the app' — same mechanic.</v>
+        <v>Needs an active user base to have anyone to compete against — correctly gated here, not earlier.</v>
       </c>
     </row>
     <row r="80">
@@ -2885,7 +2885,7 @@
         <v>Education &amp; Gamification</v>
       </c>
       <c r="C80" t="str">
-        <v>Rewards using the app</v>
+        <v>Coins / earnings or similar</v>
       </c>
       <c r="D80" t="str">
         <v>Gamification</v>
@@ -2906,39 +2906,39 @@
         <v>Not started</v>
       </c>
       <c r="J80" t="str">
-        <v>Duplicate of coins_rewards.</v>
+        <v>Merge with 'Rewards using the app' — same mechanic.</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>F</v>
+        <v>E</v>
       </c>
       <c r="B81" t="str">
-        <v>Platform &amp; Business Layer</v>
+        <v>Education &amp; Gamification</v>
       </c>
       <c r="C81" t="str">
-        <v>3D model / visualization</v>
+        <v>Rewards using the app</v>
       </c>
       <c r="D81" t="str">
-        <v>Canvas</v>
+        <v>Gamification</v>
       </c>
       <c r="E81" t="str">
-        <v>List A – #12</v>
+        <v>List B</v>
       </c>
       <c r="F81" t="str">
-        <v>web</v>
+        <v>both</v>
       </c>
       <c r="G81" t="str">
-        <v>Later</v>
+        <v>Could</v>
       </c>
       <c r="H81" t="str">
-        <v>Month 9+</v>
+        <v>Weeks 28-34</v>
       </c>
       <c r="I81" t="str">
         <v>Not started</v>
       </c>
       <c r="J81" t="str">
-        <v>Most expensive line item relative to payoff. Recommend skipping until 2D + AI + data clearly beat AgroForest Designer on their own turf.</v>
+        <v>Duplicate of coins_rewards.</v>
       </c>
     </row>
     <row r="82">
@@ -2949,16 +2949,16 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C82" t="str">
-        <v>Swales marketplace</v>
+        <v>3D model / visualization</v>
       </c>
       <c r="D82" t="str">
-        <v>Marketplace/biz</v>
+        <v>Canvas</v>
       </c>
       <c r="E82" t="str">
-        <v>List C</v>
+        <v>List A – #12</v>
       </c>
       <c r="F82" t="str">
-        <v>both</v>
+        <v>web</v>
       </c>
       <c r="G82" t="str">
         <v>Later</v>
@@ -2970,7 +2970,7 @@
         <v>Not started</v>
       </c>
       <c r="J82" t="str">
-        <v>Needs finished designs worth trading — gate on Phase B/C/D producing real content.</v>
+        <v>Most expensive line item relative to payoff. Recommend skipping until 2D + AI + data clearly beat AgroForest Designer on their own turf.</v>
       </c>
     </row>
     <row r="83">
@@ -2981,13 +2981,13 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C83" t="str">
-        <v>Services directory (consultants/designers)</v>
+        <v>Swales marketplace</v>
       </c>
       <c r="D83" t="str">
         <v>Marketplace/biz</v>
       </c>
       <c r="E83" t="str">
-        <v>List B</v>
+        <v>List C</v>
       </c>
       <c r="F83" t="str">
         <v>both</v>
@@ -3000,6 +3000,9 @@
       </c>
       <c r="I83" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J83" t="str">
+        <v>Needs finished designs worth trading — gate on Phase B/C/D producing real content.</v>
       </c>
     </row>
     <row r="84">
@@ -3010,7 +3013,7 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C84" t="str">
-        <v>Quotes (supplier/contractor quote requests)</v>
+        <v>Services directory (consultants/designers)</v>
       </c>
       <c r="D84" t="str">
         <v>Marketplace/biz</v>
@@ -3029,9 +3032,6 @@
       </c>
       <c r="I84" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J84" t="str">
-        <v>Pairs naturally with services + cost_estimation.</v>
       </c>
     </row>
     <row r="85">
@@ -3042,13 +3042,13 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C85" t="str">
-        <v>Hardware (physical products)</v>
+        <v>Quotes (supplier/contractor quote requests)</v>
       </c>
       <c r="D85" t="str">
         <v>Marketplace/biz</v>
       </c>
       <c r="E85" t="str">
-        <v>List C</v>
+        <v>List B</v>
       </c>
       <c r="F85" t="str">
         <v>both</v>
@@ -3063,7 +3063,7 @@
         <v>Not started</v>
       </c>
       <c r="J85" t="str">
-        <v>This is close to a separate business — treat as its own go/no-go decision, not a feature ticket.</v>
+        <v>Pairs naturally with services + cost_estimation.</v>
       </c>
     </row>
     <row r="86">
@@ -3074,13 +3074,13 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C86" t="str">
-        <v>School</v>
+        <v>Hardware (physical products)</v>
       </c>
       <c r="D86" t="str">
-        <v>Learning</v>
+        <v>Marketplace/biz</v>
       </c>
       <c r="E86" t="str">
-        <v>List B</v>
+        <v>List C</v>
       </c>
       <c r="F86" t="str">
         <v>both</v>
@@ -3095,7 +3095,7 @@
         <v>Not started</v>
       </c>
       <c r="J86" t="str">
-        <v>Merge with skool_mentors + mind_valley — pick one education-platform model, don't build three.</v>
+        <v>This is close to a separate business — treat as its own go/no-go decision, not a feature ticket.</v>
       </c>
     </row>
     <row r="87">
@@ -3106,7 +3106,7 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C87" t="str">
-        <v>Skool of mentors idea</v>
+        <v>School</v>
       </c>
       <c r="D87" t="str">
         <v>Learning</v>
@@ -3127,7 +3127,7 @@
         <v>Not started</v>
       </c>
       <c r="J87" t="str">
-        <v>Duplicate bucket — see school.</v>
+        <v>Merge with skool_mentors + mind_valley — pick one education-platform model, don't build three.</v>
       </c>
     </row>
     <row r="88">
@@ -3138,7 +3138,7 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C88" t="str">
-        <v>Mind Valley-style permaculture course platform</v>
+        <v>Skool of mentors idea</v>
       </c>
       <c r="D88" t="str">
         <v>Learning</v>
@@ -3170,10 +3170,10 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C89" t="str">
-        <v>Swales Media (video/photo content hub)</v>
+        <v>Mind Valley-style permaculture course platform</v>
       </c>
       <c r="D89" t="str">
-        <v>Content</v>
+        <v>Learning</v>
       </c>
       <c r="E89" t="str">
         <v>List B</v>
@@ -3191,7 +3191,7 @@
         <v>Not started</v>
       </c>
       <c r="J89" t="str">
-        <v>Merge with journal_magazine — one content hub, not two.</v>
+        <v>Duplicate bucket — see school.</v>
       </c>
     </row>
     <row r="90">
@@ -3202,7 +3202,7 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C90" t="str">
-        <v>Journal or news magazine</v>
+        <v>Swales Media (video/photo content hub)</v>
       </c>
       <c r="D90" t="str">
         <v>Content</v>
@@ -3223,7 +3223,7 @@
         <v>Not started</v>
       </c>
       <c r="J90" t="str">
-        <v>Duplicate bucket — see swales_media.</v>
+        <v>Merge with journal_magazine — one content hub, not two.</v>
       </c>
     </row>
     <row r="91">
@@ -3234,7 +3234,7 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C91" t="str">
-        <v>Permaculture Photo book</v>
+        <v>Journal or news magazine</v>
       </c>
       <c r="D91" t="str">
         <v>Content</v>
@@ -3253,6 +3253,9 @@
       </c>
       <c r="I91" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J91" t="str">
+        <v>Duplicate bucket — see swales_media.</v>
       </c>
     </row>
     <row r="92">
@@ -3263,13 +3266,13 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C92" t="str">
-        <v>A KPI-led movement (impact metrics framework)</v>
+        <v>Permaculture Photo book</v>
       </c>
       <c r="D92" t="str">
-        <v>Marketplace/biz</v>
+        <v>Content</v>
       </c>
       <c r="E92" t="str">
-        <v>List C</v>
+        <v>List B</v>
       </c>
       <c r="F92" t="str">
         <v>both</v>
@@ -3282,9 +3285,6 @@
       </c>
       <c r="I92" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J92" t="str">
-        <v>More a marketing/positioning initiative than a build item.</v>
       </c>
     </row>
     <row r="93">
@@ -3295,16 +3295,16 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C93" t="str">
-        <v>Integrations (GIS, farm tools)</v>
+        <v>A KPI-led movement (impact metrics framework)</v>
       </c>
       <c r="D93" t="str">
-        <v>Real-world data</v>
+        <v>Marketplace/biz</v>
       </c>
       <c r="E93" t="str">
-        <v>List A – Phase 5</v>
+        <v>List C</v>
       </c>
       <c r="F93" t="str">
-        <v>backend</v>
+        <v>both</v>
       </c>
       <c r="G93" t="str">
         <v>Later</v>
@@ -3314,6 +3314,9 @@
       </c>
       <c r="I93" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J93" t="str">
+        <v>More a marketing/positioning initiative than a build item.</v>
       </c>
     </row>
     <row r="94">
@@ -3324,13 +3327,13 @@
         <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C94" t="str">
-        <v>Technical considerations in the future (infra/scaling)</v>
+        <v>Integrations (GIS, farm tools)</v>
       </c>
       <c r="D94" t="str">
-        <v>Infrastructure</v>
+        <v>Real-world data</v>
       </c>
       <c r="E94" t="str">
-        <v>List C</v>
+        <v>List A – Phase 5</v>
       </c>
       <c r="F94" t="str">
         <v>backend</v>
@@ -3344,40 +3347,37 @@
       <c r="I94" t="str">
         <v>Not started</v>
       </c>
-      <c r="J94" t="str">
-        <v>Revisit once there's real load to scale for.</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="B95" t="str">
-        <v>Web Pro Track (parallel)</v>
+        <v>Platform &amp; Business Layer</v>
       </c>
       <c r="C95" t="str">
-        <v>AI design assistant ("Swales AI") — swale placement, orchard siting, windbreak recs</v>
+        <v>Technical considerations in the future (infra/scaling)</v>
       </c>
       <c r="D95" t="str">
-        <v>AI assist</v>
+        <v>Infrastructure</v>
       </c>
       <c r="E95" t="str">
-        <v>List A – Phase 2 / List C – Swales AI / List B – Design with AI help</v>
+        <v>List C</v>
       </c>
       <c r="F95" t="str">
-        <v>web</v>
+        <v>backend</v>
       </c>
       <c r="G95" t="str">
-        <v>Must</v>
+        <v>Later</v>
       </c>
       <c r="H95" t="str">
-        <v>Runs alongside B–E</v>
+        <v>Month 9+</v>
       </c>
       <c r="I95" t="str">
         <v>Not started</v>
       </c>
       <c r="J95" t="str">
-        <v>Already in background dev. Treat Swales AI, Decision Intelligent Layer, and Design-with-AI-help as ONE product surface, not three.</v>
+        <v>Revisit once there's real load to scale for.</v>
       </c>
     </row>
     <row r="96">
@@ -3388,13 +3388,13 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C96" t="str">
-        <v>Guild builder (auto-suggest combos, conflict warnings)</v>
+        <v>AI design assistant ("Swales AI") — swale placement, orchard siting, windbreak recs</v>
       </c>
       <c r="D96" t="str">
         <v>AI assist</v>
       </c>
       <c r="E96" t="str">
-        <v>List A – Phase 2</v>
+        <v>List A – Phase 2 / List C – Swales AI / List B – Design with AI help</v>
       </c>
       <c r="F96" t="str">
         <v>web</v>
@@ -3409,7 +3409,7 @@
         <v>Not started</v>
       </c>
       <c r="J96" t="str">
-        <v>Directly uses the good_companions/avoid_near fields already in the delivered schema.</v>
+        <v>Already in background dev. Treat Swales AI, Decision Intelligent Layer, and Design-with-AI-help as ONE product surface, not three.</v>
       </c>
     </row>
     <row r="97">
@@ -3420,13 +3420,13 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C97" t="str">
-        <v>Reports (site analysis, water flow, design rationale)</v>
+        <v>Guild builder (auto-suggest combos, conflict warnings)</v>
       </c>
       <c r="D97" t="str">
-        <v>Workflow</v>
+        <v>AI assist</v>
       </c>
       <c r="E97" t="str">
-        <v>List A – Phase 3 / List C</v>
+        <v>List A – Phase 2</v>
       </c>
       <c r="F97" t="str">
         <v>web</v>
@@ -3441,7 +3441,7 @@
         <v>Not started</v>
       </c>
       <c r="J97" t="str">
-        <v>This is the monetization unlock — what consultants pay for.</v>
+        <v>Directly uses the good_companions/avoid_near fields already in the delivered schema.</v>
       </c>
     </row>
     <row r="98">
@@ -3452,19 +3452,19 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C98" t="str">
-        <v>Decision intelligent layer</v>
+        <v>Reports (site analysis, water flow, design rationale)</v>
       </c>
       <c r="D98" t="str">
-        <v>AI assist</v>
+        <v>Workflow</v>
       </c>
       <c r="E98" t="str">
-        <v>List C</v>
+        <v>List A – Phase 3 / List C</v>
       </c>
       <c r="F98" t="str">
         <v>web</v>
       </c>
       <c r="G98" t="str">
-        <v>Should</v>
+        <v>Must</v>
       </c>
       <c r="H98" t="str">
         <v>Runs alongside B–E</v>
@@ -3473,7 +3473,7 @@
         <v>Not started</v>
       </c>
       <c r="J98" t="str">
-        <v>Merge into ai_advisor — same underlying engine, don't build twice. Also overlaps cross_layer_advisory below — one engine, not three.</v>
+        <v>This is the monetization unlock — what consultants pay for.</v>
       </c>
     </row>
     <row r="99">
@@ -3484,13 +3484,13 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C99" t="str">
-        <v>Zones &amp; sectors auto-generation (Zone 1-5, sun/wind/water)</v>
+        <v>Decision intelligent layer</v>
       </c>
       <c r="D99" t="str">
-        <v>Canvas</v>
+        <v>AI assist</v>
       </c>
       <c r="E99" t="str">
-        <v>List A – Phase 2</v>
+        <v>List C</v>
       </c>
       <c r="F99" t="str">
         <v>web</v>
@@ -3503,6 +3503,9 @@
       </c>
       <c r="I99" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J99" t="str">
+        <v>Merge into ai_advisor — same underlying engine, don't build twice. Also overlaps cross_layer_advisory below — one engine, not three.</v>
       </c>
     </row>
     <row r="100">
@@ -3513,13 +3516,13 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C100" t="str">
-        <v>Cost + materials estimation</v>
+        <v>Zones &amp; sectors auto-generation (Zone 1-5, sun/wind/water)</v>
       </c>
       <c r="D100" t="str">
-        <v>Workflow</v>
+        <v>Canvas</v>
       </c>
       <c r="E100" t="str">
-        <v>List A – Phase 3</v>
+        <v>List A – Phase 2</v>
       </c>
       <c r="F100" t="str">
         <v>web</v>
@@ -3542,7 +3545,7 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C101" t="str">
-        <v>Client sharing (view-only links, commenting)</v>
+        <v>Cost + materials estimation</v>
       </c>
       <c r="D101" t="str">
         <v>Workflow</v>
@@ -3571,13 +3574,13 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C102" t="str">
-        <v>Bankability for systems (financial/ROI viability)</v>
+        <v>Client sharing (view-only links, commenting)</v>
       </c>
       <c r="D102" t="str">
         <v>Workflow</v>
       </c>
       <c r="E102" t="str">
-        <v>List A – #13</v>
+        <v>List A – Phase 3</v>
       </c>
       <c r="F102" t="str">
         <v>web</v>
@@ -3590,9 +3593,6 @@
       </c>
       <c r="I102" t="str">
         <v>Not started</v>
-      </c>
-      <c r="J102" t="str">
-        <v>Real differentiator — no competitor in the teardown has this. Worth protecting time for.</v>
       </c>
     </row>
     <row r="103">
@@ -3603,19 +3603,19 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C103" t="str">
-        <v>Growth simulation (trees over 5-10 years)</v>
+        <v>Bankability for systems (financial/ROI viability)</v>
       </c>
       <c r="D103" t="str">
-        <v>Time/succession</v>
+        <v>Workflow</v>
       </c>
       <c r="E103" t="str">
-        <v>List A – Phase 4</v>
+        <v>List A – #13</v>
       </c>
       <c r="F103" t="str">
         <v>web</v>
       </c>
       <c r="G103" t="str">
-        <v>Could</v>
+        <v>Should</v>
       </c>
       <c r="H103" t="str">
         <v>Runs alongside B–E</v>
@@ -3624,7 +3624,7 @@
         <v>Not started</v>
       </c>
       <c r="J103" t="str">
-        <v>Slides to late W / early F if capacity is tight — real engineering effort.</v>
+        <v>Real differentiator — no competitor in the teardown has this. Worth protecting time for.</v>
       </c>
     </row>
     <row r="104">
@@ -3635,7 +3635,7 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C104" t="str">
-        <v>Water behavior modeling (before/after swales)</v>
+        <v>Growth simulation (trees over 5-10 years)</v>
       </c>
       <c r="D104" t="str">
         <v>Time/succession</v>
@@ -3656,7 +3656,7 @@
         <v>Not started</v>
       </c>
       <c r="J104" t="str">
-        <v>Same caveat as growth_sim.</v>
+        <v>Slides to late W / early F if capacity is tight — real engineering effort.</v>
       </c>
     </row>
     <row r="105">
@@ -3667,7 +3667,7 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C105" t="str">
-        <v>Yield projections</v>
+        <v>Water behavior modeling (before/after swales)</v>
       </c>
       <c r="D105" t="str">
         <v>Time/succession</v>
@@ -3686,6 +3686,9 @@
       </c>
       <c r="I105" t="str">
         <v>Not started</v>
+      </c>
+      <c r="J105" t="str">
+        <v>Same caveat as growth_sim.</v>
       </c>
     </row>
     <row r="106">
@@ -3696,13 +3699,13 @@
         <v>Web Pro Track (parallel)</v>
       </c>
       <c r="C106" t="str">
-        <v>Succession planning</v>
+        <v>Yield projections</v>
       </c>
       <c r="D106" t="str">
         <v>Time/succession</v>
       </c>
       <c r="E106" t="str">
-        <v>List A – #5 / Phase 4</v>
+        <v>List A – Phase 4</v>
       </c>
       <c r="F106" t="str">
         <v>web</v>
@@ -3719,33 +3722,62 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
+        <v>W</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Web Pro Track (parallel)</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Succession planning</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Time/succession</v>
+      </c>
+      <c r="E107" t="str">
+        <v>List A – #5 / Phase 4</v>
+      </c>
+      <c r="F107" t="str">
+        <v>web</v>
+      </c>
+      <c r="G107" t="str">
+        <v>Could</v>
+      </c>
+      <c r="H107" t="str">
+        <v>Runs alongside B–E</v>
+      </c>
+      <c r="I107" t="str">
+        <v>Not started</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
         <v>P</v>
       </c>
-      <c r="B107" t="str">
+      <c r="B108" t="str">
         <v>Parked / Needs Clarification</v>
       </c>
-      <c r="C107" t="str">
+      <c r="C108" t="str">
         <v>"Eco system Features" (as named in your Notion list)</v>
       </c>
-      <c r="D107" t="str">
+      <c r="D108" t="str">
         <v>Unclear</v>
       </c>
-      <c r="E107" t="str">
+      <c r="E108" t="str">
         <v>List C</v>
       </c>
-      <c r="F107" t="str">
+      <c r="F108" t="str">
         <v>—</v>
       </c>
-      <c r="G107" t="str">
+      <c r="G108" t="str">
         <v>—</v>
       </c>
-      <c r="H107" t="str">
+      <c r="H108" t="str">
         <v>—</v>
       </c>
-      <c r="I107" t="str">
-        <v>Not started</v>
-      </c>
-      <c r="J107" t="str">
+      <c r="I108" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="J108" t="str">
         <v>Title alone doesn't tell me what's inside this page — looked private/inaccessible to me. Overlaps growth_sim/water_modeling/yield_projection unless it means something else — flag for you to clarify or fold in.</v>
       </c>
     </row>
@@ -3853,10 +3885,10 @@
         <v>Web + backend</v>
       </c>
       <c r="F3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H3">
         <v>2</v>

</xml_diff>

<commit_message>
Mark AuthContext (web) as Done; note shared_backend is now unblocked
swales-services now has a working AuthContext (built in the sibling
swales-services commit this session). Both of shared_backend's predecessors
- the auth-token decision and AuthContext - are Done as of 2026-08-24, so
it's ready to start whenever prioritized. Documented the SSR-regression
catch/fix and verification approach in status.md for future reference, and
flagged two non-blocking follow-ups (MobileHeader.jsx wiring decision,
Header.jsx's duplicate auth logic) for whenever there's spare cycles.
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -218,7 +218,7 @@
     <t>Build a real AuthContext for the web app</t>
   </si>
   <si>
-    <t>MobileHeader.jsx references @/context/AuthContext, which doesn't exist yet — import path was fixed but the context itself still needs building. Needed before wiring the account-details modal, and useful groundwork for shared_backend.</t>
+    <t>Done 2026-08-24. swales-designer already had context/AuthContext.tsx; the gap was specifically swales-services. Built swales-services/src/context/AuthContext.jsx matching services' existing conventions (accessToken localStorage key, NEXT_PUBLIC_API_BASE_URL + /api), wired into providers.js and login/page.js. Caught and fixed a real SSR regression before shipping (a copied {!isLoading &amp;&amp; children} render gate was blanking Header/nav out of every static page - wrong for this SEO-dependent site). Verified end-to-end against the live rebuild backend via an invalid-token 401 -&gt; self-clearing logout() path. Header.jsx (the live header) keeps its own separate auth logic - not migrated, out of scope. See status.md for full detail.</t>
   </si>
   <si>
     <t>Decide monetization framework (Free / free-for-contact / Core paid / Post-core)</t>
@@ -257,7 +257,7 @@
     <t>New (mobile ask)</t>
   </si>
   <si>
-    <t>The technical piece that makes 'mobile links with the web version' literally true, not just a slogan. Confirmed: today's mobile experience (MobileHeader.jsx) is responsive web only, not a native app — build this so a future native app can reuse it, but Phase B below is a genuine fresh build either way. Sequence after auth_token_decision/auth_context_build — don't build shared accounts on top of an auth flow that's still an open security question.</t>
+    <t>The technical piece that makes 'mobile links with the web version' literally true, not just a slogan. Confirmed: today's mobile experience (MobileHeader.jsx) is responsive web only, not a native app - build this so a future native app can reuse it, but Phase B below is a genuine fresh build either way. Both predecessors now Done (auth_token_decision, auth_context_build, both 2026-08-24) - this item is unblocked and ready to start.</t>
   </si>
   <si>
     <t>Decide the mobile app tech stack (React Native + Expo proposed)</t>
@@ -1292,7 +1292,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J108"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -1844,7 +1844,7 @@
         <v>51</v>
       </c>
       <c r="I17" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J17" t="s">
         <v>67</v>
@@ -4679,7 +4679,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>

</xml_diff>

<commit_message>
Add future-concerns.md; scope 2FA and disposable-email blocking; clean up stale CLAUDE.md notes
New 4th tracking doc at Omar's request: a living checklist of risks/gaps
intentionally deferred rather than fixed immediately, reviewed before
starting a new phase or a real-users/monetization milestone. Seeded with
everything flagged-but-unfixed from the auth threat sweep.

Two new roadmap items added to Phase A per Omar's request: optional TOTP
2FA (target: before monetization go-live) and blocking disposable/temporary
email domains at registration. Neither built yet.

Also rewrote all three repos' CLAUDE.md files, which had accumulated
several sessions' worth of "corrected" notes on top of corrections -
now a single clean statement instead of a changelog of past mistakes.
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -8,14 +8,14 @@
     <sheet sheetId="2" name="Phase Summary" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase">Backlog!$A$1:$J$97</definedName>
+    <definedName name="_xlnm._FilterDatabase">Backlog!$A$1:$J$21,Backlog!$A$24:$J$99</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="307">
   <si>
     <t>Phase</t>
   </si>
@@ -270,6 +270,27 @@
   </si>
   <si>
     <t>Confirmed by Omar 2026-08-24: React Native + Expo (managed, TypeScript); offline-first local store (WatermelonDB/SQLite) with a sync queue; auth reused from shared_backend (auth-token decision now Done, see row 15); external vision API for photo/plant ID at MVP; Expo push for notifications. Full reasoning in roadmap.md's "First 2 weeks" item 5 and status.md.</t>
+  </si>
+  <si>
+    <t>Add optional 2FA (TOTP) for user accounts</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Added 2026-08-24 (Omar)</t>
+  </si>
+  <si>
+    <t>backend + web</t>
+  </si>
+  <si>
+    <t>Not urgent pre-monetization - account takeover today just exposes garden designs. Target: built and available before monetization goes live, not necessarily before the monetization framework itself is decided. TOTP (e.g. otplib), not SMS. See docs/future-concerns.md.</t>
+  </si>
+  <si>
+    <t>Block disposable/temporary email domains at registration</t>
+  </si>
+  <si>
+    <t>Anti-abuse: check the email domain against a maintained blocklist (e.g. disposable-email-domains) in register(), reject with a clear message. Pairs with the rate limiting already added 2026-08-24. See docs/future-concerns.md.</t>
   </si>
   <si>
     <t>Decide whether wind turbine sizing should use real wind speed</t>
@@ -1291,7 +1312,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J110"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
@@ -1989,13 +2010,13 @@
         <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E22" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="G22" t="s">
         <v>21</v>
@@ -2007,7 +2028,7 @@
         <v>25</v>
       </c>
       <c r="J22" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -2018,13 +2039,13 @@
         <v>47</v>
       </c>
       <c r="C23" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" t="s">
         <v>87</v>
-      </c>
-      <c r="D23" t="s">
-        <v>54</v>
-      </c>
-      <c r="E23" t="s">
-        <v>88</v>
       </c>
       <c r="F23" t="s">
         <v>34</v>
@@ -2039,88 +2060,88 @@
         <v>25</v>
       </c>
       <c r="J23" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="C24" t="s">
         <v>92</v>
       </c>
       <c r="D24" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="E24" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="F24" t="s">
         <v>28</v>
       </c>
       <c r="G24" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H24" t="s">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="I24" t="s">
         <v>25</v>
       </c>
       <c r="J24" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="C25" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>93</v>
+        <v>54</v>
       </c>
       <c r="E25" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F25" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G25" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H25" t="s">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="I25" t="s">
         <v>25</v>
       </c>
       <c r="J25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C26" t="s">
         <v>99</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F26" t="s">
         <v>28</v>
@@ -2129,91 +2150,94 @@
         <v>16</v>
       </c>
       <c r="H26" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I26" t="s">
         <v>25</v>
       </c>
       <c r="J26" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>90</v>
-      </c>
-      <c r="B27" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="E27" t="s">
         <v>101</v>
-      </c>
-      <c r="D27" t="s">
-        <v>93</v>
-      </c>
-      <c r="E27" t="s">
-        <v>94</v>
       </c>
       <c r="F27" t="s">
         <v>28</v>
       </c>
       <c r="G27" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H27" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I27" t="s">
         <v>25</v>
+      </c>
+      <c r="J27" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C28" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E28" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F28" t="s">
         <v>28</v>
       </c>
       <c r="G28" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H28" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I28" t="s">
         <v>25</v>
       </c>
       <c r="J28" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F29" t="s">
         <v>28</v>
@@ -2222,30 +2246,27 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I29" t="s">
         <v>25</v>
-      </c>
-      <c r="J29" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C30" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D30" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E30" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F30" t="s">
         <v>28</v>
@@ -2254,30 +2275,30 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I30" t="s">
         <v>25</v>
       </c>
       <c r="J30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D31" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E31" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F31" t="s">
         <v>28</v>
@@ -2286,30 +2307,30 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I31" t="s">
         <v>25</v>
       </c>
       <c r="J31" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D32" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="E32" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F32" t="s">
         <v>28</v>
@@ -2318,27 +2339,30 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I32" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D33" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E33" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F33" t="s">
         <v>28</v>
@@ -2347,27 +2371,30 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I33" t="s">
         <v>25</v>
+      </c>
+      <c r="J33" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D34" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="E34" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F34" t="s">
         <v>28</v>
@@ -2376,27 +2403,27 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I34" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C35" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D35" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="E35" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F35" t="s">
         <v>28</v>
@@ -2405,30 +2432,27 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I35" t="s">
         <v>25</v>
-      </c>
-      <c r="J35" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D36" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="E36" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F36" t="s">
         <v>28</v>
@@ -2437,65 +2461,68 @@
         <v>21</v>
       </c>
       <c r="H36" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I36" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C37" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D37" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="E37" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F37" t="s">
         <v>28</v>
       </c>
       <c r="G37" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H37" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I37" t="s">
         <v>25</v>
+      </c>
+      <c r="J37" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C38" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D38" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="E38" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F38" t="s">
         <v>28</v>
       </c>
       <c r="G38" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H38" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I38" t="s">
         <v>25</v>
@@ -2503,231 +2530,225 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C39" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D39" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E39" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F39" t="s">
         <v>28</v>
       </c>
       <c r="G39" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H39" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I39" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C40" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D40" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="E40" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F40" t="s">
         <v>28</v>
       </c>
       <c r="G40" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H40" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I40" t="s">
         <v>25</v>
-      </c>
-      <c r="J40" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D41" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F41" t="s">
         <v>28</v>
       </c>
       <c r="G41" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H41" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I41" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="E42" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F42" t="s">
         <v>28</v>
       </c>
       <c r="G42" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H42" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I42" t="s">
         <v>25</v>
+      </c>
+      <c r="J42" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C43" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D43" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E43" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F43" t="s">
         <v>28</v>
       </c>
       <c r="G43" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H43" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I43" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="B44" t="s">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="C44" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D44" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="E44" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
       <c r="F44" t="s">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="G44" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="H44" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="I44" t="s">
         <v>25</v>
       </c>
-      <c r="J44" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="C45" t="s">
         <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="E45" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
       <c r="F45" t="s">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="G45" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="H45" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="I45" t="s">
         <v>25</v>
-      </c>
-      <c r="J45" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B46" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C46" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D46" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="E46" t="s">
-        <v>79</v>
+        <v>138</v>
       </c>
       <c r="F46" t="s">
         <v>83</v>
@@ -2736,30 +2757,30 @@
         <v>16</v>
       </c>
       <c r="H46" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="I46" t="s">
         <v>25</v>
       </c>
       <c r="J46" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B47" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C47" t="s">
+        <v>141</v>
+      </c>
+      <c r="D47" t="s">
+        <v>123</v>
+      </c>
+      <c r="E47" t="s">
         <v>138</v>
-      </c>
-      <c r="D47" t="s">
-        <v>78</v>
-      </c>
-      <c r="E47" t="s">
-        <v>79</v>
       </c>
       <c r="F47" t="s">
         <v>83</v>
@@ -2768,59 +2789,59 @@
         <v>16</v>
       </c>
       <c r="H47" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="I47" t="s">
         <v>25</v>
       </c>
       <c r="J47" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B48" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D48" t="s">
         <v>74</v>
       </c>
       <c r="E48" t="s">
-        <v>131</v>
+        <v>79</v>
       </c>
       <c r="F48" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="G48" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H48" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="I48" t="s">
         <v>25</v>
       </c>
       <c r="J48" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B49" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D49" t="s">
-        <v>145</v>
+        <v>78</v>
       </c>
       <c r="E49" t="s">
         <v>79</v>
@@ -2832,123 +2853,123 @@
         <v>16</v>
       </c>
       <c r="H49" t="s">
+        <v>139</v>
+      </c>
+      <c r="I49" t="s">
+        <v>25</v>
+      </c>
+      <c r="J49" t="s">
         <v>146</v>
       </c>
-      <c r="I49" t="s">
-        <v>25</v>
-      </c>
-      <c r="J49" t="s">
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>135</v>
+      </c>
+      <c r="B50" t="s">
+        <v>136</v>
+      </c>
+      <c r="C50" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>142</v>
-      </c>
-      <c r="B50" t="s">
-        <v>143</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
+        <v>74</v>
+      </c>
+      <c r="E50" t="s">
+        <v>138</v>
+      </c>
+      <c r="F50" t="s">
+        <v>71</v>
+      </c>
+      <c r="G50" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" t="s">
+        <v>139</v>
+      </c>
+      <c r="I50" t="s">
+        <v>25</v>
+      </c>
+      <c r="J50" t="s">
         <v>148</v>
-      </c>
-      <c r="D50" t="s">
-        <v>145</v>
-      </c>
-      <c r="E50" t="s">
-        <v>131</v>
-      </c>
-      <c r="F50" t="s">
-        <v>83</v>
-      </c>
-      <c r="G50" t="s">
-        <v>16</v>
-      </c>
-      <c r="H50" t="s">
-        <v>146</v>
-      </c>
-      <c r="I50" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B51" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C51" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D51" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E51" t="s">
-        <v>150</v>
+        <v>79</v>
       </c>
       <c r="F51" t="s">
         <v>83</v>
       </c>
       <c r="G51" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H51" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I51" t="s">
         <v>25</v>
       </c>
       <c r="J51" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B52" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C52" t="s">
+        <v>155</v>
+      </c>
+      <c r="D52" t="s">
         <v>152</v>
       </c>
-      <c r="D52" t="s">
-        <v>74</v>
-      </c>
       <c r="E52" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F52" t="s">
         <v>83</v>
       </c>
       <c r="G52" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H52" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I52" t="s">
         <v>25</v>
       </c>
-      <c r="J52" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B53" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C53" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D53" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E53" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="F53" t="s">
         <v>83</v>
@@ -2957,27 +2978,30 @@
         <v>21</v>
       </c>
       <c r="H53" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I53" t="s">
         <v>25</v>
+      </c>
+      <c r="J53" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B54" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D54" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="E54" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
       <c r="F54" t="s">
         <v>83</v>
@@ -2986,219 +3010,219 @@
         <v>21</v>
       </c>
       <c r="H54" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I54" t="s">
         <v>25</v>
       </c>
       <c r="J54" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B55" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C55" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D55" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E55" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="F55" t="s">
         <v>83</v>
       </c>
       <c r="G55" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H55" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I55" t="s">
         <v>25</v>
-      </c>
-      <c r="J55" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B56" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C56" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D56" t="s">
-        <v>74</v>
+        <v>152</v>
       </c>
       <c r="E56" t="s">
-        <v>131</v>
+        <v>163</v>
       </c>
       <c r="F56" t="s">
         <v>83</v>
       </c>
       <c r="G56" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H56" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I56" t="s">
         <v>25</v>
       </c>
       <c r="J56" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B57" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C57" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D57" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E57" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="F57" t="s">
         <v>83</v>
       </c>
       <c r="G57" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H57" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I57" t="s">
         <v>25</v>
       </c>
       <c r="J57" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="B58" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="C58" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D58" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="E58" t="s">
-        <v>167</v>
+        <v>138</v>
       </c>
       <c r="F58" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="G58" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="H58" t="s">
+        <v>153</v>
+      </c>
+      <c r="I58" t="s">
+        <v>25</v>
+      </c>
+      <c r="J58" t="s">
         <v>168</v>
       </c>
-      <c r="I58" t="s">
-        <v>25</v>
-      </c>
-      <c r="J58" t="s">
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>149</v>
+      </c>
+      <c r="B59" t="s">
+        <v>150</v>
+      </c>
+      <c r="C59" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>164</v>
-      </c>
-      <c r="B59" t="s">
-        <v>165</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
+        <v>152</v>
+      </c>
+      <c r="E59" t="s">
+        <v>138</v>
+      </c>
+      <c r="F59" t="s">
+        <v>83</v>
+      </c>
+      <c r="G59" t="s">
+        <v>127</v>
+      </c>
+      <c r="H59" t="s">
+        <v>153</v>
+      </c>
+      <c r="I59" t="s">
+        <v>25</v>
+      </c>
+      <c r="J59" t="s">
         <v>170</v>
-      </c>
-      <c r="D59" t="s">
-        <v>171</v>
-      </c>
-      <c r="E59" t="s">
-        <v>131</v>
-      </c>
-      <c r="F59" t="s">
-        <v>71</v>
-      </c>
-      <c r="G59" t="s">
-        <v>21</v>
-      </c>
-      <c r="H59" t="s">
-        <v>168</v>
-      </c>
-      <c r="I59" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B60" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C60" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>54</v>
+        <v>114</v>
       </c>
       <c r="E60" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="F60" t="s">
         <v>71</v>
       </c>
       <c r="G60" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H60" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I60" t="s">
         <v>25</v>
       </c>
       <c r="J60" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B61" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C61" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D61" t="s">
-        <v>54</v>
+        <v>178</v>
       </c>
       <c r="E61" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F61" t="s">
         <v>71</v>
@@ -3207,30 +3231,27 @@
         <v>21</v>
       </c>
       <c r="H61" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I61" t="s">
         <v>25</v>
-      </c>
-      <c r="J61" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B62" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C62" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D62" t="s">
-        <v>114</v>
+        <v>54</v>
       </c>
       <c r="E62" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F62" t="s">
         <v>71</v>
@@ -3239,30 +3260,30 @@
         <v>21</v>
       </c>
       <c r="H62" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I62" t="s">
         <v>25</v>
       </c>
       <c r="J62" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B63" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C63" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D63" t="s">
-        <v>114</v>
+        <v>54</v>
       </c>
       <c r="E63" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F63" t="s">
         <v>71</v>
@@ -3271,27 +3292,30 @@
         <v>21</v>
       </c>
       <c r="H63" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I63" t="s">
         <v>25</v>
+      </c>
+      <c r="J63" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B64" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C64" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D64" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="E64" t="s">
-        <v>180</v>
+        <v>138</v>
       </c>
       <c r="F64" t="s">
         <v>71</v>
@@ -3300,39 +3324,39 @@
         <v>21</v>
       </c>
       <c r="H64" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I64" t="s">
         <v>25</v>
       </c>
       <c r="J64" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B65" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C65" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D65" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="E65" t="s">
-        <v>183</v>
+        <v>138</v>
       </c>
       <c r="F65" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="G65" t="s">
         <v>21</v>
       </c>
       <c r="H65" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I65" t="s">
         <v>25</v>
@@ -3340,324 +3364,327 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B66" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C66" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D66" t="s">
-        <v>54</v>
+        <v>152</v>
       </c>
       <c r="E66" t="s">
-        <v>131</v>
+        <v>187</v>
       </c>
       <c r="F66" t="s">
         <v>71</v>
       </c>
       <c r="G66" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H66" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I66" t="s">
         <v>25</v>
       </c>
       <c r="J66" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B67" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C67" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D67" t="s">
-        <v>54</v>
+        <v>114</v>
       </c>
       <c r="E67" t="s">
-        <v>131</v>
+        <v>190</v>
       </c>
       <c r="F67" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="G67" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H67" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I67" t="s">
         <v>25</v>
-      </c>
-      <c r="J67" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B68" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C68" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D68" t="s">
         <v>54</v>
       </c>
       <c r="E68" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F68" t="s">
         <v>71</v>
       </c>
       <c r="G68" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H68" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I68" t="s">
         <v>25</v>
       </c>
       <c r="J68" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B69" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C69" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D69" t="s">
         <v>54</v>
       </c>
       <c r="E69" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F69" t="s">
         <v>71</v>
       </c>
       <c r="G69" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H69" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I69" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J69" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B70" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C70" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D70" t="s">
-        <v>171</v>
+        <v>54</v>
       </c>
       <c r="E70" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F70" t="s">
         <v>71</v>
       </c>
       <c r="G70" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H70" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I70" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J70" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B71" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C71" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D71" t="s">
-        <v>171</v>
+        <v>54</v>
       </c>
       <c r="E71" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F71" t="s">
         <v>71</v>
       </c>
       <c r="G71" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H71" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I71" t="s">
         <v>25</v>
       </c>
-      <c r="J71" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B72" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C72" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D72" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="E72" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F72" t="s">
         <v>71</v>
       </c>
       <c r="G72" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H72" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I72" t="s">
         <v>25</v>
       </c>
-      <c r="J72" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B73" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C73" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D73" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="E73" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F73" t="s">
         <v>71</v>
       </c>
       <c r="G73" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H73" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I73" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J73" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>197</v>
+        <v>171</v>
       </c>
       <c r="B74" t="s">
-        <v>198</v>
+        <v>172</v>
       </c>
       <c r="C74" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D74" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="E74" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F74" t="s">
         <v>71</v>
       </c>
       <c r="G74" t="s">
-        <v>21</v>
+        <v>127</v>
       </c>
       <c r="H74" t="s">
-        <v>201</v>
+        <v>175</v>
       </c>
       <c r="I74" t="s">
         <v>25</v>
+      </c>
+      <c r="J74" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>197</v>
+        <v>171</v>
       </c>
       <c r="B75" t="s">
-        <v>198</v>
+        <v>172</v>
       </c>
       <c r="C75" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D75" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="E75" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F75" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="G75" t="s">
-        <v>21</v>
+        <v>127</v>
       </c>
       <c r="H75" t="s">
-        <v>201</v>
+        <v>175</v>
       </c>
       <c r="I75" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B76" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C76" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D76" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="E76" t="s">
-        <v>204</v>
+        <v>138</v>
       </c>
       <c r="F76" t="s">
         <v>71</v>
@@ -3666,574 +3693,571 @@
         <v>21</v>
       </c>
       <c r="H76" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="I76" t="s">
         <v>25</v>
       </c>
-      <c r="J76" t="s">
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>204</v>
+      </c>
+      <c r="B77" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>197</v>
-      </c>
-      <c r="B77" t="s">
-        <v>198</v>
-      </c>
       <c r="C77" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D77" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="E77" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F77" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="G77" t="s">
         <v>21</v>
       </c>
       <c r="H77" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="I77" t="s">
         <v>25</v>
       </c>
-      <c r="J77" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B78" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C78" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D78" t="s">
-        <v>145</v>
+        <v>178</v>
       </c>
       <c r="E78" t="s">
-        <v>131</v>
+        <v>211</v>
       </c>
       <c r="F78" t="s">
         <v>71</v>
       </c>
       <c r="G78" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H78" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="I78" t="s">
         <v>25</v>
+      </c>
+      <c r="J78" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B79" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C79" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D79" t="s">
-        <v>210</v>
+        <v>178</v>
       </c>
       <c r="E79" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F79" t="s">
         <v>71</v>
       </c>
       <c r="G79" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H79" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="I79" t="s">
         <v>25</v>
       </c>
       <c r="J79" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B80" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C80" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D80" t="s">
-        <v>210</v>
+        <v>152</v>
       </c>
       <c r="E80" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F80" t="s">
         <v>71</v>
       </c>
       <c r="G80" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H80" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="I80" t="s">
         <v>25</v>
-      </c>
-      <c r="J80" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B81" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C81" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D81" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="E81" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F81" t="s">
         <v>71</v>
       </c>
       <c r="G81" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H81" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="I81" t="s">
         <v>25</v>
       </c>
       <c r="J81" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B82" t="s">
+        <v>205</v>
+      </c>
+      <c r="C82" t="s">
+        <v>219</v>
+      </c>
+      <c r="D82" t="s">
         <v>217</v>
       </c>
-      <c r="C82" t="s">
-        <v>218</v>
-      </c>
-      <c r="D82" t="s">
-        <v>49</v>
-      </c>
       <c r="E82" t="s">
-        <v>219</v>
+        <v>138</v>
       </c>
       <c r="F82" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="G82" t="s">
+        <v>127</v>
+      </c>
+      <c r="H82" t="s">
+        <v>208</v>
+      </c>
+      <c r="I82" t="s">
+        <v>25</v>
+      </c>
+      <c r="J82" t="s">
         <v>220</v>
-      </c>
-      <c r="H82" t="s">
-        <v>221</v>
-      </c>
-      <c r="I82" t="s">
-        <v>25</v>
-      </c>
-      <c r="J82" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B83" t="s">
+        <v>205</v>
+      </c>
+      <c r="C83" t="s">
+        <v>221</v>
+      </c>
+      <c r="D83" t="s">
         <v>217</v>
       </c>
-      <c r="C83" t="s">
-        <v>223</v>
-      </c>
-      <c r="D83" t="s">
-        <v>224</v>
-      </c>
       <c r="E83" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="F83" t="s">
         <v>71</v>
       </c>
       <c r="G83" t="s">
-        <v>220</v>
+        <v>127</v>
       </c>
       <c r="H83" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="I83" t="s">
         <v>25</v>
       </c>
       <c r="J83" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>223</v>
+      </c>
+      <c r="B84" t="s">
+        <v>224</v>
+      </c>
+      <c r="C84" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>216</v>
-      </c>
-      <c r="B84" t="s">
-        <v>217</v>
-      </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
+        <v>49</v>
+      </c>
+      <c r="E84" t="s">
         <v>226</v>
       </c>
-      <c r="D84" t="s">
-        <v>224</v>
-      </c>
-      <c r="E84" t="s">
-        <v>131</v>
-      </c>
       <c r="F84" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="G84" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H84" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I84" t="s">
         <v>25</v>
+      </c>
+      <c r="J84" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B85" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C85" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D85" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E85" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="F85" t="s">
         <v>71</v>
       </c>
       <c r="G85" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H85" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I85" t="s">
         <v>25</v>
       </c>
       <c r="J85" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B86" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C86" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D86" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E86" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="F86" t="s">
         <v>71</v>
       </c>
       <c r="G86" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H86" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I86" t="s">
         <v>25</v>
-      </c>
-      <c r="J86" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B87" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C87" t="s">
+        <v>234</v>
+      </c>
+      <c r="D87" t="s">
         <v>231</v>
       </c>
-      <c r="D87" t="s">
-        <v>171</v>
-      </c>
       <c r="E87" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F87" t="s">
         <v>71</v>
       </c>
       <c r="G87" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H87" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I87" t="s">
         <v>25</v>
       </c>
       <c r="J87" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B88" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C88" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D88" t="s">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="E88" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="F88" t="s">
         <v>71</v>
       </c>
       <c r="G88" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H88" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I88" t="s">
         <v>25</v>
       </c>
       <c r="J88" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B89" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C89" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D89" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="E89" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F89" t="s">
         <v>71</v>
       </c>
       <c r="G89" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H89" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I89" t="s">
         <v>25</v>
       </c>
       <c r="J89" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B90" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C90" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D90" t="s">
-        <v>237</v>
+        <v>178</v>
       </c>
       <c r="E90" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F90" t="s">
         <v>71</v>
       </c>
       <c r="G90" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H90" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I90" t="s">
         <v>25</v>
       </c>
       <c r="J90" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B91" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C91" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D91" t="s">
-        <v>237</v>
+        <v>178</v>
       </c>
       <c r="E91" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F91" t="s">
         <v>71</v>
       </c>
       <c r="G91" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H91" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I91" t="s">
         <v>25</v>
       </c>
       <c r="J91" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B92" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C92" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D92" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E92" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F92" t="s">
         <v>71</v>
       </c>
       <c r="G92" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H92" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I92" t="s">
         <v>25</v>
+      </c>
+      <c r="J92" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B93" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C93" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D93" t="s">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="E93" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="F93" t="s">
         <v>71</v>
       </c>
       <c r="G93" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H93" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I93" t="s">
         <v>25</v>
       </c>
       <c r="J93" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B94" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C94" t="s">
+        <v>248</v>
+      </c>
+      <c r="D94" t="s">
         <v>244</v>
       </c>
-      <c r="D94" t="s">
-        <v>74</v>
-      </c>
       <c r="E94" t="s">
-        <v>183</v>
+        <v>138</v>
       </c>
       <c r="F94" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="G94" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="H94" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="I94" t="s">
         <v>25</v>
@@ -4241,112 +4265,109 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B95" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C95" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D95" t="s">
-        <v>78</v>
+        <v>231</v>
       </c>
       <c r="E95" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="F95" t="s">
+        <v>71</v>
+      </c>
+      <c r="G95" t="s">
+        <v>227</v>
+      </c>
+      <c r="H95" t="s">
+        <v>228</v>
+      </c>
+      <c r="I95" t="s">
+        <v>25</v>
+      </c>
+      <c r="J95" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>223</v>
+      </c>
+      <c r="B96" t="s">
+        <v>224</v>
+      </c>
+      <c r="C96" t="s">
+        <v>251</v>
+      </c>
+      <c r="D96" t="s">
+        <v>74</v>
+      </c>
+      <c r="E96" t="s">
+        <v>190</v>
+      </c>
+      <c r="F96" t="s">
         <v>34</v>
       </c>
-      <c r="G95" t="s">
-        <v>220</v>
-      </c>
-      <c r="H95" t="s">
-        <v>221</v>
-      </c>
-      <c r="I95" t="s">
-        <v>25</v>
-      </c>
-      <c r="J95" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>247</v>
-      </c>
-      <c r="B96" t="s">
-        <v>248</v>
-      </c>
-      <c r="C96" t="s">
-        <v>249</v>
-      </c>
-      <c r="D96" t="s">
-        <v>116</v>
-      </c>
-      <c r="E96" t="s">
-        <v>250</v>
-      </c>
-      <c r="F96" t="s">
-        <v>28</v>
-      </c>
       <c r="G96" t="s">
-        <v>16</v>
+        <v>227</v>
       </c>
       <c r="H96" t="s">
-        <v>251</v>
+        <v>228</v>
       </c>
       <c r="I96" t="s">
         <v>25</v>
-      </c>
-      <c r="J96" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>247</v>
+        <v>223</v>
       </c>
       <c r="B97" t="s">
-        <v>248</v>
+        <v>224</v>
       </c>
       <c r="C97" t="s">
+        <v>252</v>
+      </c>
+      <c r="D97" t="s">
+        <v>78</v>
+      </c>
+      <c r="E97" t="s">
+        <v>157</v>
+      </c>
+      <c r="F97" t="s">
+        <v>34</v>
+      </c>
+      <c r="G97" t="s">
+        <v>227</v>
+      </c>
+      <c r="H97" t="s">
+        <v>228</v>
+      </c>
+      <c r="I97" t="s">
+        <v>25</v>
+      </c>
+      <c r="J97" t="s">
         <v>253</v>
-      </c>
-      <c r="D97" t="s">
-        <v>116</v>
-      </c>
-      <c r="E97" t="s">
-        <v>254</v>
-      </c>
-      <c r="F97" t="s">
-        <v>28</v>
-      </c>
-      <c r="G97" t="s">
-        <v>16</v>
-      </c>
-      <c r="H97" t="s">
-        <v>251</v>
-      </c>
-      <c r="I97" t="s">
-        <v>25</v>
-      </c>
-      <c r="J97" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B98" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C98" t="s">
         <v>256</v>
       </c>
       <c r="D98" t="s">
-        <v>58</v>
+        <v>123</v>
       </c>
       <c r="E98" t="s">
         <v>257</v>
@@ -4358,91 +4379,94 @@
         <v>16</v>
       </c>
       <c r="H98" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I98" t="s">
         <v>25</v>
       </c>
       <c r="J98" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B99" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C99" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D99" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="E99" t="s">
-        <v>150</v>
+        <v>261</v>
       </c>
       <c r="F99" t="s">
         <v>28</v>
       </c>
       <c r="G99" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H99" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I99" t="s">
         <v>25</v>
       </c>
       <c r="J99" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B100" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C100" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D100" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="E100" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="F100" t="s">
         <v>28</v>
       </c>
       <c r="G100" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H100" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I100" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J100" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B101" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C101" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D101" t="s">
-        <v>58</v>
+        <v>123</v>
       </c>
       <c r="E101" t="s">
-        <v>263</v>
+        <v>157</v>
       </c>
       <c r="F101" t="s">
         <v>28</v>
@@ -4451,27 +4475,30 @@
         <v>21</v>
       </c>
       <c r="H101" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I101" t="s">
         <v>25</v>
+      </c>
+      <c r="J101" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B102" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C102" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D102" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E102" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F102" t="s">
         <v>28</v>
@@ -4480,27 +4507,27 @@
         <v>21</v>
       </c>
       <c r="H102" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I102" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B103" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C103" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D103" t="s">
         <v>58</v>
       </c>
       <c r="E103" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="F103" t="s">
         <v>28</v>
@@ -4509,167 +4536,225 @@
         <v>21</v>
       </c>
       <c r="H103" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I103" t="s">
         <v>25</v>
       </c>
-      <c r="J103" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B104" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C104" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D104" t="s">
-        <v>200</v>
+        <v>58</v>
       </c>
       <c r="E104" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F104" t="s">
         <v>28</v>
       </c>
       <c r="G104" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H104" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I104" t="s">
         <v>25</v>
-      </c>
-      <c r="J104" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B105" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C105" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D105" t="s">
-        <v>200</v>
+        <v>58</v>
       </c>
       <c r="E105" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="F105" t="s">
         <v>28</v>
       </c>
       <c r="G105" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="H105" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I105" t="s">
         <v>25</v>
       </c>
       <c r="J105" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B106" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C106" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D106" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E106" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="F106" t="s">
         <v>28</v>
       </c>
       <c r="G106" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H106" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I106" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J106" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B107" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C107" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="D107" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E107" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F107" t="s">
         <v>28</v>
       </c>
       <c r="G107" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="H107" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I107" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J107" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
+        <v>254</v>
+      </c>
+      <c r="B108" t="s">
+        <v>255</v>
+      </c>
+      <c r="C108" t="s">
+        <v>280</v>
+      </c>
+      <c r="D108" t="s">
+        <v>207</v>
+      </c>
+      <c r="E108" t="s">
         <v>276</v>
       </c>
-      <c r="B108" t="s">
-        <v>277</v>
-      </c>
-      <c r="C108" t="s">
-        <v>278</v>
-      </c>
-      <c r="D108" t="s">
-        <v>279</v>
-      </c>
-      <c r="E108" t="s">
-        <v>150</v>
-      </c>
       <c r="F108" t="s">
-        <v>280</v>
+        <v>28</v>
       </c>
       <c r="G108" t="s">
-        <v>280</v>
+        <v>127</v>
       </c>
       <c r="H108" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="I108" t="s">
         <v>25</v>
       </c>
-      <c r="J108" t="s">
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>254</v>
+      </c>
+      <c r="B109" t="s">
+        <v>255</v>
+      </c>
+      <c r="C109" t="s">
         <v>281</v>
+      </c>
+      <c r="D109" t="s">
+        <v>207</v>
+      </c>
+      <c r="E109" t="s">
+        <v>282</v>
+      </c>
+      <c r="F109" t="s">
+        <v>28</v>
+      </c>
+      <c r="G109" t="s">
+        <v>127</v>
+      </c>
+      <c r="H109" t="s">
+        <v>258</v>
+      </c>
+      <c r="I109" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>283</v>
+      </c>
+      <c r="B110" t="s">
+        <v>284</v>
+      </c>
+      <c r="C110" t="s">
+        <v>285</v>
+      </c>
+      <c r="D110" t="s">
+        <v>286</v>
+      </c>
+      <c r="E110" t="s">
+        <v>157</v>
+      </c>
+      <c r="F110" t="s">
+        <v>287</v>
+      </c>
+      <c r="G110" t="s">
+        <v>287</v>
+      </c>
+      <c r="H110" t="s">
+        <v>287</v>
+      </c>
+      <c r="I110" t="s">
+        <v>25</v>
+      </c>
+      <c r="J110" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -4695,19 +4780,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="E1" t="s">
         <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="G1" t="s">
         <v>16</v>
@@ -4716,10 +4801,10 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="J1" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4733,10 +4818,10 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="E2" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -4765,19 +4850,19 @@
         <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="E3" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G3">
         <v>10</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -4788,19 +4873,19 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="E4" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="F4">
         <v>20</v>
@@ -4820,19 +4905,19 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C5" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="D5" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="E5" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -4852,19 +4937,19 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="E6" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -4884,19 +4969,19 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B7" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C7" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="D7" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="E7" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="F7">
         <v>16</v>
@@ -4916,19 +5001,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B8" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C8" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="D8" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E8" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F8">
         <v>8</v>
@@ -4948,19 +5033,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B9" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C9" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="D9" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="E9" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F9">
         <v>14</v>
@@ -4980,19 +5065,19 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B10" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C10" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="D10" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="E10" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="F10">
         <v>12</v>
@@ -5012,19 +5097,19 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B11" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C11" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="D11" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="E11" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="F11">
         <v>1</v>

</xml_diff>

<commit_message>
Update roadmap_backlog.xlsx: mark Shareable link as Done
Built and verified live this session - see swales-services commit
"Add shareable link for the map's current pin (Phase A2 quick win)".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap_backlog.xlsx
+++ b/docs/roadmap_backlog.xlsx
@@ -2224,12 +2224,14 @@
       <c r="H27" t="s">
         <v>102</v>
       </c>
-      <c r="I27" t="s">
-        <v>25</v>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>One-line param change - near-zero cost, ship immediately. Code-checked 2026-08-28: confirmed not built - no lat/lng/active-layer URL-param handling found.</t>
+          <t>One-line param change - near-zero cost, ship immediately. STATUS UPDATE 2026-08-30: built and verified live - MapComponent.jsx's updateLocationAndTimeGeoInfo now mirrors the pin into ?lat=&amp;lng= via window.history.replaceState (the active layer was already encoded by the path itself), read back on mount via getUrlLocation() taking priority over stored location/geolocation. Added a Copy shareable link button (Share2 icon) next to the PDF-report button.</t>
         </is>
       </c>
     </row>

</xml_diff>